<commit_message>
app.js had too much workload, refactor to sub modules
</commit_message>
<xml_diff>
--- a/Arya_Phones_Supplier_Selection.xlsx
+++ b/Arya_Phones_Supplier_Selection.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\LENOVO\Desktop\Asistan\Arya Phone\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9C9ABEA2-4B77-4451-98AA-59E3368C40E5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6A20A31E-6678-4EAE-8919-6A2CCCD1F14D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Supplier" sheetId="1" r:id="rId1"/>
@@ -48,7 +48,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="602" uniqueCount="161">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="537" uniqueCount="96">
   <si>
     <t>Supplier</t>
   </si>
@@ -198,201 +198,6 @@
   </si>
   <si>
     <t>0,282x1+ 0,065x2+ 0,584x3+ 0,286x4+ 0,167x5+ -0,160x6</t>
-  </si>
-  <si>
-    <t>0,136x1+ 0,267x2+ 0,117x3+ 0,107x4+ 0,257x5+ -0,168x6</t>
-  </si>
-  <si>
-    <t>0,176x1+ 0,133x2+ 0,641x3+ 0,116x4+ 0,102x5+ -0,219x6</t>
-  </si>
-  <si>
-    <t>0,061x1+ 0,202x2+ 0,330x3+ 0,107x4+ 0,214x5+ -0,196x6</t>
-  </si>
-  <si>
-    <t>0,282x1+ 0,058x2+ 0,542x3+ 0,107x4+ 0,102x5+ -0,233x6</t>
-  </si>
-  <si>
-    <t>0,097x1+ 0,104x2+ 0,402x3+ 0,107x4+ 0,144x5+ -0,104x6</t>
-  </si>
-  <si>
-    <t>0,160x1+ 0,096x2+ 0,542x3+ 0,107x4+ 0,165x5+ -0,104x6</t>
-  </si>
-  <si>
-    <t>0,162x1+ 0,138x2+ 0,649x3+ 0,312x4+ 0,102x5+ -0,296x6</t>
-  </si>
-  <si>
-    <t>0,103x1+ 0,252x2+ 0,466x3+ 0,107x4+ 0,249x5+ -0,230x6</t>
-  </si>
-  <si>
-    <t>0,169x1+ 0,073x2+ 0,117x3+ 0,107x4+ 0,196x5+ -0,104x6</t>
-  </si>
-  <si>
-    <t>0,061x1+ 0,268x2+ 0,597x3+ 0,207x4+ 0,102x5+ -0,296x6</t>
-  </si>
-  <si>
-    <t>0,202x1+ 0,073x2+ 0,117x3+ 0,159x4+ 0,102x5+ -0,104x6</t>
-  </si>
-  <si>
-    <t>0,061x1+ 0,147x2+ 0,415x3+ 0,107x4+ 0,172x5+ -0,296x6</t>
-  </si>
-  <si>
-    <t>0,061x1+ 0,073x2+ 0,115x3+ 0,107x4+ 0,102x5+ -0,296x6</t>
-  </si>
-  <si>
-    <t>0,051x1+ 0,154x2+ 0,336x3+ 0,164x4+ 0,164x5+ -0,228x6</t>
-  </si>
-  <si>
-    <t>0,061x1+ 0,133x2+ 0,206x3+ 0,107x4+ 0,102x5+ -0,201x6</t>
-  </si>
-  <si>
-    <t>0,259x1+ 0,051x2+ 0,389x3+ 0,107x4+ 0,143x5+ -0,139x6</t>
-  </si>
-  <si>
-    <t>0,134x1+ 0,073x2+ 0,353x3+ 0,107x4+ 0,102x5+ -0,279x6</t>
-  </si>
-  <si>
-    <t>0,111x1+ 0,268x2+ 0,117x3+ 0,107x4+ 0,205x5+ -0,156x6</t>
-  </si>
-  <si>
-    <t>0,163x1+ 0,073x2+ 0,579x3+ 0,107x4+ 0,220x5+ -0,249x6</t>
-  </si>
-  <si>
-    <t>0,122x1+ 0,073x2+ 0,410x3+ 0,102x4+ 0,109x5+ -0,150x6</t>
-  </si>
-  <si>
-    <t>0,088x1+ 0,268x2+ 0,465x3+ 0,202x4+ 0,124x5+ -0,104x6</t>
-  </si>
-  <si>
-    <t>0,216x1+ 0,130x2+ 0,354x3+ 0,100x4+ 0,196x5+ -0,129x6</t>
-  </si>
-  <si>
-    <t>0,094x1+ 0,180x2+ 0,117x3+ 0,203x4+ 0,163x5+ -0,154x6</t>
-  </si>
-  <si>
-    <t>0,101x1+ 0,237x2+ 0,372x3+ 0,212x4+ 0,101x5+ -0,254x6</t>
-  </si>
-  <si>
-    <t>0,061x1+ 0,243x2+ 0,117x3+ 0,142x4+ 0,165x5+ -0,267x6</t>
-  </si>
-  <si>
-    <t>0,170x1+ 0,070x2+ 0,461x3+ 0,233x4+ 0,108x5+ -0,109x6</t>
-  </si>
-  <si>
-    <t>0,151x1+ 0,130x2+ 0,203x3+ 0,107x4+ 0,179x5+ -0,296x6</t>
-  </si>
-  <si>
-    <t>0,282x1+ 0,157x2+ 0,147x3+ 0,115x4+ 0,285x5+ -0,106x6</t>
-  </si>
-  <si>
-    <t>0,061x1+ 0,250x2+ 0,328x3+ 0,209x4+ 0,285x5+ -0,198x6</t>
-  </si>
-  <si>
-    <t>0,061x1+ 0,265x2+ 0,463x3+ 0,104x4+ 0,102x5+ -0,104x6</t>
-  </si>
-  <si>
-    <t>0,118x1+ 0,147x2+ 0,117x3+ 0,107x4+ 0,118x5+ -0,289x6</t>
-  </si>
-  <si>
-    <t>0,258x1+ 0,171x2+ 0,577x3+ 0,149x4+ 0,167x5+ -0,296x6</t>
-  </si>
-  <si>
-    <t>0,205x1+ 0,107x2+ 0,602x3+ 0,143x4+ 0,299x5+ -0,190x6</t>
-  </si>
-  <si>
-    <t>0,061x1+ 0,107x2+ 0,641x3+ 0,114x4+ 0,202x5+ -0,192x6</t>
-  </si>
-  <si>
-    <t>0,053x1+ 0,073x2+ 0,512x3+ 0,107x4+ 0,102x5+ -0,110x6</t>
-  </si>
-  <si>
-    <t>0,099x1+ 0,205x2+ 0,117x3+ 0,133x4+ 0,211x5+ -0,199x6</t>
-  </si>
-  <si>
-    <t>0,279x1+ 0,221x2+ 0,460x3+ 0,107x4+ 0,102x5+ -0,259x6</t>
-  </si>
-  <si>
-    <t>0,061x1+ 0,114x2+ 0,309x3+ 0,107x4+ 0,102x5+ -0,104x6</t>
-  </si>
-  <si>
-    <t>0,084x1+ 0,073x2+ 0,117x3+ 0,121x4+ 0,102x5+ -0,206x6</t>
-  </si>
-  <si>
-    <t>0,119x1+ 0,154x2+ 0,307x3+ 0,149x4+ 0,102x5+ -0,240x6</t>
-  </si>
-  <si>
-    <t>0,259x1+ 0,237x2+ 0,209x3+ 0,189x4+ 0,271x5+ -0,134x6</t>
-  </si>
-  <si>
-    <t>0,199x1+ 0,161x2+ 0,117x3+ 0,212x4+ 0,102x5+ -0,257x6</t>
-  </si>
-  <si>
-    <t>0,061x1+ 0,057x2+ 0,117x3+ 0,111x4+ 0,102x5+ -0,159x6</t>
-  </si>
-  <si>
-    <t>0,282x1+ 0,212x2+ 0,453x3+ 0,249x4+ 0,178x5+ -0,296x6</t>
-  </si>
-  <si>
-    <t>0,119x1+ 0,133x2+ 0,340x3+ 0,316x4+ 0,243x5+ -0,104x6</t>
-  </si>
-  <si>
-    <t>0,117x1+ 0,073x2+ 0,352x3+ 0,343x4+ 0,102x5+ -0,202x6</t>
-  </si>
-  <si>
-    <t>0,052x1+ 0,251x2+ 0,117x3+ 0,323x4+ 0,229x5+ -0,148x6</t>
-  </si>
-  <si>
-    <t>0,228x1+ 0,051x2+ 0,117x3+ 0,190x4+ 0,102x5+ -0,104x6</t>
-  </si>
-  <si>
-    <t>0,135x1+ 0,128x2+ 0,404x3+ 0,202x4+ 0,102x5+ -0,112x6</t>
-  </si>
-  <si>
-    <t>0,227x1+ 0,200x2+ 0,554x3+ 0,203x4+ 0,156x5+ -0,153x6</t>
-  </si>
-  <si>
-    <t>0,131x1+ 0,229x2+ 0,274x3+ 0,107x4+ 0,113x5+ -0,239x6</t>
-  </si>
-  <si>
-    <t>0,190x1+ 0,188x2+ 0,202x3+ 0,107x4+ 0,285x5+ -0,174x6</t>
-  </si>
-  <si>
-    <t>0,061x1+ 0,198x2+ 0,564x3+ 0,161x4+ 0,167x5+ -0,247x6</t>
-  </si>
-  <si>
-    <t>0,060x1+ 0,161x2+ 0,619x3+ 0,107x4+ 0,102x5+ -0,182x6</t>
-  </si>
-  <si>
-    <t>0,061x1+ 0,144x2+ 0,378x3+ 0,238x4+ 0,102x5+ -0,296x6</t>
-  </si>
-  <si>
-    <t>0,220x1+ 0,073x2+ 0,117x3+ 0,216x4+ 0,102x5+ -0,134x6</t>
-  </si>
-  <si>
-    <t>0,190x1+ 0,217x2+ 0,163x3+ 0,107x4+ 0,157x5+ -0,296x6</t>
-  </si>
-  <si>
-    <t>0,061x1+ 0,099x2+ 0,628x3+ 0,107x4+ 0,158x5+ -0,224x6</t>
-  </si>
-  <si>
-    <t>0,096x1+ 0,118x2+ 0,363x3+ 0,179x4+ 0,102x5+ -0,104x6</t>
-  </si>
-  <si>
-    <t>0,259x1+ 0,081x2+ 0,605x3+ 0,257x4+ 0,172x5+ -0,108x6</t>
-  </si>
-  <si>
-    <t>0,250x1+ 0,131x2+ 0,117x3+ 0,107x4+ 0,102x5+ -0,104x6</t>
-  </si>
-  <si>
-    <t>0,061x1+ 0,232x2+ 0,104x3+ 0,134x4+ 0,102x5+ -0,179x6</t>
-  </si>
-  <si>
-    <t>0,213x1+ 0,157x2+ 0,117x3+ 0,169x4+ 0,102x5+ -0,104x6</t>
-  </si>
-  <si>
-    <t>0,189x1+ 0,073x2+ 0,117x3+ 0,107x4+ 0,102x5+ -0,133x6</t>
-  </si>
-  <si>
-    <t>0,200x1+ 0,088x2+ 0,117x3+ 0,107x4+ 0,102x5+ -0,296x6</t>
   </si>
   <si>
     <t>Q1. Equal Weights</t>
@@ -986,14 +791,14 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1808,7 +1613,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:H86"/>
+  <dimension ref="A1:H21"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="8" max="8" width="39.6640625" customWidth="1"/>
@@ -2358,1696 +2163,6 @@
       </c>
       <c r="H21" s="1" t="s">
         <v>49</v>
-      </c>
-    </row>
-    <row r="22" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A22" s="43">
-        <v>21</v>
-      </c>
-      <c r="B22" s="53">
-        <v>0.13625019475941991</v>
-      </c>
-      <c r="C22" s="53">
-        <v>0.26736279280814362</v>
-      </c>
-      <c r="D22" s="53">
-        <v>0.1173714689098652</v>
-      </c>
-      <c r="E22" s="53">
-        <v>0.1067200194772385</v>
-      </c>
-      <c r="F22" s="53">
-        <v>0.25697808716493392</v>
-      </c>
-      <c r="G22" s="54">
-        <v>0.1681867427062157</v>
-      </c>
-      <c r="H22" s="1" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="23" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A23" s="43">
-        <v>22</v>
-      </c>
-      <c r="B23" s="53">
-        <v>0.1757688680245634</v>
-      </c>
-      <c r="C23" s="53">
-        <v>0.13282806155902641</v>
-      </c>
-      <c r="D23" s="53">
-        <v>0.64069937166006974</v>
-      </c>
-      <c r="E23" s="53">
-        <v>0.1156241043733628</v>
-      </c>
-      <c r="F23" s="53">
-        <v>0.10155365833498819</v>
-      </c>
-      <c r="G23" s="54">
-        <v>0.2187801270157072</v>
-      </c>
-      <c r="H23" s="1" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="24" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A24" s="43">
-        <v>23</v>
-      </c>
-      <c r="B24" s="53">
-        <v>6.067934013561796E-2</v>
-      </c>
-      <c r="C24" s="53">
-        <v>0.20207761827146961</v>
-      </c>
-      <c r="D24" s="53">
-        <v>0.33025223475584031</v>
-      </c>
-      <c r="E24" s="53">
-        <v>0.1067200194772385</v>
-      </c>
-      <c r="F24" s="53">
-        <v>0.21440445635804889</v>
-      </c>
-      <c r="G24" s="54">
-        <v>0.19588920992446079</v>
-      </c>
-      <c r="H24" s="1" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="25" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A25" s="43">
-        <v>24</v>
-      </c>
-      <c r="B25" s="53">
-        <v>0.28227114589511132</v>
-      </c>
-      <c r="C25" s="53">
-        <v>5.7928141451700603E-2</v>
-      </c>
-      <c r="D25" s="53">
-        <v>0.54249507516555229</v>
-      </c>
-      <c r="E25" s="53">
-        <v>0.1067200194772385</v>
-      </c>
-      <c r="F25" s="53">
-        <v>0.10155365833498819</v>
-      </c>
-      <c r="G25" s="54">
-        <v>0.23252083661110859</v>
-      </c>
-      <c r="H25" s="1" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="26" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A26" s="43">
-        <v>25</v>
-      </c>
-      <c r="B26" s="53">
-        <v>9.7351436399047947E-2</v>
-      </c>
-      <c r="C26" s="53">
-        <v>0.1036188640356149</v>
-      </c>
-      <c r="D26" s="53">
-        <v>0.4019932384394676</v>
-      </c>
-      <c r="E26" s="53">
-        <v>0.1067200194772385</v>
-      </c>
-      <c r="F26" s="53">
-        <v>0.14400999259416411</v>
-      </c>
-      <c r="G26" s="54">
-        <v>0.1037612453176729</v>
-      </c>
-      <c r="H26" s="1" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="27" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A27" s="43">
-        <v>26</v>
-      </c>
-      <c r="B27" s="53">
-        <v>0.16044967167869861</v>
-      </c>
-      <c r="C27" s="53">
-        <v>9.6479634751771487E-2</v>
-      </c>
-      <c r="D27" s="53">
-        <v>0.54196051403912304</v>
-      </c>
-      <c r="E27" s="53">
-        <v>0.1067200194772385</v>
-      </c>
-      <c r="F27" s="53">
-        <v>0.1652384376770844</v>
-      </c>
-      <c r="G27" s="54">
-        <v>0.1037612453176729</v>
-      </c>
-      <c r="H27" s="1" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="28" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A28" s="43">
-        <v>27</v>
-      </c>
-      <c r="B28" s="53">
-        <v>0.16205033380473799</v>
-      </c>
-      <c r="C28" s="53">
-        <v>0.13770711847088629</v>
-      </c>
-      <c r="D28" s="53">
-        <v>0.64905268959204165</v>
-      </c>
-      <c r="E28" s="53">
-        <v>0.31208115405725639</v>
-      </c>
-      <c r="F28" s="53">
-        <v>0.10155365833498819</v>
-      </c>
-      <c r="G28" s="54">
-        <v>0.29588315318380942</v>
-      </c>
-      <c r="H28" s="1" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="29" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A29" s="43">
-        <v>28</v>
-      </c>
-      <c r="B29" s="53">
-        <v>0.10340378947793161</v>
-      </c>
-      <c r="C29" s="53">
-        <v>0.25203030683265509</v>
-      </c>
-      <c r="D29" s="53">
-        <v>0.46567370647245332</v>
-      </c>
-      <c r="E29" s="53">
-        <v>0.1067200194772385</v>
-      </c>
-      <c r="F29" s="53">
-        <v>0.24907466418556179</v>
-      </c>
-      <c r="G29" s="54">
-        <v>0.23016456428897561</v>
-      </c>
-      <c r="H29" s="1" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="30" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A30" s="43">
-        <v>29</v>
-      </c>
-      <c r="B30" s="53">
-        <v>0.16931293751957649</v>
-      </c>
-      <c r="C30" s="53">
-        <v>7.3418276193979989E-2</v>
-      </c>
-      <c r="D30" s="53">
-        <v>0.1173714689098652</v>
-      </c>
-      <c r="E30" s="53">
-        <v>0.1067200194772385</v>
-      </c>
-      <c r="F30" s="53">
-        <v>0.1957158721668788</v>
-      </c>
-      <c r="G30" s="54">
-        <v>0.1037612453176729</v>
-      </c>
-      <c r="H30" s="1" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="31" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A31" s="43">
-        <v>30</v>
-      </c>
-      <c r="B31" s="53">
-        <v>6.067934013561796E-2</v>
-      </c>
-      <c r="C31" s="53">
-        <v>0.26767870281778822</v>
-      </c>
-      <c r="D31" s="53">
-        <v>0.59663284449019394</v>
-      </c>
-      <c r="E31" s="53">
-        <v>0.20702380870098461</v>
-      </c>
-      <c r="F31" s="53">
-        <v>0.10155365833498819</v>
-      </c>
-      <c r="G31" s="54">
-        <v>0.29588315318380942</v>
-      </c>
-      <c r="H31" s="1" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="32" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A32" s="43">
-        <v>31</v>
-      </c>
-      <c r="B32" s="53">
-        <v>0.20227126467397741</v>
-      </c>
-      <c r="C32" s="53">
-        <v>7.3418276193979989E-2</v>
-      </c>
-      <c r="D32" s="53">
-        <v>0.1173714689098652</v>
-      </c>
-      <c r="E32" s="53">
-        <v>0.1590724795549413</v>
-      </c>
-      <c r="F32" s="53">
-        <v>0.10155365833498819</v>
-      </c>
-      <c r="G32" s="54">
-        <v>0.1037612453176729</v>
-      </c>
-      <c r="H32" s="1" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="33" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A33" s="43">
-        <v>32</v>
-      </c>
-      <c r="B33" s="53">
-        <v>6.067934013561796E-2</v>
-      </c>
-      <c r="C33" s="53">
-        <v>0.1465153407995628</v>
-      </c>
-      <c r="D33" s="53">
-        <v>0.41532089498017971</v>
-      </c>
-      <c r="E33" s="53">
-        <v>0.1067200194772385</v>
-      </c>
-      <c r="F33" s="53">
-        <v>0.17224753528221429</v>
-      </c>
-      <c r="G33" s="54">
-        <v>0.29588315318380942</v>
-      </c>
-      <c r="H33" s="1" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="34" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A34" s="43">
-        <v>33</v>
-      </c>
-      <c r="B34" s="53">
-        <v>6.067934013561796E-2</v>
-      </c>
-      <c r="C34" s="53">
-        <v>7.3418276193979989E-2</v>
-      </c>
-      <c r="D34" s="53">
-        <v>0.1154837922041731</v>
-      </c>
-      <c r="E34" s="53">
-        <v>0.1067200194772385</v>
-      </c>
-      <c r="F34" s="53">
-        <v>0.10155365833498819</v>
-      </c>
-      <c r="G34" s="54">
-        <v>0.29588315318380942</v>
-      </c>
-      <c r="H34" s="1" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="35" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A35" s="43">
-        <v>34</v>
-      </c>
-      <c r="B35" s="53">
-        <v>5.134186292704554E-2</v>
-      </c>
-      <c r="C35" s="53">
-        <v>0.15366476497204831</v>
-      </c>
-      <c r="D35" s="53">
-        <v>0.33556322969573521</v>
-      </c>
-      <c r="E35" s="53">
-        <v>0.16387213625980671</v>
-      </c>
-      <c r="F35" s="53">
-        <v>0.1637215028212998</v>
-      </c>
-      <c r="G35" s="54">
-        <v>0.2276050181531796</v>
-      </c>
-      <c r="H35" s="1" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="36" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A36" s="43">
-        <v>35</v>
-      </c>
-      <c r="B36" s="53">
-        <v>6.067934013561796E-2</v>
-      </c>
-      <c r="C36" s="53">
-        <v>0.1334610743396101</v>
-      </c>
-      <c r="D36" s="53">
-        <v>0.2058539222183588</v>
-      </c>
-      <c r="E36" s="53">
-        <v>0.1067200194772385</v>
-      </c>
-      <c r="F36" s="53">
-        <v>0.10155365833498819</v>
-      </c>
-      <c r="G36" s="54">
-        <v>0.20102319209803529</v>
-      </c>
-      <c r="H36" s="1" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="37" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A37" s="43">
-        <v>36</v>
-      </c>
-      <c r="B37" s="53">
-        <v>0.25913391903267408</v>
-      </c>
-      <c r="C37" s="53">
-        <v>5.0744524422769353E-2</v>
-      </c>
-      <c r="D37" s="53">
-        <v>0.38923388289253702</v>
-      </c>
-      <c r="E37" s="53">
-        <v>0.1067200194772385</v>
-      </c>
-      <c r="F37" s="53">
-        <v>0.143033497693828</v>
-      </c>
-      <c r="G37" s="54">
-        <v>0.13931679933128971</v>
-      </c>
-      <c r="H37" s="1" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="38" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A38" s="43">
-        <v>37</v>
-      </c>
-      <c r="B38" s="53">
-        <v>0.1340690584823008</v>
-      </c>
-      <c r="C38" s="53">
-        <v>7.3418276193979989E-2</v>
-      </c>
-      <c r="D38" s="53">
-        <v>0.35306697941176368</v>
-      </c>
-      <c r="E38" s="53">
-        <v>0.1067200194772385</v>
-      </c>
-      <c r="F38" s="53">
-        <v>0.10155365833498819</v>
-      </c>
-      <c r="G38" s="54">
-        <v>0.27891886770336383</v>
-      </c>
-      <c r="H38" s="1" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="39" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A39" s="43">
-        <v>38</v>
-      </c>
-      <c r="B39" s="53">
-        <v>0.1111054444604742</v>
-      </c>
-      <c r="C39" s="53">
-        <v>0.2680347154590641</v>
-      </c>
-      <c r="D39" s="53">
-        <v>0.1173714689098652</v>
-      </c>
-      <c r="E39" s="53">
-        <v>0.1067200194772385</v>
-      </c>
-      <c r="F39" s="53">
-        <v>0.20487467516272609</v>
-      </c>
-      <c r="G39" s="54">
-        <v>0.15619432440371731</v>
-      </c>
-      <c r="H39" s="1" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="40" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A40" s="43">
-        <v>39</v>
-      </c>
-      <c r="B40" s="53">
-        <v>0.16339537493047609</v>
-      </c>
-      <c r="C40" s="53">
-        <v>7.3418276193979989E-2</v>
-      </c>
-      <c r="D40" s="53">
-        <v>0.57874146052893005</v>
-      </c>
-      <c r="E40" s="53">
-        <v>0.1067200194772385</v>
-      </c>
-      <c r="F40" s="53">
-        <v>0.2196715384853373</v>
-      </c>
-      <c r="G40" s="54">
-        <v>0.24853398700261081</v>
-      </c>
-      <c r="H40" s="1" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="41" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A41" s="43">
-        <v>40</v>
-      </c>
-      <c r="B41" s="53">
-        <v>0.1221317086112438</v>
-      </c>
-      <c r="C41" s="53">
-        <v>7.3418276193979989E-2</v>
-      </c>
-      <c r="D41" s="53">
-        <v>0.41005061948794591</v>
-      </c>
-      <c r="E41" s="53">
-        <v>0.1015529156194887</v>
-      </c>
-      <c r="F41" s="53">
-        <v>0.1089115152077469</v>
-      </c>
-      <c r="G41" s="54">
-        <v>0.150379238279406</v>
-      </c>
-      <c r="H41" s="1" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="42" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A42" s="43">
-        <v>41</v>
-      </c>
-      <c r="B42" s="53">
-        <v>8.8223473800809804E-2</v>
-      </c>
-      <c r="C42" s="53">
-        <v>0.26830028511204312</v>
-      </c>
-      <c r="D42" s="53">
-        <v>0.46549001597124251</v>
-      </c>
-      <c r="E42" s="53">
-        <v>0.20215479965648939</v>
-      </c>
-      <c r="F42" s="53">
-        <v>0.1239843630316539</v>
-      </c>
-      <c r="G42" s="54">
-        <v>0.1037612453176729</v>
-      </c>
-      <c r="H42" s="1" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="43" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A43" s="43">
-        <v>42</v>
-      </c>
-      <c r="B43" s="53">
-        <v>0.21568370928262151</v>
-      </c>
-      <c r="C43" s="53">
-        <v>0.1299771080090909</v>
-      </c>
-      <c r="D43" s="53">
-        <v>0.35417779531371879</v>
-      </c>
-      <c r="E43" s="53">
-        <v>0.1002248119994248</v>
-      </c>
-      <c r="F43" s="53">
-        <v>0.19568531844032089</v>
-      </c>
-      <c r="G43" s="54">
-        <v>0.12934127424786651</v>
-      </c>
-      <c r="H43" s="1" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="44" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A44" s="43">
-        <v>43</v>
-      </c>
-      <c r="B44" s="53">
-        <v>9.3856794765787496E-2</v>
-      </c>
-      <c r="C44" s="53">
-        <v>0.18045870208306161</v>
-      </c>
-      <c r="D44" s="53">
-        <v>0.1173714689098652</v>
-      </c>
-      <c r="E44" s="53">
-        <v>0.20333842209891911</v>
-      </c>
-      <c r="F44" s="53">
-        <v>0.16339607558938371</v>
-      </c>
-      <c r="G44" s="54">
-        <v>0.1542335563333018</v>
-      </c>
-      <c r="H44" s="1" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="45" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A45" s="43">
-        <v>44</v>
-      </c>
-      <c r="B45" s="53">
-        <v>0.1014260066380611</v>
-      </c>
-      <c r="C45" s="53">
-        <v>0.23709112499929019</v>
-      </c>
-      <c r="D45" s="53">
-        <v>0.3721587487588684</v>
-      </c>
-      <c r="E45" s="53">
-        <v>0.21183986142914921</v>
-      </c>
-      <c r="F45" s="53">
-        <v>0.10058845287088319</v>
-      </c>
-      <c r="G45" s="54">
-        <v>0.25398075629399858</v>
-      </c>
-      <c r="H45" s="1" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="46" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A46" s="43">
-        <v>45</v>
-      </c>
-      <c r="B46" s="53">
-        <v>6.067934013561796E-2</v>
-      </c>
-      <c r="C46" s="53">
-        <v>0.24312928948159809</v>
-      </c>
-      <c r="D46" s="53">
-        <v>0.1173714689098652</v>
-      </c>
-      <c r="E46" s="53">
-        <v>0.14228890062237479</v>
-      </c>
-      <c r="F46" s="53">
-        <v>0.16484454621576591</v>
-      </c>
-      <c r="G46" s="54">
-        <v>0.26722110127478638</v>
-      </c>
-      <c r="H46" s="1" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="47" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A47" s="43">
-        <v>46</v>
-      </c>
-      <c r="B47" s="53">
-        <v>0.16951690254088669</v>
-      </c>
-      <c r="C47" s="53">
-        <v>6.9989604187531668E-2</v>
-      </c>
-      <c r="D47" s="53">
-        <v>0.46122457490335778</v>
-      </c>
-      <c r="E47" s="53">
-        <v>0.23347442148151001</v>
-      </c>
-      <c r="F47" s="53">
-        <v>0.108486259681195</v>
-      </c>
-      <c r="G47" s="54">
-        <v>0.1085482072022719</v>
-      </c>
-      <c r="H47" s="1" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="48" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A48" s="43">
-        <v>47</v>
-      </c>
-      <c r="B48" s="53">
-        <v>0.1513138779322443</v>
-      </c>
-      <c r="C48" s="53">
-        <v>0.13019358763560041</v>
-      </c>
-      <c r="D48" s="53">
-        <v>0.20310956365453001</v>
-      </c>
-      <c r="E48" s="53">
-        <v>0.1067200194772385</v>
-      </c>
-      <c r="F48" s="53">
-        <v>0.17910803542938361</v>
-      </c>
-      <c r="G48" s="54">
-        <v>0.29588315318380942</v>
-      </c>
-      <c r="H48" s="1" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="49" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A49" s="43">
-        <v>48</v>
-      </c>
-      <c r="B49" s="53">
-        <v>0.28227114589511132</v>
-      </c>
-      <c r="C49" s="53">
-        <v>0.15693034721825261</v>
-      </c>
-      <c r="D49" s="53">
-        <v>0.14706785720015811</v>
-      </c>
-      <c r="E49" s="53">
-        <v>0.11490301116561261</v>
-      </c>
-      <c r="F49" s="53">
-        <v>0.28504245940129253</v>
-      </c>
-      <c r="G49" s="54">
-        <v>0.106113889465977</v>
-      </c>
-      <c r="H49" s="1" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="50" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A50" s="43">
-        <v>49</v>
-      </c>
-      <c r="B50" s="53">
-        <v>6.067934013561796E-2</v>
-      </c>
-      <c r="C50" s="53">
-        <v>0.24969350462760331</v>
-      </c>
-      <c r="D50" s="53">
-        <v>0.32763904185265003</v>
-      </c>
-      <c r="E50" s="53">
-        <v>0.20902823633930109</v>
-      </c>
-      <c r="F50" s="53">
-        <v>0.28504245940129253</v>
-      </c>
-      <c r="G50" s="54">
-        <v>0.19826786370595709</v>
-      </c>
-      <c r="H50" s="1" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="51" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A51" s="43">
-        <v>50</v>
-      </c>
-      <c r="B51" s="53">
-        <v>6.067934013561796E-2</v>
-      </c>
-      <c r="C51" s="53">
-        <v>0.26501176682635841</v>
-      </c>
-      <c r="D51" s="53">
-        <v>0.46258193282622911</v>
-      </c>
-      <c r="E51" s="53">
-        <v>0.1037957162819837</v>
-      </c>
-      <c r="F51" s="53">
-        <v>0.10155365833498819</v>
-      </c>
-      <c r="G51" s="54">
-        <v>0.1037612453176729</v>
-      </c>
-      <c r="H51" s="1" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="52" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A52" s="43">
-        <v>51</v>
-      </c>
-      <c r="B52" s="53">
-        <v>0.1175991397677676</v>
-      </c>
-      <c r="C52" s="53">
-        <v>0.1469244388658289</v>
-      </c>
-      <c r="D52" s="53">
-        <v>0.1173714689098652</v>
-      </c>
-      <c r="E52" s="53">
-        <v>0.1067200194772385</v>
-      </c>
-      <c r="F52" s="53">
-        <v>0.11777194028301249</v>
-      </c>
-      <c r="G52" s="54">
-        <v>0.28896487364016582</v>
-      </c>
-      <c r="H52" s="1" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="53" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A53" s="43">
-        <v>52</v>
-      </c>
-      <c r="B53" s="53">
-        <v>0.25800685024111791</v>
-      </c>
-      <c r="C53" s="53">
-        <v>0.17138357282029121</v>
-      </c>
-      <c r="D53" s="53">
-        <v>0.57728791029612658</v>
-      </c>
-      <c r="E53" s="53">
-        <v>0.149464636473506</v>
-      </c>
-      <c r="F53" s="53">
-        <v>0.16748808568104681</v>
-      </c>
-      <c r="G53" s="54">
-        <v>0.29588315318380942</v>
-      </c>
-      <c r="H53" s="1" t="s">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="54" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A54" s="43">
-        <v>53</v>
-      </c>
-      <c r="B54" s="53">
-        <v>0.2053605813455171</v>
-      </c>
-      <c r="C54" s="53">
-        <v>0.10653890295163999</v>
-      </c>
-      <c r="D54" s="53">
-        <v>0.60208365764985095</v>
-      </c>
-      <c r="E54" s="53">
-        <v>0.14254899093197351</v>
-      </c>
-      <c r="F54" s="53">
-        <v>0.29853015698608709</v>
-      </c>
-      <c r="G54" s="54">
-        <v>0.1904581977681119</v>
-      </c>
-      <c r="H54" s="1" t="s">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="55" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A55" s="43">
-        <v>54</v>
-      </c>
-      <c r="B55" s="53">
-        <v>6.067934013561796E-2</v>
-      </c>
-      <c r="C55" s="53">
-        <v>0.1073585477196994</v>
-      </c>
-      <c r="D55" s="53">
-        <v>0.64063348930747244</v>
-      </c>
-      <c r="E55" s="53">
-        <v>0.1142146218775906</v>
-      </c>
-      <c r="F55" s="53">
-        <v>0.20220010699353549</v>
-      </c>
-      <c r="G55" s="54">
-        <v>0.19184264719125629</v>
-      </c>
-      <c r="H55" s="1" t="s">
-        <v>83</v>
-      </c>
-    </row>
-    <row r="56" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A56" s="43">
-        <v>55</v>
-      </c>
-      <c r="B56" s="53">
-        <v>5.3464562024973718E-2</v>
-      </c>
-      <c r="C56" s="53">
-        <v>7.3418276193979989E-2</v>
-      </c>
-      <c r="D56" s="53">
-        <v>0.51226112386527278</v>
-      </c>
-      <c r="E56" s="53">
-        <v>0.1067200194772385</v>
-      </c>
-      <c r="F56" s="53">
-        <v>0.10155365833498819</v>
-      </c>
-      <c r="G56" s="54">
-        <v>0.11036010556078429</v>
-      </c>
-      <c r="H56" s="1" t="s">
-        <v>84</v>
-      </c>
-    </row>
-    <row r="57" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A57" s="43">
-        <v>56</v>
-      </c>
-      <c r="B57" s="53">
-        <v>9.9422997992527795E-2</v>
-      </c>
-      <c r="C57" s="53">
-        <v>0.20485963590004941</v>
-      </c>
-      <c r="D57" s="53">
-        <v>0.1173714689098652</v>
-      </c>
-      <c r="E57" s="53">
-        <v>0.133480215965539</v>
-      </c>
-      <c r="F57" s="53">
-        <v>0.21062885236821061</v>
-      </c>
-      <c r="G57" s="54">
-        <v>0.19903089893942519</v>
-      </c>
-      <c r="H57" s="1" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="58" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A58" s="43">
-        <v>57</v>
-      </c>
-      <c r="B58" s="53">
-        <v>0.27945138447608309</v>
-      </c>
-      <c r="C58" s="53">
-        <v>0.2214529737016164</v>
-      </c>
-      <c r="D58" s="53">
-        <v>0.45978232248877882</v>
-      </c>
-      <c r="E58" s="53">
-        <v>0.1067200194772385</v>
-      </c>
-      <c r="F58" s="53">
-        <v>0.10155365833498819</v>
-      </c>
-      <c r="G58" s="54">
-        <v>0.25945445798155242</v>
-      </c>
-      <c r="H58" s="1" t="s">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="59" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A59" s="43">
-        <v>58</v>
-      </c>
-      <c r="B59" s="53">
-        <v>6.067934013561796E-2</v>
-      </c>
-      <c r="C59" s="53">
-        <v>0.1138701515768725</v>
-      </c>
-      <c r="D59" s="53">
-        <v>0.3090645198651516</v>
-      </c>
-      <c r="E59" s="53">
-        <v>0.1067200194772385</v>
-      </c>
-      <c r="F59" s="53">
-        <v>0.10155365833498819</v>
-      </c>
-      <c r="G59" s="54">
-        <v>0.1037612453176729</v>
-      </c>
-      <c r="H59" s="1" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="60" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A60" s="43">
-        <v>59</v>
-      </c>
-      <c r="B60" s="53">
-        <v>8.4278654950868628E-2</v>
-      </c>
-      <c r="C60" s="53">
-        <v>7.3418276193979989E-2</v>
-      </c>
-      <c r="D60" s="53">
-        <v>0.1173714689098652</v>
-      </c>
-      <c r="E60" s="53">
-        <v>0.12072736402712431</v>
-      </c>
-      <c r="F60" s="53">
-        <v>0.10155365833498819</v>
-      </c>
-      <c r="G60" s="54">
-        <v>0.20599214113259301</v>
-      </c>
-      <c r="H60" s="1" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="61" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A61" s="43">
-        <v>60</v>
-      </c>
-      <c r="B61" s="53">
-        <v>0.11901363367872959</v>
-      </c>
-      <c r="C61" s="53">
-        <v>0.1536416740498148</v>
-      </c>
-      <c r="D61" s="53">
-        <v>0.30696057711104469</v>
-      </c>
-      <c r="E61" s="53">
-        <v>0.1487412317999304</v>
-      </c>
-      <c r="F61" s="53">
-        <v>0.10155365833498819</v>
-      </c>
-      <c r="G61" s="54">
-        <v>0.2398555760396581</v>
-      </c>
-      <c r="H61" s="1" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="62" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A62" s="43">
-        <v>61</v>
-      </c>
-      <c r="B62" s="53">
-        <v>0.25936821240217889</v>
-      </c>
-      <c r="C62" s="53">
-        <v>0.23693484222728531</v>
-      </c>
-      <c r="D62" s="53">
-        <v>0.20852677229958089</v>
-      </c>
-      <c r="E62" s="53">
-        <v>0.18919982941990091</v>
-      </c>
-      <c r="F62" s="53">
-        <v>0.27064667383885299</v>
-      </c>
-      <c r="G62" s="54">
-        <v>0.13390128223747311</v>
-      </c>
-      <c r="H62" s="1" t="s">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="63" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A63" s="43">
-        <v>62</v>
-      </c>
-      <c r="B63" s="53">
-        <v>0.19856365275434321</v>
-      </c>
-      <c r="C63" s="53">
-        <v>0.16050738213281421</v>
-      </c>
-      <c r="D63" s="53">
-        <v>0.1173714689098652</v>
-      </c>
-      <c r="E63" s="53">
-        <v>0.21224472255481461</v>
-      </c>
-      <c r="F63" s="53">
-        <v>0.10155365833498819</v>
-      </c>
-      <c r="G63" s="54">
-        <v>0.25675525644100877</v>
-      </c>
-      <c r="H63" s="1" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="64" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A64" s="43">
-        <v>63</v>
-      </c>
-      <c r="B64" s="53">
-        <v>6.067934013561796E-2</v>
-      </c>
-      <c r="C64" s="53">
-        <v>5.7376663614083813E-2</v>
-      </c>
-      <c r="D64" s="53">
-        <v>0.1173714689098652</v>
-      </c>
-      <c r="E64" s="53">
-        <v>0.11054962373983709</v>
-      </c>
-      <c r="F64" s="53">
-        <v>0.10155365833498819</v>
-      </c>
-      <c r="G64" s="54">
-        <v>0.158852729855506</v>
-      </c>
-      <c r="H64" s="1" t="s">
-        <v>92</v>
-      </c>
-    </row>
-    <row r="65" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A65" s="43">
-        <v>64</v>
-      </c>
-      <c r="B65" s="53">
-        <v>0.28227114589511132</v>
-      </c>
-      <c r="C65" s="53">
-        <v>0.212331678874112</v>
-      </c>
-      <c r="D65" s="53">
-        <v>0.45312359110430561</v>
-      </c>
-      <c r="E65" s="53">
-        <v>0.2490120155106896</v>
-      </c>
-      <c r="F65" s="53">
-        <v>0.1783657868491324</v>
-      </c>
-      <c r="G65" s="54">
-        <v>0.29588315318380942</v>
-      </c>
-      <c r="H65" s="1" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="66" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A66" s="43">
-        <v>65</v>
-      </c>
-      <c r="B66" s="53">
-        <v>0.1190538508732612</v>
-      </c>
-      <c r="C66" s="53">
-        <v>0.1325408991239094</v>
-      </c>
-      <c r="D66" s="53">
-        <v>0.33978523192567822</v>
-      </c>
-      <c r="E66" s="53">
-        <v>0.31638928969095981</v>
-      </c>
-      <c r="F66" s="53">
-        <v>0.2427815164509334</v>
-      </c>
-      <c r="G66" s="54">
-        <v>0.1037612453176729</v>
-      </c>
-      <c r="H66" s="1" t="s">
-        <v>94</v>
-      </c>
-    </row>
-    <row r="67" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A67" s="43">
-        <v>66</v>
-      </c>
-      <c r="B67" s="53">
-        <v>0.116788101821462</v>
-      </c>
-      <c r="C67" s="53">
-        <v>7.3418276193979989E-2</v>
-      </c>
-      <c r="D67" s="53">
-        <v>0.35232499897691949</v>
-      </c>
-      <c r="E67" s="53">
-        <v>0.34265896865144752</v>
-      </c>
-      <c r="F67" s="53">
-        <v>0.10155365833498819</v>
-      </c>
-      <c r="G67" s="54">
-        <v>0.20156419128149439</v>
-      </c>
-      <c r="H67" s="1" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="68" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A68" s="43">
-        <v>67</v>
-      </c>
-      <c r="B68" s="53">
-        <v>5.2068742855322217E-2</v>
-      </c>
-      <c r="C68" s="53">
-        <v>0.25081029847352249</v>
-      </c>
-      <c r="D68" s="53">
-        <v>0.1173714689098652</v>
-      </c>
-      <c r="E68" s="53">
-        <v>0.32257457420205621</v>
-      </c>
-      <c r="F68" s="53">
-        <v>0.22943484656898061</v>
-      </c>
-      <c r="G68" s="54">
-        <v>0.14830624149888891</v>
-      </c>
-      <c r="H68" s="1" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="69" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A69" s="43">
-        <v>68</v>
-      </c>
-      <c r="B69" s="53">
-        <v>0.22758230554703091</v>
-      </c>
-      <c r="C69" s="53">
-        <v>5.115908718075865E-2</v>
-      </c>
-      <c r="D69" s="53">
-        <v>0.1173714689098652</v>
-      </c>
-      <c r="E69" s="53">
-        <v>0.19048771262786501</v>
-      </c>
-      <c r="F69" s="53">
-        <v>0.10155365833498819</v>
-      </c>
-      <c r="G69" s="54">
-        <v>0.1037612453176729</v>
-      </c>
-      <c r="H69" s="1" t="s">
-        <v>97</v>
-      </c>
-    </row>
-    <row r="70" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A70" s="43">
-        <v>69</v>
-      </c>
-      <c r="B70" s="53">
-        <v>0.1350232158513508</v>
-      </c>
-      <c r="C70" s="53">
-        <v>0.12782123382981969</v>
-      </c>
-      <c r="D70" s="53">
-        <v>0.40422497750557268</v>
-      </c>
-      <c r="E70" s="53">
-        <v>0.20234825575670909</v>
-      </c>
-      <c r="F70" s="53">
-        <v>0.10155365833498819</v>
-      </c>
-      <c r="G70" s="54">
-        <v>0.111813182028243</v>
-      </c>
-      <c r="H70" s="1" t="s">
-        <v>98</v>
-      </c>
-    </row>
-    <row r="71" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A71" s="43">
-        <v>70</v>
-      </c>
-      <c r="B71" s="53">
-        <v>0.22701082384268501</v>
-      </c>
-      <c r="C71" s="53">
-        <v>0.19964583053240739</v>
-      </c>
-      <c r="D71" s="53">
-        <v>0.55369081972117706</v>
-      </c>
-      <c r="E71" s="53">
-        <v>0.20288260422305929</v>
-      </c>
-      <c r="F71" s="53">
-        <v>0.1564162547741986</v>
-      </c>
-      <c r="G71" s="54">
-        <v>0.15263963860264779</v>
-      </c>
-      <c r="H71" s="1" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="72" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A72" s="43">
-        <v>71</v>
-      </c>
-      <c r="B72" s="53">
-        <v>0.13118403160571501</v>
-      </c>
-      <c r="C72" s="53">
-        <v>0.22894606623347799</v>
-      </c>
-      <c r="D72" s="53">
-        <v>0.27445535696904622</v>
-      </c>
-      <c r="E72" s="53">
-        <v>0.1067200194772385</v>
-      </c>
-      <c r="F72" s="53">
-        <v>0.1125509934157027</v>
-      </c>
-      <c r="G72" s="54">
-        <v>0.2387384883482179</v>
-      </c>
-      <c r="H72" s="1" t="s">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="73" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A73" s="43">
-        <v>72</v>
-      </c>
-      <c r="B73" s="53">
-        <v>0.1897862689985608</v>
-      </c>
-      <c r="C73" s="53">
-        <v>0.18777241366070119</v>
-      </c>
-      <c r="D73" s="53">
-        <v>0.2016889073478641</v>
-      </c>
-      <c r="E73" s="53">
-        <v>0.1067200194772385</v>
-      </c>
-      <c r="F73" s="53">
-        <v>0.28504245940129253</v>
-      </c>
-      <c r="G73" s="54">
-        <v>0.17386365440714929</v>
-      </c>
-      <c r="H73" s="1" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="74" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A74" s="43">
-        <v>73</v>
-      </c>
-      <c r="B74" s="53">
-        <v>6.067934013561796E-2</v>
-      </c>
-      <c r="C74" s="53">
-        <v>0.19834242346672279</v>
-      </c>
-      <c r="D74" s="53">
-        <v>0.56434929387098109</v>
-      </c>
-      <c r="E74" s="53">
-        <v>0.16085281630366621</v>
-      </c>
-      <c r="F74" s="53">
-        <v>0.16698638705651511</v>
-      </c>
-      <c r="G74" s="54">
-        <v>0.24748103103225411</v>
-      </c>
-      <c r="H74" s="1" t="s">
-        <v>102</v>
-      </c>
-    </row>
-    <row r="75" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A75" s="43">
-        <v>74</v>
-      </c>
-      <c r="B75" s="53">
-        <v>6.0424947634262469E-2</v>
-      </c>
-      <c r="C75" s="53">
-        <v>0.16074902282319159</v>
-      </c>
-      <c r="D75" s="53">
-        <v>0.61878707308067438</v>
-      </c>
-      <c r="E75" s="53">
-        <v>0.1067200194772385</v>
-      </c>
-      <c r="F75" s="53">
-        <v>0.10155365833498819</v>
-      </c>
-      <c r="G75" s="54">
-        <v>0.18242398353369979</v>
-      </c>
-      <c r="H75" s="1" t="s">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="76" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A76" s="43">
-        <v>75</v>
-      </c>
-      <c r="B76" s="53">
-        <v>6.067934013561796E-2</v>
-      </c>
-      <c r="C76" s="53">
-        <v>0.14399758436686641</v>
-      </c>
-      <c r="D76" s="53">
-        <v>0.37818650982603241</v>
-      </c>
-      <c r="E76" s="53">
-        <v>0.23778599127184649</v>
-      </c>
-      <c r="F76" s="53">
-        <v>0.10155365833498819</v>
-      </c>
-      <c r="G76" s="54">
-        <v>0.29588315318380942</v>
-      </c>
-      <c r="H76" s="1" t="s">
-        <v>104</v>
-      </c>
-    </row>
-    <row r="77" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A77" s="43">
-        <v>76</v>
-      </c>
-      <c r="B77" s="53">
-        <v>0.2201644859546123</v>
-      </c>
-      <c r="C77" s="53">
-        <v>7.3418276193979989E-2</v>
-      </c>
-      <c r="D77" s="53">
-        <v>0.1173714689098652</v>
-      </c>
-      <c r="E77" s="53">
-        <v>0.21627562567087549</v>
-      </c>
-      <c r="F77" s="53">
-        <v>0.10155365833498819</v>
-      </c>
-      <c r="G77" s="54">
-        <v>0.13375465841557649</v>
-      </c>
-      <c r="H77" s="1" t="s">
-        <v>105</v>
-      </c>
-    </row>
-    <row r="78" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A78" s="43">
-        <v>77</v>
-      </c>
-      <c r="B78" s="53">
-        <v>0.19012955657250361</v>
-      </c>
-      <c r="C78" s="53">
-        <v>0.2170766766474195</v>
-      </c>
-      <c r="D78" s="53">
-        <v>0.16273560292693731</v>
-      </c>
-      <c r="E78" s="53">
-        <v>0.1067200194772385</v>
-      </c>
-      <c r="F78" s="53">
-        <v>0.15713816585675031</v>
-      </c>
-      <c r="G78" s="54">
-        <v>0.29588315318380942</v>
-      </c>
-      <c r="H78" s="1" t="s">
-        <v>106</v>
-      </c>
-    </row>
-    <row r="79" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A79" s="43">
-        <v>78</v>
-      </c>
-      <c r="B79" s="53">
-        <v>6.067934013561796E-2</v>
-      </c>
-      <c r="C79" s="53">
-        <v>9.863864266867195E-2</v>
-      </c>
-      <c r="D79" s="53">
-        <v>0.62809146099064606</v>
-      </c>
-      <c r="E79" s="53">
-        <v>0.1067200194772385</v>
-      </c>
-      <c r="F79" s="53">
-        <v>0.15797186818884421</v>
-      </c>
-      <c r="G79" s="54">
-        <v>0.223874636619184</v>
-      </c>
-      <c r="H79" s="1" t="s">
-        <v>107</v>
-      </c>
-    </row>
-    <row r="80" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A80" s="43">
-        <v>79</v>
-      </c>
-      <c r="B80" s="53">
-        <v>9.6409140322764958E-2</v>
-      </c>
-      <c r="C80" s="53">
-        <v>0.1178095021537309</v>
-      </c>
-      <c r="D80" s="53">
-        <v>0.36304695434099471</v>
-      </c>
-      <c r="E80" s="53">
-        <v>0.1787578657179677</v>
-      </c>
-      <c r="F80" s="53">
-        <v>0.10155365833498819</v>
-      </c>
-      <c r="G80" s="54">
-        <v>0.1037612453176729</v>
-      </c>
-      <c r="H80" s="1" t="s">
-        <v>108</v>
-      </c>
-    </row>
-    <row r="81" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A81" s="43">
-        <v>80</v>
-      </c>
-      <c r="B81" s="53">
-        <v>0.25862711938542182</v>
-      </c>
-      <c r="C81" s="53">
-        <v>8.0836881656427856E-2</v>
-      </c>
-      <c r="D81" s="53">
-        <v>0.60509302735721415</v>
-      </c>
-      <c r="E81" s="53">
-        <v>0.25731103273616202</v>
-      </c>
-      <c r="F81" s="53">
-        <v>0.1722261835639485</v>
-      </c>
-      <c r="G81" s="54">
-        <v>0.1081123450893785</v>
-      </c>
-      <c r="H81" s="1" t="s">
-        <v>109</v>
-      </c>
-    </row>
-    <row r="82" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A82" s="43">
-        <v>81</v>
-      </c>
-      <c r="B82" s="53">
-        <v>0.25016531147050192</v>
-      </c>
-      <c r="C82" s="53">
-        <v>0.1313251318496359</v>
-      </c>
-      <c r="D82" s="53">
-        <v>0.1173714689098652</v>
-      </c>
-      <c r="E82" s="53">
-        <v>0.1067200194772385</v>
-      </c>
-      <c r="F82" s="53">
-        <v>0.10155365833498819</v>
-      </c>
-      <c r="G82" s="54">
-        <v>0.1037612453176729</v>
-      </c>
-      <c r="H82" s="1" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="83" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A83" s="43">
-        <v>82</v>
-      </c>
-      <c r="B83" s="53">
-        <v>6.067934013561796E-2</v>
-      </c>
-      <c r="C83" s="53">
-        <v>0.2317581568417193</v>
-      </c>
-      <c r="D83" s="53">
-        <v>0.1035525026170963</v>
-      </c>
-      <c r="E83" s="53">
-        <v>0.1341484941667232</v>
-      </c>
-      <c r="F83" s="53">
-        <v>0.10155365833498819</v>
-      </c>
-      <c r="G83" s="54">
-        <v>0.17926553439786669</v>
-      </c>
-      <c r="H83" s="1" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="84" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A84" s="43">
-        <v>83</v>
-      </c>
-      <c r="B84" s="53">
-        <v>0.21345828270069139</v>
-      </c>
-      <c r="C84" s="53">
-        <v>0.15665770887369149</v>
-      </c>
-      <c r="D84" s="53">
-        <v>0.1173714689098652</v>
-      </c>
-      <c r="E84" s="53">
-        <v>0.16917951698405739</v>
-      </c>
-      <c r="F84" s="53">
-        <v>0.10155365833498819</v>
-      </c>
-      <c r="G84" s="54">
-        <v>0.1037612453176729</v>
-      </c>
-      <c r="H84" s="1" t="s">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="85" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A85" s="43">
-        <v>84</v>
-      </c>
-      <c r="B85" s="53">
-        <v>0.1887369497598379</v>
-      </c>
-      <c r="C85" s="53">
-        <v>7.3418276193979989E-2</v>
-      </c>
-      <c r="D85" s="53">
-        <v>0.1173714689098652</v>
-      </c>
-      <c r="E85" s="53">
-        <v>0.1067200194772385</v>
-      </c>
-      <c r="F85" s="53">
-        <v>0.10155365833498819</v>
-      </c>
-      <c r="G85" s="54">
-        <v>0.1329224790637355</v>
-      </c>
-      <c r="H85" s="1" t="s">
-        <v>113</v>
-      </c>
-    </row>
-    <row r="86" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A86" s="43">
-        <v>85</v>
-      </c>
-      <c r="B86" s="53">
-        <v>0.20030730312033859</v>
-      </c>
-      <c r="C86" s="53">
-        <v>8.7786316731294944E-2</v>
-      </c>
-      <c r="D86" s="53">
-        <v>0.1173714689098652</v>
-      </c>
-      <c r="E86" s="53">
-        <v>0.1067200194772385</v>
-      </c>
-      <c r="F86" s="53">
-        <v>0.10155365833498819</v>
-      </c>
-      <c r="G86" s="54">
-        <v>0.29588315318380942</v>
-      </c>
-      <c r="H86" s="1" t="s">
-        <v>114</v>
       </c>
     </row>
   </sheetData>
@@ -4075,7 +2190,7 @@
   <sheetData>
     <row r="1" spans="2:24" x14ac:dyDescent="0.3">
       <c r="B1" s="35" t="s">
-        <v>115</v>
+        <v>50</v>
       </c>
       <c r="C1" s="34">
         <v>1</v>
@@ -4095,7 +2210,7 @@
     </row>
     <row r="2" spans="2:24" x14ac:dyDescent="0.3">
       <c r="B2" s="35" t="s">
-        <v>116</v>
+        <v>51</v>
       </c>
       <c r="C2" s="34">
         <v>1</v>
@@ -4145,10 +2260,10 @@
         <v>9</v>
       </c>
       <c r="L3" s="14" t="s">
-        <v>117</v>
+        <v>52</v>
       </c>
       <c r="M3" s="18" t="s">
-        <v>118</v>
+        <v>53</v>
       </c>
       <c r="R3" s="4" t="s">
         <v>0</v>
@@ -4608,7 +2723,7 @@
     </row>
     <row r="12" spans="2:24" x14ac:dyDescent="0.3">
       <c r="B12" s="57" t="s">
-        <v>119</v>
+        <v>54</v>
       </c>
       <c r="C12" s="61" t="s">
         <v>1</v>
@@ -4626,13 +2741,13 @@
         <v>5</v>
       </c>
       <c r="J12" s="19" t="s">
-        <v>120</v>
+        <v>55</v>
       </c>
       <c r="K12" s="21" t="s">
-        <v>121</v>
+        <v>56</v>
       </c>
       <c r="L12" s="20" t="s">
-        <v>122</v>
+        <v>57</v>
       </c>
     </row>
     <row r="13" spans="2:24" ht="34.950000000000003" customHeight="1" x14ac:dyDescent="0.3">
@@ -4643,16 +2758,16 @@
       <c r="F13" s="60"/>
       <c r="G13" s="64"/>
       <c r="J13" s="19" t="s">
-        <v>123</v>
+        <v>58</v>
       </c>
       <c r="K13" s="22" t="s">
-        <v>124</v>
+        <v>59</v>
       </c>
       <c r="L13" s="17" t="s">
-        <v>125</v>
+        <v>60</v>
       </c>
       <c r="R13" s="44" t="s">
-        <v>126</v>
+        <v>61</v>
       </c>
       <c r="S13" s="48">
         <v>1</v>
@@ -4675,7 +2790,7 @@
     </row>
     <row r="14" spans="2:24" x14ac:dyDescent="0.3">
       <c r="B14" s="9" t="s">
-        <v>127</v>
+        <v>62</v>
       </c>
       <c r="C14" s="2" t="str">
         <f t="array" ref="C14:C20">_xlfn.SORTBY($B$4:$B$10, C4:C10, 1)</f>
@@ -4713,7 +2828,7 @@
     </row>
     <row r="15" spans="2:24" x14ac:dyDescent="0.3">
       <c r="B15" s="9" t="s">
-        <v>128</v>
+        <v>63</v>
       </c>
       <c r="C15" s="2" t="str">
         <v>C</v>
@@ -4740,14 +2855,14 @@
         <v>11</v>
       </c>
       <c r="M15" s="28" t="s">
-        <v>129</v>
+        <v>64</v>
       </c>
       <c r="Q15" s="8"/>
       <c r="R15" s="8"/>
     </row>
     <row r="16" spans="2:24" x14ac:dyDescent="0.3">
       <c r="B16" s="9" t="s">
-        <v>130</v>
+        <v>65</v>
       </c>
       <c r="C16" s="2" t="str">
         <v>D</v>
@@ -4779,7 +2894,7 @@
     <row r="17" spans="1:27" ht="55.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A17" s="5"/>
       <c r="B17" s="9" t="s">
-        <v>131</v>
+        <v>66</v>
       </c>
       <c r="C17" s="2" t="str">
         <v>G</v>
@@ -4831,16 +2946,16 @@
         <v>9</v>
       </c>
       <c r="Z17" s="14" t="s">
-        <v>117</v>
+        <v>52</v>
       </c>
       <c r="AA17" s="18" t="s">
-        <v>118</v>
+        <v>53</v>
       </c>
     </row>
     <row r="18" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A18" s="5"/>
       <c r="B18" s="9" t="s">
-        <v>132</v>
+        <v>67</v>
       </c>
       <c r="C18" s="2" t="str">
         <v>B</v>
@@ -4867,7 +2982,7 @@
         <v>14</v>
       </c>
       <c r="M18" s="28" t="s">
-        <v>129</v>
+        <v>64</v>
       </c>
       <c r="R18" s="10" t="s">
         <v>10</v>
@@ -4912,7 +3027,7 @@
     <row r="19" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A19" s="5"/>
       <c r="B19" s="9" t="s">
-        <v>133</v>
+        <v>68</v>
       </c>
       <c r="C19" s="2" t="str">
         <v>E</v>
@@ -4980,7 +3095,7 @@
     </row>
     <row r="20" spans="1:27" x14ac:dyDescent="0.3">
       <c r="B20" s="9" t="s">
-        <v>134</v>
+        <v>69</v>
       </c>
       <c r="C20" s="2" t="str">
         <v>F</v>
@@ -5048,16 +3163,16 @@
     </row>
     <row r="21" spans="1:27" x14ac:dyDescent="0.3">
       <c r="I21" s="39" t="s">
-        <v>135</v>
+        <v>70</v>
       </c>
       <c r="J21" s="40" t="s">
-        <v>136</v>
+        <v>71</v>
       </c>
       <c r="K21" s="40" t="s">
-        <v>137</v>
+        <v>72</v>
       </c>
       <c r="L21" s="40" t="s">
-        <v>138</v>
+        <v>73</v>
       </c>
       <c r="R21" s="10" t="s">
         <v>13</v>
@@ -5348,7 +3463,7 @@
         <v>8</v>
       </c>
       <c r="Y27" s="33" t="s">
-        <v>139</v>
+        <v>74</v>
       </c>
     </row>
     <row r="28" spans="1:27" x14ac:dyDescent="0.3">
@@ -5759,7 +3874,7 @@
     </row>
     <row r="36" spans="2:25" ht="57" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B36" s="47" t="s">
-        <v>140</v>
+        <v>75</v>
       </c>
       <c r="C36" s="46">
         <v>1</v>
@@ -5792,10 +3907,10 @@
         <v>10</v>
       </c>
       <c r="M36" s="50" t="s">
-        <v>141</v>
+        <v>76</v>
       </c>
       <c r="R36" s="45" t="s">
-        <v>142</v>
+        <v>77</v>
       </c>
     </row>
     <row r="37" spans="2:25" x14ac:dyDescent="0.3">
@@ -6220,7 +4335,7 @@
     </row>
     <row r="44" spans="2:25" x14ac:dyDescent="0.3">
       <c r="B44" s="52" t="s">
-        <v>141</v>
+        <v>76</v>
       </c>
       <c r="C44">
         <f t="shared" ref="C44:M44" si="14">SUM(C37:C43)</f>
@@ -6269,10 +4384,10 @@
     </row>
     <row r="46" spans="2:25" x14ac:dyDescent="0.3">
       <c r="B46" s="41" t="s">
-        <v>143</v>
+        <v>78</v>
       </c>
       <c r="E46" s="41" t="s">
-        <v>144</v>
+        <v>79</v>
       </c>
     </row>
     <row r="47" spans="2:25" x14ac:dyDescent="0.3">
@@ -6290,7 +4405,7 @@
     </row>
     <row r="48" spans="2:25" x14ac:dyDescent="0.3">
       <c r="B48" s="41" t="s">
-        <v>145</v>
+        <v>80</v>
       </c>
     </row>
     <row r="49" spans="2:3" x14ac:dyDescent="0.3">
@@ -6305,7 +4420,7 @@
     </row>
     <row r="50" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B50" s="41" t="s">
-        <v>146</v>
+        <v>81</v>
       </c>
     </row>
     <row r="51" spans="2:3" x14ac:dyDescent="0.3">
@@ -6316,12 +4431,12 @@
     </row>
     <row r="54" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B54" s="41" t="s">
-        <v>147</v>
+        <v>82</v>
       </c>
     </row>
     <row r="55" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B55" s="41" t="s">
-        <v>148</v>
+        <v>83</v>
       </c>
       <c r="C55">
         <f>C49</f>
@@ -6330,7 +4445,7 @@
     </row>
     <row r="56" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B56" s="41" t="s">
-        <v>149</v>
+        <v>84</v>
       </c>
       <c r="C56">
         <v>6</v>
@@ -6338,7 +4453,7 @@
     </row>
     <row r="57" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B57" s="41" t="s">
-        <v>150</v>
+        <v>85</v>
       </c>
       <c r="C57">
         <v>0</v>
@@ -6377,7 +4492,7 @@
   <sheetData>
     <row r="1" spans="2:26" x14ac:dyDescent="0.3">
       <c r="B1" s="35" t="s">
-        <v>115</v>
+        <v>50</v>
       </c>
       <c r="C1" s="34">
         <v>1</v>
@@ -6397,7 +4512,7 @@
     </row>
     <row r="2" spans="2:26" x14ac:dyDescent="0.3">
       <c r="B2" s="35" t="s">
-        <v>116</v>
+        <v>51</v>
       </c>
       <c r="C2" s="34">
         <v>1</v>
@@ -6447,10 +4562,10 @@
         <v>9</v>
       </c>
       <c r="L3" s="14" t="s">
-        <v>117</v>
+        <v>52</v>
       </c>
       <c r="M3" s="18" t="s">
-        <v>118</v>
+        <v>53</v>
       </c>
       <c r="R3" s="4" t="s">
         <v>0</v>
@@ -6910,7 +5025,7 @@
     </row>
     <row r="12" spans="2:26" x14ac:dyDescent="0.3">
       <c r="B12" s="57" t="s">
-        <v>119</v>
+        <v>54</v>
       </c>
       <c r="C12" s="61" t="s">
         <v>1</v>
@@ -6928,19 +5043,19 @@
         <v>5</v>
       </c>
       <c r="J12" s="19" t="s">
-        <v>120</v>
+        <v>55</v>
       </c>
       <c r="K12" s="21" t="s">
-        <v>121</v>
+        <v>56</v>
       </c>
       <c r="L12" s="20" t="s">
-        <v>122</v>
+        <v>57</v>
       </c>
       <c r="Y12" s="51" t="s">
-        <v>151</v>
+        <v>86</v>
       </c>
       <c r="Z12" s="51" t="s">
-        <v>152</v>
+        <v>87</v>
       </c>
     </row>
     <row r="13" spans="2:26" ht="34.950000000000003" customHeight="1" x14ac:dyDescent="0.3">
@@ -6951,16 +5066,16 @@
       <c r="F13" s="60"/>
       <c r="G13" s="64"/>
       <c r="J13" s="19" t="s">
-        <v>123</v>
+        <v>58</v>
       </c>
       <c r="K13" s="22" t="s">
-        <v>124</v>
+        <v>59</v>
       </c>
       <c r="L13" s="17" t="s">
-        <v>125</v>
+        <v>60</v>
       </c>
       <c r="R13" s="44" t="s">
-        <v>126</v>
+        <v>61</v>
       </c>
       <c r="S13" s="48">
         <v>1</v>
@@ -6989,7 +5104,7 @@
     </row>
     <row r="14" spans="2:26" x14ac:dyDescent="0.3">
       <c r="B14" s="9" t="s">
-        <v>127</v>
+        <v>62</v>
       </c>
       <c r="C14" s="2" t="str">
         <f t="array" ref="C14:C20">_xlfn.SORTBY($B$4:$B$10, C4:C10, 1)</f>
@@ -7027,7 +5142,7 @@
     </row>
     <row r="15" spans="2:26" x14ac:dyDescent="0.3">
       <c r="B15" s="9" t="s">
-        <v>128</v>
+        <v>63</v>
       </c>
       <c r="C15" s="2" t="str">
         <v>C</v>
@@ -7054,14 +5169,14 @@
         <v>11</v>
       </c>
       <c r="M15" s="28" t="s">
-        <v>129</v>
+        <v>64</v>
       </c>
       <c r="Q15" s="8"/>
       <c r="R15" s="8"/>
     </row>
     <row r="16" spans="2:26" x14ac:dyDescent="0.3">
       <c r="B16" s="9" t="s">
-        <v>130</v>
+        <v>65</v>
       </c>
       <c r="C16" s="2" t="str">
         <v>D</v>
@@ -7093,7 +5208,7 @@
     <row r="17" spans="1:27" ht="55.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A17" s="5"/>
       <c r="B17" s="9" t="s">
-        <v>131</v>
+        <v>66</v>
       </c>
       <c r="C17" s="2" t="str">
         <v>G</v>
@@ -7145,16 +5260,16 @@
         <v>9</v>
       </c>
       <c r="Z17" s="14" t="s">
-        <v>117</v>
+        <v>52</v>
       </c>
       <c r="AA17" s="18" t="s">
-        <v>118</v>
+        <v>53</v>
       </c>
     </row>
     <row r="18" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A18" s="5"/>
       <c r="B18" s="9" t="s">
-        <v>132</v>
+        <v>67</v>
       </c>
       <c r="C18" s="2" t="str">
         <v>B</v>
@@ -7181,7 +5296,7 @@
         <v>14</v>
       </c>
       <c r="M18" s="28" t="s">
-        <v>129</v>
+        <v>64</v>
       </c>
       <c r="R18" s="10" t="s">
         <v>10</v>
@@ -7226,7 +5341,7 @@
     <row r="19" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A19" s="5"/>
       <c r="B19" s="9" t="s">
-        <v>133</v>
+        <v>68</v>
       </c>
       <c r="C19" s="2" t="str">
         <v>E</v>
@@ -7294,7 +5409,7 @@
     </row>
     <row r="20" spans="1:27" x14ac:dyDescent="0.3">
       <c r="B20" s="9" t="s">
-        <v>134</v>
+        <v>69</v>
       </c>
       <c r="C20" s="2" t="str">
         <v>F</v>
@@ -7362,16 +5477,16 @@
     </row>
     <row r="21" spans="1:27" x14ac:dyDescent="0.3">
       <c r="I21" s="39" t="s">
-        <v>135</v>
+        <v>70</v>
       </c>
       <c r="J21" s="40" t="s">
-        <v>136</v>
+        <v>71</v>
       </c>
       <c r="K21" s="40" t="s">
-        <v>137</v>
+        <v>72</v>
       </c>
       <c r="L21" s="40" t="s">
-        <v>138</v>
+        <v>73</v>
       </c>
       <c r="R21" s="10" t="s">
         <v>13</v>
@@ -7662,7 +5777,7 @@
         <v>8</v>
       </c>
       <c r="Y27" s="33" t="s">
-        <v>139</v>
+        <v>74</v>
       </c>
     </row>
     <row r="28" spans="1:27" x14ac:dyDescent="0.3">
@@ -8073,7 +6188,7 @@
     </row>
     <row r="36" spans="2:25" ht="57" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B36" s="47" t="s">
-        <v>140</v>
+        <v>75</v>
       </c>
       <c r="C36" s="46">
         <v>1</v>
@@ -8106,7 +6221,7 @@
         <v>10</v>
       </c>
       <c r="R36" s="45" t="s">
-        <v>142</v>
+        <v>77</v>
       </c>
     </row>
     <row r="37" spans="2:25" x14ac:dyDescent="0.3">
@@ -8526,7 +6641,7 @@
   <sheetData>
     <row r="1" spans="2:24" x14ac:dyDescent="0.3">
       <c r="B1" s="35" t="s">
-        <v>115</v>
+        <v>50</v>
       </c>
       <c r="C1" s="34">
         <v>1</v>
@@ -8546,7 +6661,7 @@
     </row>
     <row r="2" spans="2:24" x14ac:dyDescent="0.3">
       <c r="B2" s="35" t="s">
-        <v>116</v>
+        <v>51</v>
       </c>
       <c r="C2" s="34">
         <v>1</v>
@@ -8596,10 +6711,10 @@
         <v>9</v>
       </c>
       <c r="L3" s="14" t="s">
-        <v>117</v>
+        <v>52</v>
       </c>
       <c r="M3" s="18" t="s">
-        <v>118</v>
+        <v>53</v>
       </c>
       <c r="R3" s="4" t="s">
         <v>0</v>
@@ -9059,7 +7174,7 @@
     </row>
     <row r="12" spans="2:24" x14ac:dyDescent="0.3">
       <c r="B12" s="57" t="s">
-        <v>119</v>
+        <v>54</v>
       </c>
       <c r="C12" s="61" t="s">
         <v>1</v>
@@ -9077,13 +7192,13 @@
         <v>5</v>
       </c>
       <c r="J12" s="19" t="s">
-        <v>120</v>
+        <v>55</v>
       </c>
       <c r="K12" s="21" t="s">
-        <v>121</v>
+        <v>56</v>
       </c>
       <c r="L12" s="20" t="s">
-        <v>122</v>
+        <v>57</v>
       </c>
     </row>
     <row r="13" spans="2:24" ht="34.950000000000003" customHeight="1" x14ac:dyDescent="0.3">
@@ -9094,16 +7209,16 @@
       <c r="F13" s="60"/>
       <c r="G13" s="64"/>
       <c r="J13" s="19" t="s">
-        <v>123</v>
+        <v>58</v>
       </c>
       <c r="K13" s="22" t="s">
-        <v>124</v>
+        <v>59</v>
       </c>
       <c r="L13" s="17" t="s">
-        <v>125</v>
+        <v>60</v>
       </c>
       <c r="R13" s="44" t="s">
-        <v>126</v>
+        <v>61</v>
       </c>
       <c r="S13" s="48">
         <v>1</v>
@@ -9126,7 +7241,7 @@
     </row>
     <row r="14" spans="2:24" x14ac:dyDescent="0.3">
       <c r="B14" s="9" t="s">
-        <v>127</v>
+        <v>62</v>
       </c>
       <c r="C14" s="2" t="str">
         <f t="array" ref="C14:C20">_xlfn.SORTBY($B$4:$B$10, C4:C10, 1)</f>
@@ -9164,7 +7279,7 @@
     </row>
     <row r="15" spans="2:24" x14ac:dyDescent="0.3">
       <c r="B15" s="9" t="s">
-        <v>128</v>
+        <v>63</v>
       </c>
       <c r="C15" s="2" t="str">
         <v>C</v>
@@ -9191,14 +7306,14 @@
         <v>11</v>
       </c>
       <c r="M15" s="28" t="s">
-        <v>129</v>
+        <v>64</v>
       </c>
       <c r="Q15" s="8"/>
       <c r="R15" s="8"/>
     </row>
     <row r="16" spans="2:24" x14ac:dyDescent="0.3">
       <c r="B16" s="9" t="s">
-        <v>130</v>
+        <v>65</v>
       </c>
       <c r="C16" s="2" t="str">
         <v>D</v>
@@ -9230,7 +7345,7 @@
     <row r="17" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A17" s="5"/>
       <c r="B17" s="9" t="s">
-        <v>131</v>
+        <v>66</v>
       </c>
       <c r="C17" s="2" t="str">
         <v>G</v>
@@ -9262,7 +7377,7 @@
     <row r="18" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A18" s="5"/>
       <c r="B18" s="9" t="s">
-        <v>132</v>
+        <v>67</v>
       </c>
       <c r="C18" s="2" t="str">
         <v>B</v>
@@ -9289,13 +7404,13 @@
         <v>14</v>
       </c>
       <c r="M18" s="28" t="s">
-        <v>129</v>
+        <v>64</v>
       </c>
     </row>
     <row r="19" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A19" s="5"/>
       <c r="B19" s="9" t="s">
-        <v>133</v>
+        <v>68</v>
       </c>
       <c r="C19" s="2" t="str">
         <v>E</v>
@@ -9324,7 +7439,7 @@
     </row>
     <row r="20" spans="1:18" x14ac:dyDescent="0.3">
       <c r="B20" s="9" t="s">
-        <v>134</v>
+        <v>69</v>
       </c>
       <c r="C20" s="2" t="str">
         <v>F</v>
@@ -9353,16 +7468,16 @@
     </row>
     <row r="21" spans="1:18" x14ac:dyDescent="0.3">
       <c r="I21" s="39" t="s">
-        <v>135</v>
+        <v>70</v>
       </c>
       <c r="J21" s="40" t="s">
-        <v>136</v>
+        <v>71</v>
       </c>
       <c r="K21" s="40" t="s">
-        <v>137</v>
+        <v>72</v>
       </c>
       <c r="L21" s="40" t="s">
-        <v>138</v>
+        <v>73</v>
       </c>
     </row>
     <row r="24" spans="1:18" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
@@ -9663,7 +7778,7 @@
     </row>
     <row r="36" spans="2:12" ht="57" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B36" s="47" t="s">
-        <v>140</v>
+        <v>75</v>
       </c>
       <c r="C36" s="46">
         <v>1</v>
@@ -10113,7 +8228,7 @@
   <sheetData>
     <row r="1" spans="2:24" x14ac:dyDescent="0.3">
       <c r="B1" s="35" t="s">
-        <v>115</v>
+        <v>50</v>
       </c>
       <c r="C1" s="34">
         <v>1</v>
@@ -10133,7 +8248,7 @@
     </row>
     <row r="2" spans="2:24" x14ac:dyDescent="0.3">
       <c r="B2" s="35" t="s">
-        <v>116</v>
+        <v>51</v>
       </c>
       <c r="C2" s="34">
         <v>1</v>
@@ -10183,10 +8298,10 @@
         <v>9</v>
       </c>
       <c r="L3" s="14" t="s">
-        <v>117</v>
+        <v>52</v>
       </c>
       <c r="M3" s="18" t="s">
-        <v>118</v>
+        <v>53</v>
       </c>
       <c r="R3" s="4" t="s">
         <v>0</v>
@@ -10646,7 +8761,7 @@
     </row>
     <row r="12" spans="2:24" x14ac:dyDescent="0.3">
       <c r="B12" s="57" t="s">
-        <v>119</v>
+        <v>54</v>
       </c>
       <c r="C12" s="61" t="s">
         <v>1</v>
@@ -10664,13 +8779,13 @@
         <v>5</v>
       </c>
       <c r="J12" s="19" t="s">
-        <v>120</v>
+        <v>55</v>
       </c>
       <c r="K12" s="21" t="s">
-        <v>121</v>
+        <v>56</v>
       </c>
       <c r="L12" s="20" t="s">
-        <v>122</v>
+        <v>57</v>
       </c>
     </row>
     <row r="13" spans="2:24" ht="34.950000000000003" customHeight="1" x14ac:dyDescent="0.3">
@@ -10681,16 +8796,16 @@
       <c r="F13" s="60"/>
       <c r="G13" s="64"/>
       <c r="J13" s="19" t="s">
-        <v>123</v>
+        <v>58</v>
       </c>
       <c r="K13" s="22" t="s">
-        <v>124</v>
+        <v>59</v>
       </c>
       <c r="L13" s="17" t="s">
-        <v>125</v>
+        <v>60</v>
       </c>
       <c r="R13" s="44" t="s">
-        <v>126</v>
+        <v>61</v>
       </c>
       <c r="S13" s="48">
         <v>1</v>
@@ -10713,7 +8828,7 @@
     </row>
     <row r="14" spans="2:24" x14ac:dyDescent="0.3">
       <c r="B14" s="9" t="s">
-        <v>127</v>
+        <v>62</v>
       </c>
       <c r="C14" s="2" t="str">
         <f t="array" ref="C14:C20">_xlfn.SORTBY($B$4:$B$10, C4:C10, 1)</f>
@@ -10750,7 +8865,7 @@
     </row>
     <row r="15" spans="2:24" x14ac:dyDescent="0.3">
       <c r="B15" s="9" t="s">
-        <v>128</v>
+        <v>63</v>
       </c>
       <c r="C15" s="2" t="str">
         <v>C</v>
@@ -10777,14 +8892,14 @@
         <v>11</v>
       </c>
       <c r="M15" s="28" t="s">
-        <v>129</v>
+        <v>64</v>
       </c>
       <c r="Q15" s="8"/>
       <c r="R15" s="8"/>
     </row>
     <row r="16" spans="2:24" x14ac:dyDescent="0.3">
       <c r="B16" s="9" t="s">
-        <v>130</v>
+        <v>65</v>
       </c>
       <c r="C16" s="2" t="str">
         <v>D</v>
@@ -10816,7 +8931,7 @@
     <row r="17" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A17" s="5"/>
       <c r="B17" s="9" t="s">
-        <v>131</v>
+        <v>66</v>
       </c>
       <c r="C17" s="2" t="str">
         <v>G</v>
@@ -10848,7 +8963,7 @@
     <row r="18" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A18" s="5"/>
       <c r="B18" s="9" t="s">
-        <v>132</v>
+        <v>67</v>
       </c>
       <c r="C18" s="2" t="str">
         <v>B</v>
@@ -10875,13 +8990,13 @@
         <v>14</v>
       </c>
       <c r="M18" s="28" t="s">
-        <v>129</v>
+        <v>64</v>
       </c>
     </row>
     <row r="19" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A19" s="5"/>
       <c r="B19" s="9" t="s">
-        <v>133</v>
+        <v>68</v>
       </c>
       <c r="C19" s="2" t="str">
         <v>E</v>
@@ -10910,7 +9025,7 @@
     </row>
     <row r="20" spans="1:18" x14ac:dyDescent="0.3">
       <c r="B20" s="9" t="s">
-        <v>134</v>
+        <v>69</v>
       </c>
       <c r="C20" s="2" t="str">
         <v>F</v>
@@ -10939,16 +9054,16 @@
     </row>
     <row r="21" spans="1:18" x14ac:dyDescent="0.3">
       <c r="I21" s="39" t="s">
-        <v>135</v>
+        <v>70</v>
       </c>
       <c r="J21" s="40" t="s">
-        <v>136</v>
+        <v>71</v>
       </c>
       <c r="K21" s="40" t="s">
-        <v>137</v>
+        <v>72</v>
       </c>
       <c r="L21" s="40" t="s">
-        <v>138</v>
+        <v>73</v>
       </c>
     </row>
     <row r="24" spans="1:18" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
@@ -11249,7 +9364,7 @@
     </row>
     <row r="36" spans="2:12" ht="57" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B36" s="47" t="s">
-        <v>140</v>
+        <v>75</v>
       </c>
       <c r="C36" s="46">
         <v>1</v>
@@ -11696,7 +9811,7 @@
   <sheetData>
     <row r="1" spans="2:18" x14ac:dyDescent="0.3">
       <c r="B1" s="35" t="s">
-        <v>115</v>
+        <v>50</v>
       </c>
       <c r="C1" s="34">
         <v>1</v>
@@ -11716,7 +9831,7 @@
     </row>
     <row r="2" spans="2:18" x14ac:dyDescent="0.3">
       <c r="B2" s="35" t="s">
-        <v>116</v>
+        <v>51</v>
       </c>
       <c r="C2" s="34">
         <v>1</v>
@@ -11766,10 +9881,10 @@
         <v>9</v>
       </c>
       <c r="L3" s="14" t="s">
-        <v>117</v>
+        <v>52</v>
       </c>
       <c r="M3" s="18" t="s">
-        <v>118</v>
+        <v>53</v>
       </c>
     </row>
     <row r="4" spans="2:18" x14ac:dyDescent="0.3">
@@ -12061,7 +10176,7 @@
     </row>
     <row r="12" spans="2:18" x14ac:dyDescent="0.3">
       <c r="B12" s="57" t="s">
-        <v>119</v>
+        <v>54</v>
       </c>
       <c r="C12" s="61" t="s">
         <v>1</v>
@@ -12079,13 +10194,13 @@
         <v>5</v>
       </c>
       <c r="J12" s="19" t="s">
-        <v>120</v>
+        <v>55</v>
       </c>
       <c r="K12" s="21" t="s">
-        <v>121</v>
+        <v>56</v>
       </c>
       <c r="L12" s="20" t="s">
-        <v>122</v>
+        <v>57</v>
       </c>
     </row>
     <row r="13" spans="2:18" ht="34.950000000000003" customHeight="1" x14ac:dyDescent="0.3">
@@ -12096,18 +10211,18 @@
       <c r="F13" s="60"/>
       <c r="G13" s="64"/>
       <c r="J13" s="19" t="s">
-        <v>123</v>
+        <v>58</v>
       </c>
       <c r="K13" s="22" t="s">
-        <v>124</v>
+        <v>59</v>
       </c>
       <c r="L13" s="17" t="s">
-        <v>125</v>
+        <v>60</v>
       </c>
     </row>
     <row r="14" spans="2:18" x14ac:dyDescent="0.3">
       <c r="B14" s="9" t="s">
-        <v>127</v>
+        <v>62</v>
       </c>
       <c r="C14" s="2" t="str">
         <f t="array" ref="C14:C20">_xlfn.SORTBY($B$4:$B$10, C4:C10, 1)</f>
@@ -12145,7 +10260,7 @@
     </row>
     <row r="15" spans="2:18" x14ac:dyDescent="0.3">
       <c r="B15" s="9" t="s">
-        <v>128</v>
+        <v>63</v>
       </c>
       <c r="C15" s="2" t="str">
         <v>C</v>
@@ -12172,14 +10287,14 @@
         <v>11</v>
       </c>
       <c r="M15" s="28" t="s">
-        <v>129</v>
+        <v>64</v>
       </c>
       <c r="Q15" s="8"/>
       <c r="R15" s="8"/>
     </row>
     <row r="16" spans="2:18" x14ac:dyDescent="0.3">
       <c r="B16" s="9" t="s">
-        <v>130</v>
+        <v>65</v>
       </c>
       <c r="C16" s="2" t="str">
         <v>D</v>
@@ -12211,7 +10326,7 @@
     <row r="17" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A17" s="5"/>
       <c r="B17" s="9" t="s">
-        <v>131</v>
+        <v>66</v>
       </c>
       <c r="C17" s="2" t="str">
         <v>G</v>
@@ -12243,7 +10358,7 @@
     <row r="18" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A18" s="5"/>
       <c r="B18" s="9" t="s">
-        <v>132</v>
+        <v>67</v>
       </c>
       <c r="C18" s="2" t="str">
         <v>B</v>
@@ -12270,13 +10385,13 @@
         <v>14</v>
       </c>
       <c r="M18" s="28" t="s">
-        <v>129</v>
+        <v>64</v>
       </c>
     </row>
     <row r="19" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A19" s="5"/>
       <c r="B19" s="9" t="s">
-        <v>133</v>
+        <v>68</v>
       </c>
       <c r="C19" s="2" t="str">
         <v>E</v>
@@ -12305,7 +10420,7 @@
     </row>
     <row r="20" spans="1:18" x14ac:dyDescent="0.3">
       <c r="B20" s="9" t="s">
-        <v>134</v>
+        <v>69</v>
       </c>
       <c r="C20" s="2" t="str">
         <v>F</v>
@@ -12334,42 +10449,42 @@
     </row>
     <row r="21" spans="1:18" x14ac:dyDescent="0.3">
       <c r="I21" s="39" t="s">
-        <v>135</v>
+        <v>70</v>
       </c>
       <c r="J21" s="40" t="s">
-        <v>136</v>
+        <v>71</v>
       </c>
       <c r="K21" s="40" t="s">
-        <v>137</v>
+        <v>72</v>
       </c>
       <c r="L21" s="40" t="s">
-        <v>138</v>
+        <v>73</v>
       </c>
     </row>
     <row r="31" spans="1:18" x14ac:dyDescent="0.3">
-      <c r="B31" s="71" t="s">
-        <v>0</v>
-      </c>
-      <c r="C31" s="68" t="s">
-        <v>153</v>
-      </c>
-      <c r="D31" s="69"/>
-      <c r="E31" s="69"/>
-      <c r="F31" s="69"/>
+      <c r="B31" s="68" t="s">
+        <v>0</v>
+      </c>
+      <c r="C31" s="69" t="s">
+        <v>88</v>
+      </c>
+      <c r="D31" s="70"/>
+      <c r="E31" s="70"/>
+      <c r="F31" s="70"/>
     </row>
     <row r="32" spans="1:18" x14ac:dyDescent="0.3">
       <c r="B32" s="58"/>
-      <c r="C32" s="70"/>
-      <c r="D32" s="69"/>
-      <c r="E32" s="69"/>
-      <c r="F32" s="69"/>
+      <c r="C32" s="71"/>
+      <c r="D32" s="70"/>
+      <c r="E32" s="70"/>
+      <c r="F32" s="70"/>
     </row>
     <row r="33" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B33" s="7" t="s">
         <v>16</v>
       </c>
       <c r="C33" s="65" t="s">
-        <v>154</v>
+        <v>89</v>
       </c>
       <c r="D33" s="66"/>
       <c r="E33" s="66"/>
@@ -12380,7 +10495,7 @@
         <v>13</v>
       </c>
       <c r="C34" s="65" t="s">
-        <v>155</v>
+        <v>90</v>
       </c>
       <c r="D34" s="66"/>
       <c r="E34" s="66"/>
@@ -12391,7 +10506,7 @@
         <v>10</v>
       </c>
       <c r="C35" s="65" t="s">
-        <v>156</v>
+        <v>91</v>
       </c>
       <c r="D35" s="66"/>
       <c r="E35" s="66"/>
@@ -12402,7 +10517,7 @@
         <v>12</v>
       </c>
       <c r="C36" s="65" t="s">
-        <v>157</v>
+        <v>92</v>
       </c>
       <c r="D36" s="66"/>
       <c r="E36" s="66"/>
@@ -12410,10 +10525,10 @@
     </row>
     <row r="37" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B37" s="13" t="s">
-        <v>158</v>
+        <v>93</v>
       </c>
       <c r="C37" s="65" t="s">
-        <v>159</v>
+        <v>94</v>
       </c>
       <c r="D37" s="66"/>
       <c r="E37" s="66"/>
@@ -12424,7 +10539,7 @@
         <v>15</v>
       </c>
       <c r="C38" s="65" t="s">
-        <v>160</v>
+        <v>95</v>
       </c>
       <c r="D38" s="66"/>
       <c r="E38" s="66"/>
@@ -12432,12 +10547,6 @@
     </row>
   </sheetData>
   <mergeCells count="14">
-    <mergeCell ref="B12:B13"/>
-    <mergeCell ref="E12:E13"/>
-    <mergeCell ref="C34:F34"/>
-    <mergeCell ref="C12:C13"/>
-    <mergeCell ref="F12:F13"/>
-    <mergeCell ref="B31:B32"/>
     <mergeCell ref="G12:G13"/>
     <mergeCell ref="C38:F38"/>
     <mergeCell ref="C33:F33"/>
@@ -12446,6 +10555,12 @@
     <mergeCell ref="C37:F37"/>
     <mergeCell ref="C36:F36"/>
     <mergeCell ref="C35:F35"/>
+    <mergeCell ref="B12:B13"/>
+    <mergeCell ref="E12:E13"/>
+    <mergeCell ref="C34:F34"/>
+    <mergeCell ref="C12:C13"/>
+    <mergeCell ref="F12:F13"/>
+    <mergeCell ref="B31:B32"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
bulk update, update to optimization logic, market added as density. necessary modules updated accordingly. Trials done with the new market. excel header etc. renamed
</commit_message>
<xml_diff>
--- a/Arya_Phones_Supplier_Selection.xlsx
+++ b/Arya_Phones_Supplier_Selection.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\LENOVO\Desktop\Asistan\Arya Phone\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6A20A31E-6678-4EAE-8919-6A2CCCD1F14D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F44D1E76-439A-4084-8C10-8A1C9952E830}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -48,7 +48,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="537" uniqueCount="96">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="537" uniqueCount="97">
   <si>
     <t>Supplier</t>
   </si>
@@ -336,6 +336,9 @@
   </si>
   <si>
     <t>High risk and suspected both child labor and banned chemicals.</t>
+  </si>
+  <si>
+    <t>Price Sensitivity</t>
   </si>
 </sst>
 </file>
@@ -791,14 +794,14 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1630,7 +1633,7 @@
         <v>2</v>
       </c>
       <c r="D1" s="15" t="s">
-        <v>3</v>
+        <v>96</v>
       </c>
       <c r="E1" s="15" t="s">
         <v>4</v>
@@ -10462,22 +10465,22 @@
       </c>
     </row>
     <row r="31" spans="1:18" x14ac:dyDescent="0.3">
-      <c r="B31" s="68" t="s">
-        <v>0</v>
-      </c>
-      <c r="C31" s="69" t="s">
+      <c r="B31" s="71" t="s">
+        <v>0</v>
+      </c>
+      <c r="C31" s="68" t="s">
         <v>88</v>
       </c>
-      <c r="D31" s="70"/>
-      <c r="E31" s="70"/>
-      <c r="F31" s="70"/>
+      <c r="D31" s="69"/>
+      <c r="E31" s="69"/>
+      <c r="F31" s="69"/>
     </row>
     <row r="32" spans="1:18" x14ac:dyDescent="0.3">
       <c r="B32" s="58"/>
-      <c r="C32" s="71"/>
-      <c r="D32" s="70"/>
-      <c r="E32" s="70"/>
-      <c r="F32" s="70"/>
+      <c r="C32" s="70"/>
+      <c r="D32" s="69"/>
+      <c r="E32" s="69"/>
+      <c r="F32" s="69"/>
     </row>
     <row r="33" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B33" s="7" t="s">
@@ -10547,6 +10550,12 @@
     </row>
   </sheetData>
   <mergeCells count="14">
+    <mergeCell ref="B12:B13"/>
+    <mergeCell ref="E12:E13"/>
+    <mergeCell ref="C34:F34"/>
+    <mergeCell ref="C12:C13"/>
+    <mergeCell ref="F12:F13"/>
+    <mergeCell ref="B31:B32"/>
     <mergeCell ref="G12:G13"/>
     <mergeCell ref="C38:F38"/>
     <mergeCell ref="C33:F33"/>
@@ -10555,12 +10564,6 @@
     <mergeCell ref="C37:F37"/>
     <mergeCell ref="C36:F36"/>
     <mergeCell ref="C35:F35"/>
-    <mergeCell ref="B12:B13"/>
-    <mergeCell ref="E12:E13"/>
-    <mergeCell ref="C34:F34"/>
-    <mergeCell ref="C12:C13"/>
-    <mergeCell ref="F12:F13"/>
-    <mergeCell ref="B31:B32"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
batch update, remaining is adjustment to UI, adjustments to price's effect.
</commit_message>
<xml_diff>
--- a/Arya_Phones_Supplier_Selection.xlsx
+++ b/Arya_Phones_Supplier_Selection.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\LENOVO\Desktop\Asistan\Arya Phone\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F44D1E76-439A-4084-8C10-8A1C9952E830}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{965119F1-749C-4B01-A8A3-DCA7FB80E1B2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -794,14 +794,14 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1653,25 +1653,25 @@
         <v>1</v>
       </c>
       <c r="B2" s="53">
-        <v>6.2008630366313218E-2</v>
+        <v>0.18141826864259999</v>
       </c>
       <c r="C2" s="53">
-        <v>0.26040571421757103</v>
+        <v>5.4450791916772837E-2</v>
       </c>
       <c r="D2" s="53">
-        <v>0.43524476184674188</v>
+        <v>0.61191053879833257</v>
       </c>
       <c r="E2" s="53">
-        <v>0.1067200194772385</v>
+        <v>0.106720019477238</v>
       </c>
       <c r="F2" s="53">
-        <v>0.10155365833498819</v>
+        <v>0.152651963522863</v>
       </c>
       <c r="G2" s="54">
-        <v>0.2560017363633072</v>
+        <v>0.1037612453176729</v>
       </c>
       <c r="H2" s="1" t="s">
-        <v>30</v>
+        <v>47</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
@@ -1679,25 +1679,25 @@
         <v>2</v>
       </c>
       <c r="B3" s="53">
-        <v>0.1262867946106227</v>
+        <v>0.29731528292090348</v>
       </c>
       <c r="C3" s="53">
-        <v>7.3418276193979989E-2</v>
+        <v>9.1150810219638279E-2</v>
       </c>
       <c r="D3" s="53">
-        <v>0.14790607253205079</v>
+        <v>0.61026173707464948</v>
       </c>
       <c r="E3" s="53">
-        <v>0.29100442200694832</v>
+        <v>0.18945464506061421</v>
       </c>
       <c r="F3" s="53">
-        <v>0.108246470664996</v>
+        <v>0.10155365833498819</v>
       </c>
       <c r="G3" s="54">
-        <v>0.1139929232648282</v>
+        <v>0.29588315318380942</v>
       </c>
       <c r="H3" s="1" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.3">
@@ -1705,25 +1705,25 @@
         <v>3</v>
       </c>
       <c r="B4" s="53">
-        <v>6.067934013561796E-2</v>
+        <v>5.133819847534786E-2</v>
       </c>
       <c r="C4" s="53">
-        <v>6.6813196513184861E-2</v>
+        <v>0.25457641457483893</v>
       </c>
       <c r="D4" s="53">
-        <v>0.36495054503131058</v>
+        <v>0.60726173707464903</v>
       </c>
       <c r="E4" s="53">
-        <v>0.12896323351417149</v>
+        <v>0.24824483374410089</v>
       </c>
       <c r="F4" s="53">
-        <v>0.12518162852531989</v>
+        <v>0.2881274398577503</v>
       </c>
       <c r="G4" s="54">
-        <v>0.21570645620864939</v>
+        <v>0.26426915998857842</v>
       </c>
       <c r="H4" s="1" t="s">
-        <v>32</v>
+        <v>42</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.3">
@@ -1731,25 +1731,25 @@
         <v>4</v>
       </c>
       <c r="B5" s="53">
-        <v>0.19188915259436859</v>
+        <v>0.28227114589511132</v>
       </c>
       <c r="C5" s="53">
-        <v>9.6546504644227593E-2</v>
+        <v>6.516607737331874E-2</v>
       </c>
       <c r="D5" s="53">
-        <v>0.1173714689098652</v>
+        <v>0.58371425606695315</v>
       </c>
       <c r="E5" s="53">
-        <v>0.1067200194772385</v>
+        <v>0.28577314002182541</v>
       </c>
       <c r="F5" s="53">
-        <v>0.10155365833498819</v>
+        <v>0.16710661185701839</v>
       </c>
       <c r="G5" s="54">
-        <v>0.27864380253183429</v>
+        <v>0.15996685766432919</v>
       </c>
       <c r="H5" s="1" t="s">
-        <v>33</v>
+        <v>49</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.3">
@@ -1757,25 +1757,25 @@
         <v>5</v>
       </c>
       <c r="B6" s="53">
-        <v>0.29731528292090348</v>
+        <v>0.1202053717041603</v>
       </c>
       <c r="C6" s="53">
-        <v>9.1150810219638279E-2</v>
+        <v>0.16109848730107321</v>
       </c>
       <c r="D6" s="53">
-        <v>0.61026173707464948</v>
+        <v>0.54893726307541901</v>
       </c>
       <c r="E6" s="53">
-        <v>0.18945464506061421</v>
+        <v>0.17008933186008149</v>
       </c>
       <c r="F6" s="53">
-        <v>0.10155365833498819</v>
+        <v>0.27528967563063772</v>
       </c>
       <c r="G6" s="54">
-        <v>0.29588315318380942</v>
+        <v>0.16758907375405899</v>
       </c>
       <c r="H6" s="1" t="s">
-        <v>34</v>
+        <v>37</v>
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.3">
@@ -1783,25 +1783,25 @@
         <v>6</v>
       </c>
       <c r="B7" s="53">
-        <v>6.4227033173094625E-2</v>
+        <v>6.2008630366313218E-2</v>
       </c>
       <c r="C7" s="53">
-        <v>0.15483029452809721</v>
+        <v>0.26040571421757103</v>
       </c>
       <c r="D7" s="53">
-        <v>0.39507948585385322</v>
+        <v>0.53524476184674197</v>
       </c>
       <c r="E7" s="53">
-        <v>0.16962970966432209</v>
+        <v>0.1067200194772385</v>
       </c>
       <c r="F7" s="53">
         <v>0.10155365833498819</v>
       </c>
       <c r="G7" s="54">
-        <v>0.29345450745565288</v>
+        <v>0.2560017363633072</v>
       </c>
       <c r="H7" s="1" t="s">
-        <v>35</v>
+        <v>30</v>
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.3">
@@ -1809,25 +1809,25 @@
         <v>7</v>
       </c>
       <c r="B8" s="53">
-        <v>0.1039433720356735</v>
+        <v>8.4653338407399248E-2</v>
       </c>
       <c r="C8" s="53">
-        <v>0.19024045650357649</v>
+        <v>0.12208818407051721</v>
       </c>
       <c r="D8" s="53">
-        <v>0.24034996285317831</v>
+        <v>0.50118862071605097</v>
       </c>
       <c r="E8" s="53">
-        <v>0.27804323994842262</v>
+        <v>0.32446059664501697</v>
       </c>
       <c r="F8" s="53">
-        <v>0.119152078029859</v>
+        <v>0.10155365833498819</v>
       </c>
       <c r="G8" s="54">
-        <v>0.1037612453176729</v>
+        <v>0.13823591172591559</v>
       </c>
       <c r="H8" s="1" t="s">
-        <v>36</v>
+        <v>46</v>
       </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.3">
@@ -1835,25 +1835,25 @@
         <v>8</v>
       </c>
       <c r="B9" s="53">
-        <v>0.1202053717041603</v>
+        <v>0.10536952724685961</v>
       </c>
       <c r="C9" s="53">
-        <v>0.16109848730107321</v>
+        <v>0.26693912830951111</v>
       </c>
       <c r="D9" s="53">
-        <v>0.44893726307541931</v>
+        <v>0.47418990241855702</v>
       </c>
       <c r="E9" s="53">
-        <v>0.17008933186008149</v>
+        <v>0.1067200194772385</v>
       </c>
       <c r="F9" s="53">
-        <v>0.27528967563063772</v>
+        <v>0.10155365833498819</v>
       </c>
       <c r="G9" s="54">
-        <v>0.16758907375405899</v>
+        <v>0.1037612453176729</v>
       </c>
       <c r="H9" s="1" t="s">
-        <v>37</v>
+        <v>45</v>
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.3">
@@ -1861,25 +1861,25 @@
         <v>9</v>
       </c>
       <c r="B10" s="53">
-        <v>0.1216495133482835</v>
+        <v>6.4227033173094625E-2</v>
       </c>
       <c r="C10" s="53">
-        <v>0.16985306196136299</v>
+        <v>0.15483029452809721</v>
       </c>
       <c r="D10" s="53">
-        <v>0.28856355425735408</v>
+        <v>0.43507948585385298</v>
       </c>
       <c r="E10" s="53">
-        <v>0.24861374555913729</v>
+        <v>0.16962970966432209</v>
       </c>
       <c r="F10" s="53">
-        <v>0.25064404411660468</v>
+        <v>0.10155365833498819</v>
       </c>
       <c r="G10" s="54">
-        <v>0.16999576138077049</v>
+        <v>0.29345450745565288</v>
       </c>
       <c r="H10" s="1" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.3">
@@ -1887,25 +1887,25 @@
         <v>10</v>
       </c>
       <c r="B11" s="53">
-        <v>5.6765667715111448E-2</v>
+        <v>6.067934013561796E-2</v>
       </c>
       <c r="C11" s="53">
-        <v>0.14383486573349161</v>
+        <v>6.6813196513184861E-2</v>
       </c>
       <c r="D11" s="53">
-        <v>0.1173714689098652</v>
+        <v>0.399950545031311</v>
       </c>
       <c r="E11" s="53">
-        <v>0.183331251224816</v>
+        <v>0.12896323351417149</v>
       </c>
       <c r="F11" s="53">
-        <v>0.10155365833498819</v>
+        <v>0.12518162852531989</v>
       </c>
       <c r="G11" s="54">
-        <v>0.10840881707564209</v>
+        <v>0.21570645620864939</v>
       </c>
       <c r="H11" s="1" t="s">
-        <v>39</v>
+        <v>32</v>
       </c>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.3">
@@ -1913,25 +1913,25 @@
         <v>11</v>
       </c>
       <c r="B12" s="53">
-        <v>6.067934013561796E-2</v>
+        <v>0.1216495133482835</v>
       </c>
       <c r="C12" s="53">
-        <v>0.10691631099167261</v>
+        <v>0.16985306196136299</v>
       </c>
       <c r="D12" s="53">
-        <v>0.1173714689098652</v>
+        <v>0.388563554257354</v>
       </c>
       <c r="E12" s="53">
-        <v>0.29128321359242249</v>
+        <v>0.24861374555913729</v>
       </c>
       <c r="F12" s="53">
-        <v>0.10155365833498819</v>
+        <v>0.25064404411660468</v>
       </c>
       <c r="G12" s="54">
-        <v>0.1096077760804178</v>
+        <v>0.16999576138077049</v>
       </c>
       <c r="H12" s="1" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.3">
@@ -1939,25 +1939,25 @@
         <v>12</v>
       </c>
       <c r="B13" s="53">
-        <v>0.19511378053770029</v>
+        <v>0.1039433720356735</v>
       </c>
       <c r="C13" s="53">
-        <v>7.3418276193979989E-2</v>
+        <v>0.19024045650357649</v>
       </c>
       <c r="D13" s="53">
-        <v>0.1173714689098652</v>
+        <v>0.34034996285317798</v>
       </c>
       <c r="E13" s="53">
-        <v>0.31938813314298031</v>
+        <v>0.27804323994842262</v>
       </c>
       <c r="F13" s="53">
-        <v>0.10155365833498819</v>
+        <v>0.119152078029859</v>
       </c>
       <c r="G13" s="54">
-        <v>0.100629661763317</v>
+        <v>0.1037612453176729</v>
       </c>
       <c r="H13" s="1" t="s">
-        <v>41</v>
+        <v>36</v>
       </c>
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.3">
@@ -1965,25 +1965,25 @@
         <v>13</v>
       </c>
       <c r="B14" s="53">
-        <v>5.133819847534786E-2</v>
+        <v>0.25691282528883602</v>
       </c>
       <c r="C14" s="53">
         <v>0.25457641457483893</v>
       </c>
       <c r="D14" s="53">
-        <v>0.61026173707464948</v>
+        <v>0.28126564060459602</v>
       </c>
       <c r="E14" s="53">
-        <v>0.24824483374410089</v>
+        <v>0.24206895072120549</v>
       </c>
       <c r="F14" s="53">
-        <v>0.2881274398577503</v>
+        <v>0.10155365833498819</v>
       </c>
       <c r="G14" s="54">
-        <v>0.26426915998857842</v>
+        <v>0.1037612453176729</v>
       </c>
       <c r="H14" s="1" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.3">
@@ -1991,25 +1991,25 @@
         <v>14</v>
       </c>
       <c r="B15" s="53">
-        <v>0.28227114589511132</v>
+        <v>0.1262867946106227</v>
       </c>
       <c r="C15" s="53">
         <v>7.3418276193979989E-2</v>
       </c>
       <c r="D15" s="53">
-        <v>0.1173714689098652</v>
+        <v>0.24790607253205099</v>
       </c>
       <c r="E15" s="53">
-        <v>0.102500150077396</v>
+        <v>0.29100442200694832</v>
       </c>
       <c r="F15" s="53">
-        <v>0.1127673895923734</v>
+        <v>0.108246470664996</v>
       </c>
       <c r="G15" s="54">
-        <v>0.1020081514064624</v>
+        <v>0.1139929232648282</v>
       </c>
       <c r="H15" s="1" t="s">
-        <v>43</v>
+        <v>31</v>
       </c>
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.3">
@@ -2017,25 +2017,25 @@
         <v>15</v>
       </c>
       <c r="B16" s="53">
-        <v>0.25691282528883602</v>
+        <v>0.19188915259436859</v>
       </c>
       <c r="C16" s="53">
-        <v>0.25457641457483893</v>
+        <v>9.6546504644227593E-2</v>
       </c>
       <c r="D16" s="53">
-        <v>0.1712656406045957</v>
+        <v>0.21705211340986499</v>
       </c>
       <c r="E16" s="53">
-        <v>0.24206895072120549</v>
+        <v>0.1067200194772385</v>
       </c>
       <c r="F16" s="53">
         <v>0.10155365833498819</v>
       </c>
       <c r="G16" s="54">
-        <v>0.1037612453176729</v>
+        <v>0.27864380253183429</v>
       </c>
       <c r="H16" s="1" t="s">
-        <v>44</v>
+        <v>33</v>
       </c>
     </row>
     <row r="17" spans="1:8" x14ac:dyDescent="0.3">
@@ -2043,25 +2043,25 @@
         <v>16</v>
       </c>
       <c r="B17" s="53">
-        <v>0.10536952724685961</v>
+        <v>0.156765667715111</v>
       </c>
       <c r="C17" s="53">
-        <v>0.26693912830951111</v>
+        <v>0.243834865733492</v>
       </c>
       <c r="D17" s="53">
-        <v>0.42418990241855742</v>
+        <v>0.19145012390986499</v>
       </c>
       <c r="E17" s="53">
-        <v>0.1067200194772385</v>
+        <v>0.183331251224816</v>
       </c>
       <c r="F17" s="53">
-        <v>0.10155365833498819</v>
+        <v>0.20155365833498801</v>
       </c>
       <c r="G17" s="54">
-        <v>0.1037612453176729</v>
+        <v>0.10840881707564209</v>
       </c>
       <c r="H17" s="1" t="s">
-        <v>45</v>
+        <v>39</v>
       </c>
     </row>
     <row r="18" spans="1:8" x14ac:dyDescent="0.3">
@@ -2069,25 +2069,25 @@
         <v>17</v>
       </c>
       <c r="B18" s="53">
-        <v>8.4653338407399248E-2</v>
+        <v>6.067934013561796E-2</v>
       </c>
       <c r="C18" s="53">
-        <v>0.12208818407051721</v>
+        <v>0.10691631099167261</v>
       </c>
       <c r="D18" s="53">
-        <v>0.43518862071605141</v>
+        <v>0.17137146890986499</v>
       </c>
       <c r="E18" s="53">
-        <v>0.32446059664501697</v>
+        <v>0.29128321359242249</v>
       </c>
       <c r="F18" s="53">
-        <v>0.10155365833498819</v>
+        <v>0.23155365833498801</v>
       </c>
       <c r="G18" s="54">
-        <v>0.13823591172591559</v>
+        <v>0.1096077760804178</v>
       </c>
       <c r="H18" s="1" t="s">
-        <v>46</v>
+        <v>40</v>
       </c>
     </row>
     <row r="19" spans="1:8" x14ac:dyDescent="0.3">
@@ -2095,25 +2095,25 @@
         <v>18</v>
       </c>
       <c r="B19" s="53">
-        <v>0.28141826864260022</v>
+        <v>0.19511378053770029</v>
       </c>
       <c r="C19" s="53">
-        <v>5.4450791916772837E-2</v>
+        <v>7.3418276193979989E-2</v>
       </c>
       <c r="D19" s="53">
-        <v>0.61191053879833257</v>
+        <v>0.13737146890986501</v>
       </c>
       <c r="E19" s="53">
-        <v>0.1067200194772385</v>
+        <v>0.31938813314298031</v>
       </c>
       <c r="F19" s="53">
-        <v>0.15265196352286331</v>
+        <v>0.10155365833498819</v>
       </c>
       <c r="G19" s="54">
-        <v>0.1037612453176729</v>
+        <v>0.100629661763317</v>
       </c>
       <c r="H19" s="1" t="s">
-        <v>47</v>
+        <v>41</v>
       </c>
     </row>
     <row r="20" spans="1:8" x14ac:dyDescent="0.3">
@@ -2121,25 +2121,25 @@
         <v>19</v>
       </c>
       <c r="B20" s="53">
-        <v>0.1184919934586543</v>
+        <v>0.28227114589511132</v>
       </c>
       <c r="C20" s="53">
-        <v>0.2048960971299689</v>
+        <v>0.27341827619398001</v>
       </c>
       <c r="D20" s="53">
-        <v>0.1173714689098652</v>
+        <v>0.117371468909865</v>
       </c>
       <c r="E20" s="53">
-        <v>0.1067200194772385</v>
+        <v>0.102500150077396</v>
       </c>
       <c r="F20" s="53">
-        <v>0.10155365833498819</v>
+        <v>0.1127673895923734</v>
       </c>
       <c r="G20" s="54">
-        <v>0.27114700608346642</v>
+        <v>0.1020081514064624</v>
       </c>
       <c r="H20" s="1" t="s">
-        <v>48</v>
+        <v>43</v>
       </c>
     </row>
     <row r="21" spans="1:8" x14ac:dyDescent="0.3">
@@ -2147,25 +2147,25 @@
         <v>20</v>
       </c>
       <c r="B21" s="53">
-        <v>0.28227114589511132</v>
+        <v>0.19849199345865401</v>
       </c>
       <c r="C21" s="53">
-        <v>6.516607737331874E-2</v>
+        <v>0.2048960971299689</v>
       </c>
       <c r="D21" s="53">
-        <v>0.58371425606695315</v>
+        <v>9.7371468909865005E-2</v>
       </c>
       <c r="E21" s="53">
-        <v>0.28577314002182541</v>
+        <v>0.15672001947723799</v>
       </c>
       <c r="F21" s="53">
-        <v>0.16710661185701839</v>
+        <v>0.10155365833498819</v>
       </c>
       <c r="G21" s="54">
-        <v>0.15996685766432919</v>
+        <v>0.27114700608346642</v>
       </c>
       <c r="H21" s="1" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
   </sheetData>
@@ -10465,22 +10465,22 @@
       </c>
     </row>
     <row r="31" spans="1:18" x14ac:dyDescent="0.3">
-      <c r="B31" s="71" t="s">
-        <v>0</v>
-      </c>
-      <c r="C31" s="68" t="s">
+      <c r="B31" s="68" t="s">
+        <v>0</v>
+      </c>
+      <c r="C31" s="69" t="s">
         <v>88</v>
       </c>
-      <c r="D31" s="69"/>
-      <c r="E31" s="69"/>
-      <c r="F31" s="69"/>
+      <c r="D31" s="70"/>
+      <c r="E31" s="70"/>
+      <c r="F31" s="70"/>
     </row>
     <row r="32" spans="1:18" x14ac:dyDescent="0.3">
       <c r="B32" s="58"/>
-      <c r="C32" s="70"/>
-      <c r="D32" s="69"/>
-      <c r="E32" s="69"/>
-      <c r="F32" s="69"/>
+      <c r="C32" s="71"/>
+      <c r="D32" s="70"/>
+      <c r="E32" s="70"/>
+      <c r="F32" s="70"/>
     </row>
     <row r="33" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B33" s="7" t="s">
@@ -10550,12 +10550,6 @@
     </row>
   </sheetData>
   <mergeCells count="14">
-    <mergeCell ref="B12:B13"/>
-    <mergeCell ref="E12:E13"/>
-    <mergeCell ref="C34:F34"/>
-    <mergeCell ref="C12:C13"/>
-    <mergeCell ref="F12:F13"/>
-    <mergeCell ref="B31:B32"/>
     <mergeCell ref="G12:G13"/>
     <mergeCell ref="C38:F38"/>
     <mergeCell ref="C33:F33"/>
@@ -10564,6 +10558,12 @@
     <mergeCell ref="C37:F37"/>
     <mergeCell ref="C36:F36"/>
     <mergeCell ref="C35:F35"/>
+    <mergeCell ref="B12:B13"/>
+    <mergeCell ref="E12:E13"/>
+    <mergeCell ref="C34:F34"/>
+    <mergeCell ref="C12:C13"/>
+    <mergeCell ref="F12:F13"/>
+    <mergeCell ref="B31:B32"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
different supplier categories enforced
</commit_message>
<xml_diff>
--- a/Arya_Phones_Supplier_Selection.xlsx
+++ b/Arya_Phones_Supplier_Selection.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\LENOVO\Desktop\Asistan\Arya Phone\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{965119F1-749C-4B01-A8A3-DCA7FB80E1B2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BABD0C94-E181-445E-8C77-98DF3D42CB3D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Supplier" sheetId="1" r:id="rId1"/>
@@ -48,7 +48,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="537" uniqueCount="97">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="556" uniqueCount="101">
   <si>
     <t>Supplier</t>
   </si>
@@ -339,6 +339,18 @@
   </si>
   <si>
     <t>Price Sensitivity</t>
+  </si>
+  <si>
+    <t>Category</t>
+  </si>
+  <si>
+    <t>keyboard</t>
+  </si>
+  <si>
+    <t>camera</t>
+  </si>
+  <si>
+    <t>cable</t>
   </si>
 </sst>
 </file>
@@ -995,13 +1007,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:J19"/>
+  <dimension ref="A1:K19"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="6" max="6" width="20" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1032,8 +1044,11 @@
       <c r="J1" t="s">
         <v>9</v>
       </c>
-    </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K1" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>10</v>
       </c>
@@ -1064,8 +1079,11 @@
       <c r="J2" s="55">
         <v>13.183999999999999</v>
       </c>
-    </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K2" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>11</v>
       </c>
@@ -1096,8 +1114,11 @@
       <c r="J3" s="55">
         <v>15.289</v>
       </c>
-    </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K3" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>12</v>
       </c>
@@ -1128,8 +1149,11 @@
       <c r="J4" s="55">
         <v>18.82</v>
       </c>
-    </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K4" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>13</v>
       </c>
@@ -1160,8 +1184,11 @@
       <c r="J5" s="55">
         <v>10.851000000000001</v>
       </c>
-    </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K5" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>14</v>
       </c>
@@ -1192,8 +1219,11 @@
       <c r="J6" s="55">
         <v>16.122</v>
       </c>
-    </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K6" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>15</v>
       </c>
@@ -1224,8 +1254,11 @@
       <c r="J7" s="55">
         <v>14.927</v>
       </c>
-    </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K7" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>16</v>
       </c>
@@ -1256,8 +1289,11 @@
       <c r="J8" s="55">
         <v>12.97</v>
       </c>
-    </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K8" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="9" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>17</v>
       </c>
@@ -1288,8 +1324,11 @@
       <c r="J9" s="55">
         <v>14.163</v>
       </c>
-    </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K9" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="10" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>18</v>
       </c>
@@ -1320,8 +1359,11 @@
       <c r="J10" s="55">
         <v>10.255000000000001</v>
       </c>
-    </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K10" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="11" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>19</v>
       </c>
@@ -1352,8 +1394,11 @@
       <c r="J11" s="55">
         <v>14.522</v>
       </c>
-    </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K11" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="12" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>20</v>
       </c>
@@ -1384,8 +1429,11 @@
       <c r="J12" s="55">
         <v>13.813000000000001</v>
       </c>
-    </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K12" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="13" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>21</v>
       </c>
@@ -1416,8 +1464,11 @@
       <c r="J13" s="55">
         <v>11.195</v>
       </c>
-    </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K13" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="14" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>22</v>
       </c>
@@ -1448,8 +1499,11 @@
       <c r="J14" s="55">
         <v>11.151</v>
       </c>
-    </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K14" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="15" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>23</v>
       </c>
@@ -1480,8 +1534,11 @@
       <c r="J15" s="55">
         <v>12.885</v>
       </c>
-    </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K15" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="16" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>24</v>
       </c>
@@ -1512,8 +1569,11 @@
       <c r="J16" s="55">
         <v>13.406000000000001</v>
       </c>
-    </row>
-    <row r="17" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K16" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="17" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>25</v>
       </c>
@@ -1544,8 +1604,11 @@
       <c r="J17" s="55">
         <v>10.837999999999999</v>
       </c>
-    </row>
-    <row r="18" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K17" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="18" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>26</v>
       </c>
@@ -1576,8 +1639,11 @@
       <c r="J18" s="55">
         <v>13.193</v>
       </c>
-    </row>
-    <row r="19" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K18" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="19" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
         <v>27</v>
       </c>
@@ -1607,6 +1673,9 @@
       </c>
       <c r="J19" s="55">
         <v>19.715</v>
+      </c>
+      <c r="K19" t="s">
+        <v>100</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Changes: get rid of unnecessarry columns of the data. Those include strategic importance vs., excluded. All calculations (optimization models vs), updated accordingly. Random events (random audits) added. Penalties are excluded. Leadbord corrected.
</commit_message>
<xml_diff>
--- a/Arya_Phones_Supplier_Selection.xlsx
+++ b/Arya_Phones_Supplier_Selection.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\LENOVO\Desktop\Asistan\Arya Phone\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BABD0C94-E181-445E-8C77-98DF3D42CB3D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DA322D21-0643-4B5A-A016-86D2005A72B5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Supplier" sheetId="1" r:id="rId1"/>
@@ -433,7 +433,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="14">
+  <fills count="17">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -504,6 +504,24 @@
       <patternFill patternType="solid">
         <fgColor theme="0" tint="-0.14999847407452621"/>
         <bgColor indexed="65"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFF0000"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF92D050"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="2"/>
+        <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
@@ -657,7 +675,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="72">
+  <cellXfs count="81">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
@@ -784,7 +802,6 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -806,14 +823,32 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="14" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="164" fontId="0" fillId="14" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="1" fontId="0" fillId="14" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="5" fillId="15" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="15" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="15" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="16" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="1" fontId="0" fillId="16" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="5" fillId="14" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="14" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1010,7 +1045,10 @@
   <dimension ref="A1:K19"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="6" max="6" width="20" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="18.21875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="20" style="71" bestFit="1" customWidth="1"/>
+    <col min="7" max="8" width="8.88671875" style="77"/>
+    <col min="9" max="9" width="8.88671875" style="71"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:11" x14ac:dyDescent="0.3">
@@ -1029,16 +1067,16 @@
       <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="71" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="77" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="77" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="71" t="s">
         <v>8</v>
       </c>
       <c r="J1" t="s">
@@ -1064,16 +1102,16 @@
       <c r="E2" s="55">
         <v>1.9430000000000001</v>
       </c>
-      <c r="F2" s="55">
-        <v>3</v>
-      </c>
-      <c r="G2" s="56">
-        <v>0</v>
-      </c>
-      <c r="H2" s="56">
-        <v>1</v>
-      </c>
-      <c r="I2" s="56">
+      <c r="F2" s="72">
+        <v>3</v>
+      </c>
+      <c r="G2" s="78">
+        <v>0</v>
+      </c>
+      <c r="H2" s="78">
+        <v>1</v>
+      </c>
+      <c r="I2" s="73">
         <v>1</v>
       </c>
       <c r="J2" s="55">
@@ -1099,16 +1137,16 @@
       <c r="E3" s="55">
         <v>1.0640000000000001</v>
       </c>
-      <c r="F3" s="55">
-        <v>4</v>
-      </c>
-      <c r="G3" s="56">
-        <v>0</v>
-      </c>
-      <c r="H3" s="56">
-        <v>0</v>
-      </c>
-      <c r="I3" s="56">
+      <c r="F3" s="72">
+        <v>4</v>
+      </c>
+      <c r="G3" s="78">
+        <v>0</v>
+      </c>
+      <c r="H3" s="78">
+        <v>0</v>
+      </c>
+      <c r="I3" s="73">
         <v>0</v>
       </c>
       <c r="J3" s="55">
@@ -1134,16 +1172,16 @@
       <c r="E4" s="55">
         <v>2.4159999999999999</v>
       </c>
-      <c r="F4" s="55">
+      <c r="F4" s="72">
         <v>1.0980000000000001</v>
       </c>
-      <c r="G4" s="56">
-        <v>0</v>
-      </c>
-      <c r="H4" s="56">
-        <v>0</v>
-      </c>
-      <c r="I4" s="56">
+      <c r="G4" s="78">
+        <v>0</v>
+      </c>
+      <c r="H4" s="78">
+        <v>0</v>
+      </c>
+      <c r="I4" s="73">
         <v>0</v>
       </c>
       <c r="J4" s="55">
@@ -1169,16 +1207,16 @@
       <c r="E5" s="55">
         <v>1.01</v>
       </c>
-      <c r="F5" s="55">
+      <c r="F5" s="72">
         <v>2.823</v>
       </c>
-      <c r="G5" s="56">
-        <v>0</v>
-      </c>
-      <c r="H5" s="56">
-        <v>1</v>
-      </c>
-      <c r="I5" s="56">
+      <c r="G5" s="78">
+        <v>0</v>
+      </c>
+      <c r="H5" s="78">
+        <v>1</v>
+      </c>
+      <c r="I5" s="73">
         <v>0</v>
       </c>
       <c r="J5" s="55">
@@ -1204,16 +1242,16 @@
       <c r="E6" s="55">
         <v>2.0790000000000002</v>
       </c>
-      <c r="F6" s="55">
+      <c r="F6" s="72">
         <v>5</v>
       </c>
-      <c r="G6" s="56">
-        <v>0</v>
-      </c>
-      <c r="H6" s="56">
-        <v>1</v>
-      </c>
-      <c r="I6" s="56">
+      <c r="G6" s="78">
+        <v>0</v>
+      </c>
+      <c r="H6" s="78">
+        <v>1</v>
+      </c>
+      <c r="I6" s="73">
         <v>1</v>
       </c>
       <c r="J6" s="55">
@@ -1239,16 +1277,16 @@
       <c r="E7" s="55">
         <v>1.9950000000000001</v>
       </c>
-      <c r="F7" s="55">
+      <c r="F7" s="72">
         <v>3.234</v>
       </c>
-      <c r="G7" s="56">
-        <v>1</v>
-      </c>
-      <c r="H7" s="56">
-        <v>0</v>
-      </c>
-      <c r="I7" s="56">
+      <c r="G7" s="78">
+        <v>1</v>
+      </c>
+      <c r="H7" s="78">
+        <v>0</v>
+      </c>
+      <c r="I7" s="73">
         <v>0</v>
       </c>
       <c r="J7" s="55">
@@ -1274,16 +1312,16 @@
       <c r="E8" s="55">
         <v>1.796</v>
       </c>
-      <c r="F8" s="55">
+      <c r="F8" s="72">
         <v>4.7770000000000001</v>
       </c>
-      <c r="G8" s="56">
-        <v>0</v>
-      </c>
-      <c r="H8" s="56">
-        <v>1</v>
-      </c>
-      <c r="I8" s="56">
+      <c r="G8" s="78">
+        <v>0</v>
+      </c>
+      <c r="H8" s="78">
+        <v>1</v>
+      </c>
+      <c r="I8" s="73">
         <v>0</v>
       </c>
       <c r="J8" s="55">
@@ -1309,16 +1347,16 @@
       <c r="E9" s="55">
         <v>2.516</v>
       </c>
-      <c r="F9" s="55">
+      <c r="F9" s="72">
         <v>3.234</v>
       </c>
-      <c r="G9" s="56">
-        <v>1</v>
-      </c>
-      <c r="H9" s="56">
-        <v>0</v>
-      </c>
-      <c r="I9" s="56">
+      <c r="G9" s="78">
+        <v>1</v>
+      </c>
+      <c r="H9" s="78">
+        <v>0</v>
+      </c>
+      <c r="I9" s="73">
         <v>0</v>
       </c>
       <c r="J9" s="55">
@@ -1344,16 +1382,16 @@
       <c r="E10" s="55">
         <v>2.323</v>
       </c>
-      <c r="F10" s="55">
+      <c r="F10" s="72">
         <v>4.0999999999999996</v>
       </c>
-      <c r="G10" s="56">
-        <v>0</v>
-      </c>
-      <c r="H10" s="56">
-        <v>0</v>
-      </c>
-      <c r="I10" s="56">
+      <c r="G10" s="78">
+        <v>0</v>
+      </c>
+      <c r="H10" s="78">
+        <v>0</v>
+      </c>
+      <c r="I10" s="73">
         <v>0</v>
       </c>
       <c r="J10" s="55">
@@ -1379,16 +1417,16 @@
       <c r="E11" s="55">
         <v>4.6269999999999998</v>
       </c>
-      <c r="F11" s="55">
+      <c r="F11" s="72">
         <v>3.21</v>
       </c>
-      <c r="G11" s="56">
-        <v>1</v>
-      </c>
-      <c r="H11" s="56">
-        <v>1</v>
-      </c>
-      <c r="I11" s="56">
+      <c r="G11" s="78">
+        <v>1</v>
+      </c>
+      <c r="H11" s="78">
+        <v>1</v>
+      </c>
+      <c r="I11" s="73">
         <v>0</v>
       </c>
       <c r="J11" s="55">
@@ -1414,16 +1452,16 @@
       <c r="E12" s="55">
         <v>1.861</v>
       </c>
-      <c r="F12" s="55">
+      <c r="F12" s="72">
         <v>1.19</v>
       </c>
-      <c r="G12" s="56">
-        <v>1</v>
-      </c>
-      <c r="H12" s="56">
-        <v>1</v>
-      </c>
-      <c r="I12" s="56">
+      <c r="G12" s="78">
+        <v>1</v>
+      </c>
+      <c r="H12" s="78">
+        <v>1</v>
+      </c>
+      <c r="I12" s="73">
         <v>1</v>
       </c>
       <c r="J12" s="55">
@@ -1449,16 +1487,16 @@
       <c r="E13" s="55">
         <v>3.0529999999999999</v>
       </c>
-      <c r="F13" s="55">
+      <c r="F13" s="72">
         <v>1.234</v>
       </c>
-      <c r="G13" s="56">
-        <v>0</v>
-      </c>
-      <c r="H13" s="56">
-        <v>1</v>
-      </c>
-      <c r="I13" s="56">
+      <c r="G13" s="78">
+        <v>0</v>
+      </c>
+      <c r="H13" s="78">
+        <v>1</v>
+      </c>
+      <c r="I13" s="73">
         <v>1</v>
       </c>
       <c r="J13" s="55">
@@ -1484,16 +1522,16 @@
       <c r="E14" s="55">
         <v>1.657</v>
       </c>
-      <c r="F14" s="55">
+      <c r="F14" s="72">
         <v>4.12</v>
       </c>
-      <c r="G14" s="56">
-        <v>0</v>
-      </c>
-      <c r="H14" s="56">
-        <v>0</v>
-      </c>
-      <c r="I14" s="56">
+      <c r="G14" s="78">
+        <v>0</v>
+      </c>
+      <c r="H14" s="78">
+        <v>0</v>
+      </c>
+      <c r="I14" s="73">
         <v>1</v>
       </c>
       <c r="J14" s="55">
@@ -1519,16 +1557,16 @@
       <c r="E15" s="55">
         <v>1.3029999999999999</v>
       </c>
-      <c r="F15" s="55">
-        <v>2</v>
-      </c>
-      <c r="G15" s="56">
-        <v>1</v>
-      </c>
-      <c r="H15" s="56">
-        <v>0</v>
-      </c>
-      <c r="I15" s="56">
+      <c r="F15" s="72">
+        <v>2</v>
+      </c>
+      <c r="G15" s="78">
+        <v>1</v>
+      </c>
+      <c r="H15" s="78">
+        <v>0</v>
+      </c>
+      <c r="I15" s="73">
         <v>0</v>
       </c>
       <c r="J15" s="55">
@@ -1554,16 +1592,16 @@
       <c r="E16" s="55">
         <v>1.405</v>
       </c>
-      <c r="F16" s="55">
+      <c r="F16" s="72">
         <v>4.4000000000000004</v>
       </c>
-      <c r="G16" s="56">
-        <v>1</v>
-      </c>
-      <c r="H16" s="56">
-        <v>0</v>
-      </c>
-      <c r="I16" s="56">
+      <c r="G16" s="78">
+        <v>1</v>
+      </c>
+      <c r="H16" s="78">
+        <v>0</v>
+      </c>
+      <c r="I16" s="73">
         <v>0</v>
       </c>
       <c r="J16" s="55">
@@ -1589,16 +1627,16 @@
       <c r="E17" s="55">
         <v>3.6720000000000002</v>
       </c>
-      <c r="F17" s="55">
-        <v>2</v>
-      </c>
-      <c r="G17" s="56">
-        <v>0</v>
-      </c>
-      <c r="H17" s="56">
-        <v>0</v>
-      </c>
-      <c r="I17" s="56">
+      <c r="F17" s="72">
+        <v>2</v>
+      </c>
+      <c r="G17" s="78">
+        <v>0</v>
+      </c>
+      <c r="H17" s="78">
+        <v>0</v>
+      </c>
+      <c r="I17" s="73">
         <v>1</v>
       </c>
       <c r="J17" s="55">
@@ -1624,16 +1662,16 @@
       <c r="E18" s="55">
         <v>1.806</v>
       </c>
-      <c r="F18" s="55">
+      <c r="F18" s="72">
         <v>2.234</v>
       </c>
-      <c r="G18" s="56">
-        <v>1</v>
-      </c>
-      <c r="H18" s="56">
-        <v>0</v>
-      </c>
-      <c r="I18" s="56">
+      <c r="G18" s="78">
+        <v>1</v>
+      </c>
+      <c r="H18" s="78">
+        <v>0</v>
+      </c>
+      <c r="I18" s="73">
         <v>1</v>
       </c>
       <c r="J18" s="55">
@@ -1659,16 +1697,16 @@
       <c r="E19" s="55">
         <v>3.8740000000000001</v>
       </c>
-      <c r="F19" s="55">
+      <c r="F19" s="72">
         <v>0.23400000000000001</v>
       </c>
-      <c r="G19" s="56">
-        <v>1</v>
-      </c>
-      <c r="H19" s="56">
-        <v>0</v>
-      </c>
-      <c r="I19" s="56">
+      <c r="G19" s="78">
+        <v>1</v>
+      </c>
+      <c r="H19" s="78">
+        <v>0</v>
+      </c>
+      <c r="I19" s="73">
         <v>0</v>
       </c>
       <c r="J19" s="55">
@@ -1688,6 +1726,8 @@
   <dimension ref="A1:H21"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
+    <col min="4" max="4" width="8.88671875" style="76"/>
+    <col min="5" max="6" width="8.88671875" style="71"/>
     <col min="8" max="8" width="39.6640625" customWidth="1"/>
   </cols>
   <sheetData>
@@ -1701,13 +1741,13 @@
       <c r="C1" s="15" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="15" t="s">
+      <c r="D1" s="74" t="s">
         <v>96</v>
       </c>
-      <c r="E1" s="15" t="s">
-        <v>4</v>
-      </c>
-      <c r="F1" s="15" t="s">
+      <c r="E1" s="79" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="79" t="s">
         <v>5</v>
       </c>
       <c r="G1" s="17" t="s">
@@ -1727,13 +1767,13 @@
       <c r="C2" s="53">
         <v>5.4450791916772837E-2</v>
       </c>
-      <c r="D2" s="53">
+      <c r="D2" s="75">
         <v>0.61191053879833257</v>
       </c>
-      <c r="E2" s="53">
+      <c r="E2" s="80">
         <v>0.106720019477238</v>
       </c>
-      <c r="F2" s="53">
+      <c r="F2" s="80">
         <v>0.152651963522863</v>
       </c>
       <c r="G2" s="54">
@@ -1753,13 +1793,13 @@
       <c r="C3" s="53">
         <v>9.1150810219638279E-2</v>
       </c>
-      <c r="D3" s="53">
+      <c r="D3" s="75">
         <v>0.61026173707464948</v>
       </c>
-      <c r="E3" s="53">
+      <c r="E3" s="80">
         <v>0.18945464506061421</v>
       </c>
-      <c r="F3" s="53">
+      <c r="F3" s="80">
         <v>0.10155365833498819</v>
       </c>
       <c r="G3" s="54">
@@ -1779,13 +1819,13 @@
       <c r="C4" s="53">
         <v>0.25457641457483893</v>
       </c>
-      <c r="D4" s="53">
+      <c r="D4" s="75">
         <v>0.60726173707464903</v>
       </c>
-      <c r="E4" s="53">
+      <c r="E4" s="80">
         <v>0.24824483374410089</v>
       </c>
-      <c r="F4" s="53">
+      <c r="F4" s="80">
         <v>0.2881274398577503</v>
       </c>
       <c r="G4" s="54">
@@ -1805,13 +1845,13 @@
       <c r="C5" s="53">
         <v>6.516607737331874E-2</v>
       </c>
-      <c r="D5" s="53">
+      <c r="D5" s="75">
         <v>0.58371425606695315</v>
       </c>
-      <c r="E5" s="53">
+      <c r="E5" s="80">
         <v>0.28577314002182541</v>
       </c>
-      <c r="F5" s="53">
+      <c r="F5" s="80">
         <v>0.16710661185701839</v>
       </c>
       <c r="G5" s="54">
@@ -1831,13 +1871,13 @@
       <c r="C6" s="53">
         <v>0.16109848730107321</v>
       </c>
-      <c r="D6" s="53">
+      <c r="D6" s="75">
         <v>0.54893726307541901</v>
       </c>
-      <c r="E6" s="53">
+      <c r="E6" s="80">
         <v>0.17008933186008149</v>
       </c>
-      <c r="F6" s="53">
+      <c r="F6" s="80">
         <v>0.27528967563063772</v>
       </c>
       <c r="G6" s="54">
@@ -1857,13 +1897,13 @@
       <c r="C7" s="53">
         <v>0.26040571421757103</v>
       </c>
-      <c r="D7" s="53">
+      <c r="D7" s="75">
         <v>0.53524476184674197</v>
       </c>
-      <c r="E7" s="53">
+      <c r="E7" s="80">
         <v>0.1067200194772385</v>
       </c>
-      <c r="F7" s="53">
+      <c r="F7" s="80">
         <v>0.10155365833498819</v>
       </c>
       <c r="G7" s="54">
@@ -1883,13 +1923,13 @@
       <c r="C8" s="53">
         <v>0.12208818407051721</v>
       </c>
-      <c r="D8" s="53">
+      <c r="D8" s="75">
         <v>0.50118862071605097</v>
       </c>
-      <c r="E8" s="53">
+      <c r="E8" s="80">
         <v>0.32446059664501697</v>
       </c>
-      <c r="F8" s="53">
+      <c r="F8" s="80">
         <v>0.10155365833498819</v>
       </c>
       <c r="G8" s="54">
@@ -1909,13 +1949,13 @@
       <c r="C9" s="53">
         <v>0.26693912830951111</v>
       </c>
-      <c r="D9" s="53">
+      <c r="D9" s="75">
         <v>0.47418990241855702</v>
       </c>
-      <c r="E9" s="53">
+      <c r="E9" s="80">
         <v>0.1067200194772385</v>
       </c>
-      <c r="F9" s="53">
+      <c r="F9" s="80">
         <v>0.10155365833498819</v>
       </c>
       <c r="G9" s="54">
@@ -1935,13 +1975,13 @@
       <c r="C10" s="53">
         <v>0.15483029452809721</v>
       </c>
-      <c r="D10" s="53">
+      <c r="D10" s="75">
         <v>0.43507948585385298</v>
       </c>
-      <c r="E10" s="53">
+      <c r="E10" s="80">
         <v>0.16962970966432209</v>
       </c>
-      <c r="F10" s="53">
+      <c r="F10" s="80">
         <v>0.10155365833498819</v>
       </c>
       <c r="G10" s="54">
@@ -1961,13 +2001,13 @@
       <c r="C11" s="53">
         <v>6.6813196513184861E-2</v>
       </c>
-      <c r="D11" s="53">
+      <c r="D11" s="75">
         <v>0.399950545031311</v>
       </c>
-      <c r="E11" s="53">
+      <c r="E11" s="80">
         <v>0.12896323351417149</v>
       </c>
-      <c r="F11" s="53">
+      <c r="F11" s="80">
         <v>0.12518162852531989</v>
       </c>
       <c r="G11" s="54">
@@ -1987,13 +2027,13 @@
       <c r="C12" s="53">
         <v>0.16985306196136299</v>
       </c>
-      <c r="D12" s="53">
+      <c r="D12" s="75">
         <v>0.388563554257354</v>
       </c>
-      <c r="E12" s="53">
+      <c r="E12" s="80">
         <v>0.24861374555913729</v>
       </c>
-      <c r="F12" s="53">
+      <c r="F12" s="80">
         <v>0.25064404411660468</v>
       </c>
       <c r="G12" s="54">
@@ -2013,13 +2053,13 @@
       <c r="C13" s="53">
         <v>0.19024045650357649</v>
       </c>
-      <c r="D13" s="53">
+      <c r="D13" s="75">
         <v>0.34034996285317798</v>
       </c>
-      <c r="E13" s="53">
+      <c r="E13" s="80">
         <v>0.27804323994842262</v>
       </c>
-      <c r="F13" s="53">
+      <c r="F13" s="80">
         <v>0.119152078029859</v>
       </c>
       <c r="G13" s="54">
@@ -2039,13 +2079,13 @@
       <c r="C14" s="53">
         <v>0.25457641457483893</v>
       </c>
-      <c r="D14" s="53">
+      <c r="D14" s="75">
         <v>0.28126564060459602</v>
       </c>
-      <c r="E14" s="53">
+      <c r="E14" s="80">
         <v>0.24206895072120549</v>
       </c>
-      <c r="F14" s="53">
+      <c r="F14" s="80">
         <v>0.10155365833498819</v>
       </c>
       <c r="G14" s="54">
@@ -2065,13 +2105,13 @@
       <c r="C15" s="53">
         <v>7.3418276193979989E-2</v>
       </c>
-      <c r="D15" s="53">
+      <c r="D15" s="75">
         <v>0.24790607253205099</v>
       </c>
-      <c r="E15" s="53">
+      <c r="E15" s="80">
         <v>0.29100442200694832</v>
       </c>
-      <c r="F15" s="53">
+      <c r="F15" s="80">
         <v>0.108246470664996</v>
       </c>
       <c r="G15" s="54">
@@ -2091,13 +2131,13 @@
       <c r="C16" s="53">
         <v>9.6546504644227593E-2</v>
       </c>
-      <c r="D16" s="53">
+      <c r="D16" s="75">
         <v>0.21705211340986499</v>
       </c>
-      <c r="E16" s="53">
+      <c r="E16" s="80">
         <v>0.1067200194772385</v>
       </c>
-      <c r="F16" s="53">
+      <c r="F16" s="80">
         <v>0.10155365833498819</v>
       </c>
       <c r="G16" s="54">
@@ -2117,13 +2157,13 @@
       <c r="C17" s="53">
         <v>0.243834865733492</v>
       </c>
-      <c r="D17" s="53">
+      <c r="D17" s="75">
         <v>0.19145012390986499</v>
       </c>
-      <c r="E17" s="53">
+      <c r="E17" s="80">
         <v>0.183331251224816</v>
       </c>
-      <c r="F17" s="53">
+      <c r="F17" s="80">
         <v>0.20155365833498801</v>
       </c>
       <c r="G17" s="54">
@@ -2143,13 +2183,13 @@
       <c r="C18" s="53">
         <v>0.10691631099167261</v>
       </c>
-      <c r="D18" s="53">
+      <c r="D18" s="75">
         <v>0.17137146890986499</v>
       </c>
-      <c r="E18" s="53">
+      <c r="E18" s="80">
         <v>0.29128321359242249</v>
       </c>
-      <c r="F18" s="53">
+      <c r="F18" s="80">
         <v>0.23155365833498801</v>
       </c>
       <c r="G18" s="54">
@@ -2169,13 +2209,13 @@
       <c r="C19" s="53">
         <v>7.3418276193979989E-2</v>
       </c>
-      <c r="D19" s="53">
+      <c r="D19" s="75">
         <v>0.13737146890986501</v>
       </c>
-      <c r="E19" s="53">
+      <c r="E19" s="80">
         <v>0.31938813314298031</v>
       </c>
-      <c r="F19" s="53">
+      <c r="F19" s="80">
         <v>0.10155365833498819</v>
       </c>
       <c r="G19" s="54">
@@ -2195,13 +2235,13 @@
       <c r="C20" s="53">
         <v>0.27341827619398001</v>
       </c>
-      <c r="D20" s="53">
+      <c r="D20" s="75">
         <v>0.117371468909865</v>
       </c>
-      <c r="E20" s="53">
+      <c r="E20" s="80">
         <v>0.102500150077396</v>
       </c>
-      <c r="F20" s="53">
+      <c r="F20" s="80">
         <v>0.1127673895923734</v>
       </c>
       <c r="G20" s="54">
@@ -2221,13 +2261,13 @@
       <c r="C21" s="53">
         <v>0.2048960971299689</v>
       </c>
-      <c r="D21" s="53">
+      <c r="D21" s="75">
         <v>9.7371468909865005E-2</v>
       </c>
-      <c r="E21" s="53">
+      <c r="E21" s="80">
         <v>0.15672001947723799</v>
       </c>
-      <c r="F21" s="53">
+      <c r="F21" s="80">
         <v>0.10155365833498819</v>
       </c>
       <c r="G21" s="54">
@@ -2794,22 +2834,22 @@
       </c>
     </row>
     <row r="12" spans="2:24" x14ac:dyDescent="0.3">
-      <c r="B12" s="57" t="s">
+      <c r="B12" s="56" t="s">
         <v>54</v>
       </c>
-      <c r="C12" s="61" t="s">
-        <v>1</v>
-      </c>
-      <c r="D12" s="59" t="s">
-        <v>2</v>
-      </c>
-      <c r="E12" s="59" t="s">
-        <v>3</v>
-      </c>
-      <c r="F12" s="59" t="s">
-        <v>4</v>
-      </c>
-      <c r="G12" s="63" t="s">
+      <c r="C12" s="60" t="s">
+        <v>1</v>
+      </c>
+      <c r="D12" s="58" t="s">
+        <v>2</v>
+      </c>
+      <c r="E12" s="58" t="s">
+        <v>3</v>
+      </c>
+      <c r="F12" s="58" t="s">
+        <v>4</v>
+      </c>
+      <c r="G12" s="62" t="s">
         <v>5</v>
       </c>
       <c r="J12" s="19" t="s">
@@ -2823,12 +2863,12 @@
       </c>
     </row>
     <row r="13" spans="2:24" ht="34.950000000000003" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B13" s="58"/>
-      <c r="C13" s="62"/>
-      <c r="D13" s="60"/>
-      <c r="E13" s="60"/>
-      <c r="F13" s="60"/>
-      <c r="G13" s="64"/>
+      <c r="B13" s="57"/>
+      <c r="C13" s="61"/>
+      <c r="D13" s="59"/>
+      <c r="E13" s="59"/>
+      <c r="F13" s="59"/>
+      <c r="G13" s="63"/>
       <c r="J13" s="19" t="s">
         <v>58</v>
       </c>
@@ -5096,22 +5136,22 @@
       </c>
     </row>
     <row r="12" spans="2:26" x14ac:dyDescent="0.3">
-      <c r="B12" s="57" t="s">
+      <c r="B12" s="56" t="s">
         <v>54</v>
       </c>
-      <c r="C12" s="61" t="s">
-        <v>1</v>
-      </c>
-      <c r="D12" s="59" t="s">
-        <v>2</v>
-      </c>
-      <c r="E12" s="59" t="s">
-        <v>3</v>
-      </c>
-      <c r="F12" s="59" t="s">
-        <v>4</v>
-      </c>
-      <c r="G12" s="63" t="s">
+      <c r="C12" s="60" t="s">
+        <v>1</v>
+      </c>
+      <c r="D12" s="58" t="s">
+        <v>2</v>
+      </c>
+      <c r="E12" s="58" t="s">
+        <v>3</v>
+      </c>
+      <c r="F12" s="58" t="s">
+        <v>4</v>
+      </c>
+      <c r="G12" s="62" t="s">
         <v>5</v>
       </c>
       <c r="J12" s="19" t="s">
@@ -5131,12 +5171,12 @@
       </c>
     </row>
     <row r="13" spans="2:26" ht="34.950000000000003" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B13" s="58"/>
-      <c r="C13" s="62"/>
-      <c r="D13" s="60"/>
-      <c r="E13" s="60"/>
-      <c r="F13" s="60"/>
-      <c r="G13" s="64"/>
+      <c r="B13" s="57"/>
+      <c r="C13" s="61"/>
+      <c r="D13" s="59"/>
+      <c r="E13" s="59"/>
+      <c r="F13" s="59"/>
+      <c r="G13" s="63"/>
       <c r="J13" s="19" t="s">
         <v>58</v>
       </c>
@@ -7245,22 +7285,22 @@
       </c>
     </row>
     <row r="12" spans="2:24" x14ac:dyDescent="0.3">
-      <c r="B12" s="57" t="s">
+      <c r="B12" s="56" t="s">
         <v>54</v>
       </c>
-      <c r="C12" s="61" t="s">
-        <v>1</v>
-      </c>
-      <c r="D12" s="59" t="s">
-        <v>2</v>
-      </c>
-      <c r="E12" s="59" t="s">
-        <v>3</v>
-      </c>
-      <c r="F12" s="59" t="s">
-        <v>4</v>
-      </c>
-      <c r="G12" s="63" t="s">
+      <c r="C12" s="60" t="s">
+        <v>1</v>
+      </c>
+      <c r="D12" s="58" t="s">
+        <v>2</v>
+      </c>
+      <c r="E12" s="58" t="s">
+        <v>3</v>
+      </c>
+      <c r="F12" s="58" t="s">
+        <v>4</v>
+      </c>
+      <c r="G12" s="62" t="s">
         <v>5</v>
       </c>
       <c r="J12" s="19" t="s">
@@ -7274,12 +7314,12 @@
       </c>
     </row>
     <row r="13" spans="2:24" ht="34.950000000000003" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B13" s="58"/>
-      <c r="C13" s="62"/>
-      <c r="D13" s="60"/>
-      <c r="E13" s="60"/>
-      <c r="F13" s="60"/>
-      <c r="G13" s="64"/>
+      <c r="B13" s="57"/>
+      <c r="C13" s="61"/>
+      <c r="D13" s="59"/>
+      <c r="E13" s="59"/>
+      <c r="F13" s="59"/>
+      <c r="G13" s="63"/>
       <c r="J13" s="19" t="s">
         <v>58</v>
       </c>
@@ -8832,22 +8872,22 @@
       </c>
     </row>
     <row r="12" spans="2:24" x14ac:dyDescent="0.3">
-      <c r="B12" s="57" t="s">
+      <c r="B12" s="56" t="s">
         <v>54</v>
       </c>
-      <c r="C12" s="61" t="s">
-        <v>1</v>
-      </c>
-      <c r="D12" s="59" t="s">
-        <v>2</v>
-      </c>
-      <c r="E12" s="59" t="s">
-        <v>3</v>
-      </c>
-      <c r="F12" s="59" t="s">
-        <v>4</v>
-      </c>
-      <c r="G12" s="63" t="s">
+      <c r="C12" s="60" t="s">
+        <v>1</v>
+      </c>
+      <c r="D12" s="58" t="s">
+        <v>2</v>
+      </c>
+      <c r="E12" s="58" t="s">
+        <v>3</v>
+      </c>
+      <c r="F12" s="58" t="s">
+        <v>4</v>
+      </c>
+      <c r="G12" s="62" t="s">
         <v>5</v>
       </c>
       <c r="J12" s="19" t="s">
@@ -8861,12 +8901,12 @@
       </c>
     </row>
     <row r="13" spans="2:24" ht="34.950000000000003" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B13" s="58"/>
-      <c r="C13" s="62"/>
-      <c r="D13" s="60"/>
-      <c r="E13" s="60"/>
-      <c r="F13" s="60"/>
-      <c r="G13" s="64"/>
+      <c r="B13" s="57"/>
+      <c r="C13" s="61"/>
+      <c r="D13" s="59"/>
+      <c r="E13" s="59"/>
+      <c r="F13" s="59"/>
+      <c r="G13" s="63"/>
       <c r="J13" s="19" t="s">
         <v>58</v>
       </c>
@@ -10247,22 +10287,22 @@
       </c>
     </row>
     <row r="12" spans="2:18" x14ac:dyDescent="0.3">
-      <c r="B12" s="57" t="s">
+      <c r="B12" s="56" t="s">
         <v>54</v>
       </c>
-      <c r="C12" s="61" t="s">
-        <v>1</v>
-      </c>
-      <c r="D12" s="59" t="s">
-        <v>2</v>
-      </c>
-      <c r="E12" s="59" t="s">
-        <v>3</v>
-      </c>
-      <c r="F12" s="59" t="s">
-        <v>4</v>
-      </c>
-      <c r="G12" s="63" t="s">
+      <c r="C12" s="60" t="s">
+        <v>1</v>
+      </c>
+      <c r="D12" s="58" t="s">
+        <v>2</v>
+      </c>
+      <c r="E12" s="58" t="s">
+        <v>3</v>
+      </c>
+      <c r="F12" s="58" t="s">
+        <v>4</v>
+      </c>
+      <c r="G12" s="62" t="s">
         <v>5</v>
       </c>
       <c r="J12" s="19" t="s">
@@ -10276,12 +10316,12 @@
       </c>
     </row>
     <row r="13" spans="2:18" ht="34.950000000000003" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B13" s="58"/>
-      <c r="C13" s="62"/>
-      <c r="D13" s="60"/>
-      <c r="E13" s="60"/>
-      <c r="F13" s="60"/>
-      <c r="G13" s="64"/>
+      <c r="B13" s="57"/>
+      <c r="C13" s="61"/>
+      <c r="D13" s="59"/>
+      <c r="E13" s="59"/>
+      <c r="F13" s="59"/>
+      <c r="G13" s="63"/>
       <c r="J13" s="19" t="s">
         <v>58</v>
       </c>
@@ -10534,91 +10574,97 @@
       </c>
     </row>
     <row r="31" spans="1:18" x14ac:dyDescent="0.3">
-      <c r="B31" s="68" t="s">
-        <v>0</v>
-      </c>
-      <c r="C31" s="69" t="s">
+      <c r="B31" s="70" t="s">
+        <v>0</v>
+      </c>
+      <c r="C31" s="67" t="s">
         <v>88</v>
       </c>
-      <c r="D31" s="70"/>
-      <c r="E31" s="70"/>
-      <c r="F31" s="70"/>
+      <c r="D31" s="68"/>
+      <c r="E31" s="68"/>
+      <c r="F31" s="68"/>
     </row>
     <row r="32" spans="1:18" x14ac:dyDescent="0.3">
-      <c r="B32" s="58"/>
-      <c r="C32" s="71"/>
-      <c r="D32" s="70"/>
-      <c r="E32" s="70"/>
-      <c r="F32" s="70"/>
+      <c r="B32" s="57"/>
+      <c r="C32" s="69"/>
+      <c r="D32" s="68"/>
+      <c r="E32" s="68"/>
+      <c r="F32" s="68"/>
     </row>
     <row r="33" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B33" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="C33" s="65" t="s">
+      <c r="C33" s="64" t="s">
         <v>89</v>
       </c>
-      <c r="D33" s="66"/>
-      <c r="E33" s="66"/>
-      <c r="F33" s="67"/>
+      <c r="D33" s="65"/>
+      <c r="E33" s="65"/>
+      <c r="F33" s="66"/>
     </row>
     <row r="34" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B34" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="C34" s="65" t="s">
+      <c r="C34" s="64" t="s">
         <v>90</v>
       </c>
-      <c r="D34" s="66"/>
-      <c r="E34" s="66"/>
-      <c r="F34" s="67"/>
+      <c r="D34" s="65"/>
+      <c r="E34" s="65"/>
+      <c r="F34" s="66"/>
     </row>
     <row r="35" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B35" s="12" t="s">
         <v>10</v>
       </c>
-      <c r="C35" s="65" t="s">
+      <c r="C35" s="64" t="s">
         <v>91</v>
       </c>
-      <c r="D35" s="66"/>
-      <c r="E35" s="66"/>
-      <c r="F35" s="67"/>
+      <c r="D35" s="65"/>
+      <c r="E35" s="65"/>
+      <c r="F35" s="66"/>
     </row>
     <row r="36" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B36" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="C36" s="65" t="s">
+      <c r="C36" s="64" t="s">
         <v>92</v>
       </c>
-      <c r="D36" s="66"/>
-      <c r="E36" s="66"/>
-      <c r="F36" s="67"/>
+      <c r="D36" s="65"/>
+      <c r="E36" s="65"/>
+      <c r="F36" s="66"/>
     </row>
     <row r="37" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B37" s="13" t="s">
         <v>93</v>
       </c>
-      <c r="C37" s="65" t="s">
+      <c r="C37" s="64" t="s">
         <v>94</v>
       </c>
-      <c r="D37" s="66"/>
-      <c r="E37" s="66"/>
-      <c r="F37" s="67"/>
+      <c r="D37" s="65"/>
+      <c r="E37" s="65"/>
+      <c r="F37" s="66"/>
     </row>
     <row r="38" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B38" s="12" t="s">
         <v>15</v>
       </c>
-      <c r="C38" s="65" t="s">
+      <c r="C38" s="64" t="s">
         <v>95</v>
       </c>
-      <c r="D38" s="66"/>
-      <c r="E38" s="66"/>
-      <c r="F38" s="67"/>
+      <c r="D38" s="65"/>
+      <c r="E38" s="65"/>
+      <c r="F38" s="66"/>
     </row>
   </sheetData>
   <mergeCells count="14">
+    <mergeCell ref="B12:B13"/>
+    <mergeCell ref="E12:E13"/>
+    <mergeCell ref="C34:F34"/>
+    <mergeCell ref="C12:C13"/>
+    <mergeCell ref="F12:F13"/>
+    <mergeCell ref="B31:B32"/>
     <mergeCell ref="G12:G13"/>
     <mergeCell ref="C38:F38"/>
     <mergeCell ref="C33:F33"/>
@@ -10627,12 +10673,6 @@
     <mergeCell ref="C37:F37"/>
     <mergeCell ref="C36:F36"/>
     <mergeCell ref="C35:F35"/>
-    <mergeCell ref="B12:B13"/>
-    <mergeCell ref="E12:E13"/>
-    <mergeCell ref="C34:F34"/>
-    <mergeCell ref="C12:C13"/>
-    <mergeCell ref="F12:F13"/>
-    <mergeCell ref="B31:B32"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
supplier sheet edited to have more feasible results
</commit_message>
<xml_diff>
--- a/Arya_Phones_Supplier_Selection.xlsx
+++ b/Arya_Phones_Supplier_Selection.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\LENOVO\Desktop\Asistan\Arya Phone\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DA322D21-0643-4B5A-A016-86D2005A72B5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8020EA01-E9B5-4B13-A759-906C1D96E5F3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Supplier" sheetId="1" r:id="rId1"/>
@@ -802,6 +802,24 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="14" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="164" fontId="0" fillId="14" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="1" fontId="0" fillId="14" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="5" fillId="15" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="15" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="15" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="16" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="1" fontId="0" fillId="16" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="5" fillId="14" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="14" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -823,32 +841,14 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="14" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="164" fontId="0" fillId="14" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
-    <xf numFmtId="1" fontId="0" fillId="14" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="5" fillId="15" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="15" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="15" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="16" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="1" fontId="0" fillId="16" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="5" fillId="14" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="14" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1046,9 +1046,9 @@
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="5" max="5" width="18.21875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="20" style="71" bestFit="1" customWidth="1"/>
-    <col min="7" max="8" width="8.88671875" style="77"/>
-    <col min="9" max="9" width="8.88671875" style="71"/>
+    <col min="6" max="6" width="20" style="56" bestFit="1" customWidth="1"/>
+    <col min="7" max="8" width="8.88671875" style="62"/>
+    <col min="9" max="9" width="8.88671875" style="56"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:11" x14ac:dyDescent="0.3">
@@ -1067,16 +1067,16 @@
       <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="71" t="s">
+      <c r="F1" s="56" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="77" t="s">
+      <c r="G1" s="62" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="77" t="s">
+      <c r="H1" s="62" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="71" t="s">
+      <c r="I1" s="56" t="s">
         <v>8</v>
       </c>
       <c r="J1" t="s">
@@ -1091,10 +1091,10 @@
         <v>10</v>
       </c>
       <c r="B2" s="55">
-        <v>2.4119999999999999</v>
+        <v>2.2120000000000002</v>
       </c>
       <c r="C2" s="55">
-        <v>4.3710000000000004</v>
+        <v>3.371</v>
       </c>
       <c r="D2" s="55">
         <v>2.4569999999999999</v>
@@ -1102,16 +1102,16 @@
       <c r="E2" s="55">
         <v>1.9430000000000001</v>
       </c>
-      <c r="F2" s="72">
-        <v>3</v>
-      </c>
-      <c r="G2" s="78">
-        <v>0</v>
-      </c>
-      <c r="H2" s="78">
-        <v>1</v>
-      </c>
-      <c r="I2" s="73">
+      <c r="F2" s="57">
+        <v>3</v>
+      </c>
+      <c r="G2" s="63">
+        <v>0</v>
+      </c>
+      <c r="H2" s="63">
+        <v>1</v>
+      </c>
+      <c r="I2" s="58">
         <v>1</v>
       </c>
       <c r="J2" s="55">
@@ -1126,10 +1126,10 @@
         <v>11</v>
       </c>
       <c r="B3" s="55">
-        <v>4.056</v>
+        <v>3.056</v>
       </c>
       <c r="C3" s="55">
-        <v>1.33</v>
+        <v>0.63</v>
       </c>
       <c r="D3" s="55">
         <v>4.8390000000000004</v>
@@ -1137,16 +1137,16 @@
       <c r="E3" s="55">
         <v>1.0640000000000001</v>
       </c>
-      <c r="F3" s="72">
-        <v>4</v>
-      </c>
-      <c r="G3" s="78">
-        <v>0</v>
-      </c>
-      <c r="H3" s="78">
-        <v>0</v>
-      </c>
-      <c r="I3" s="73">
+      <c r="F3" s="57">
+        <v>4</v>
+      </c>
+      <c r="G3" s="63">
+        <v>0</v>
+      </c>
+      <c r="H3" s="63">
+        <v>0</v>
+      </c>
+      <c r="I3" s="58">
         <v>0</v>
       </c>
       <c r="J3" s="55">
@@ -1161,27 +1161,27 @@
         <v>12</v>
       </c>
       <c r="B4" s="55">
-        <v>4.1349999999999998</v>
+        <v>2.2349999999999999</v>
       </c>
       <c r="C4" s="55">
         <v>4.3710000000000004</v>
       </c>
       <c r="D4" s="55">
-        <v>2.8980000000000001</v>
+        <v>2.3380000000000001</v>
       </c>
       <c r="E4" s="55">
         <v>2.4159999999999999</v>
       </c>
-      <c r="F4" s="72">
+      <c r="F4" s="57">
         <v>1.0980000000000001</v>
       </c>
-      <c r="G4" s="78">
-        <v>0</v>
-      </c>
-      <c r="H4" s="78">
-        <v>0</v>
-      </c>
-      <c r="I4" s="73">
+      <c r="G4" s="63">
+        <v>0</v>
+      </c>
+      <c r="H4" s="63">
+        <v>0</v>
+      </c>
+      <c r="I4" s="58">
         <v>0</v>
       </c>
       <c r="J4" s="55">
@@ -1196,7 +1196,7 @@
         <v>13</v>
       </c>
       <c r="B5" s="55">
-        <v>3.5910000000000002</v>
+        <v>1.7909999999999999</v>
       </c>
       <c r="C5" s="55">
         <v>1.629</v>
@@ -1207,16 +1207,16 @@
       <c r="E5" s="55">
         <v>1.01</v>
       </c>
-      <c r="F5" s="72">
+      <c r="F5" s="57">
         <v>2.823</v>
       </c>
-      <c r="G5" s="78">
-        <v>0</v>
-      </c>
-      <c r="H5" s="78">
-        <v>1</v>
-      </c>
-      <c r="I5" s="73">
+      <c r="G5" s="63">
+        <v>0</v>
+      </c>
+      <c r="H5" s="63">
+        <v>1</v>
+      </c>
+      <c r="I5" s="58">
         <v>0</v>
       </c>
       <c r="J5" s="55">
@@ -1234,7 +1234,7 @@
         <v>1.7050000000000001</v>
       </c>
       <c r="C6" s="55">
-        <v>4.3710000000000004</v>
+        <v>3.371</v>
       </c>
       <c r="D6" s="55">
         <v>2.9670000000000001</v>
@@ -1242,16 +1242,16 @@
       <c r="E6" s="55">
         <v>2.0790000000000002</v>
       </c>
-      <c r="F6" s="72">
+      <c r="F6" s="57">
         <v>5</v>
       </c>
-      <c r="G6" s="78">
-        <v>0</v>
-      </c>
-      <c r="H6" s="78">
-        <v>1</v>
-      </c>
-      <c r="I6" s="73">
+      <c r="G6" s="63">
+        <v>0</v>
+      </c>
+      <c r="H6" s="63">
+        <v>1</v>
+      </c>
+      <c r="I6" s="58">
         <v>1</v>
       </c>
       <c r="J6" s="55">
@@ -1277,16 +1277,16 @@
       <c r="E7" s="55">
         <v>1.9950000000000001</v>
       </c>
-      <c r="F7" s="72">
+      <c r="F7" s="57">
         <v>3.234</v>
       </c>
-      <c r="G7" s="78">
-        <v>1</v>
-      </c>
-      <c r="H7" s="78">
-        <v>0</v>
-      </c>
-      <c r="I7" s="73">
+      <c r="G7" s="63">
+        <v>1</v>
+      </c>
+      <c r="H7" s="63">
+        <v>0</v>
+      </c>
+      <c r="I7" s="58">
         <v>0</v>
       </c>
       <c r="J7" s="55">
@@ -1312,16 +1312,16 @@
       <c r="E8" s="55">
         <v>1.796</v>
       </c>
-      <c r="F8" s="72">
+      <c r="F8" s="57">
         <v>4.7770000000000001</v>
       </c>
-      <c r="G8" s="78">
-        <v>0</v>
-      </c>
-      <c r="H8" s="78">
-        <v>1</v>
-      </c>
-      <c r="I8" s="73">
+      <c r="G8" s="63">
+        <v>0</v>
+      </c>
+      <c r="H8" s="63">
+        <v>1</v>
+      </c>
+      <c r="I8" s="58">
         <v>0</v>
       </c>
       <c r="J8" s="55">
@@ -1347,16 +1347,16 @@
       <c r="E9" s="55">
         <v>2.516</v>
       </c>
-      <c r="F9" s="72">
+      <c r="F9" s="57">
         <v>3.234</v>
       </c>
-      <c r="G9" s="78">
-        <v>1</v>
-      </c>
-      <c r="H9" s="78">
-        <v>0</v>
-      </c>
-      <c r="I9" s="73">
+      <c r="G9" s="63">
+        <v>1</v>
+      </c>
+      <c r="H9" s="63">
+        <v>0</v>
+      </c>
+      <c r="I9" s="58">
         <v>0</v>
       </c>
       <c r="J9" s="55">
@@ -1382,16 +1382,16 @@
       <c r="E10" s="55">
         <v>2.323</v>
       </c>
-      <c r="F10" s="72">
+      <c r="F10" s="57">
         <v>4.0999999999999996</v>
       </c>
-      <c r="G10" s="78">
-        <v>0</v>
-      </c>
-      <c r="H10" s="78">
-        <v>0</v>
-      </c>
-      <c r="I10" s="73">
+      <c r="G10" s="63">
+        <v>0</v>
+      </c>
+      <c r="H10" s="63">
+        <v>0</v>
+      </c>
+      <c r="I10" s="58">
         <v>0</v>
       </c>
       <c r="J10" s="55">
@@ -1406,10 +1406,10 @@
         <v>19</v>
       </c>
       <c r="B11" s="55">
-        <v>4.056</v>
+        <v>3.556</v>
       </c>
       <c r="C11" s="55">
-        <v>1.218</v>
+        <v>1.008</v>
       </c>
       <c r="D11" s="55">
         <v>2.6219999999999999</v>
@@ -1417,16 +1417,16 @@
       <c r="E11" s="55">
         <v>4.6269999999999998</v>
       </c>
-      <c r="F11" s="72">
+      <c r="F11" s="57">
         <v>3.21</v>
       </c>
-      <c r="G11" s="78">
-        <v>1</v>
-      </c>
-      <c r="H11" s="78">
-        <v>1</v>
-      </c>
-      <c r="I11" s="73">
+      <c r="G11" s="63">
+        <v>1</v>
+      </c>
+      <c r="H11" s="63">
+        <v>1</v>
+      </c>
+      <c r="I11" s="58">
         <v>0</v>
       </c>
       <c r="J11" s="55">
@@ -1444,7 +1444,7 @@
         <v>4.056</v>
       </c>
       <c r="C12" s="55">
-        <v>3.589</v>
+        <v>2.589</v>
       </c>
       <c r="D12" s="55">
         <v>2.3079999999999998</v>
@@ -1452,16 +1452,16 @@
       <c r="E12" s="55">
         <v>1.861</v>
       </c>
-      <c r="F12" s="72">
+      <c r="F12" s="57">
         <v>1.19</v>
       </c>
-      <c r="G12" s="78">
-        <v>1</v>
-      </c>
-      <c r="H12" s="78">
-        <v>1</v>
-      </c>
-      <c r="I12" s="73">
+      <c r="G12" s="63">
+        <v>1</v>
+      </c>
+      <c r="H12" s="63">
+        <v>1</v>
+      </c>
+      <c r="I12" s="58">
         <v>1</v>
       </c>
       <c r="J12" s="55">
@@ -1487,16 +1487,16 @@
       <c r="E13" s="55">
         <v>3.0529999999999999</v>
       </c>
-      <c r="F13" s="72">
+      <c r="F13" s="57">
         <v>1.234</v>
       </c>
-      <c r="G13" s="78">
-        <v>0</v>
-      </c>
-      <c r="H13" s="78">
-        <v>1</v>
-      </c>
-      <c r="I13" s="73">
+      <c r="G13" s="63">
+        <v>0</v>
+      </c>
+      <c r="H13" s="63">
+        <v>1</v>
+      </c>
+      <c r="I13" s="58">
         <v>1</v>
       </c>
       <c r="J13" s="55">
@@ -1522,16 +1522,16 @@
       <c r="E14" s="55">
         <v>1.657</v>
       </c>
-      <c r="F14" s="72">
+      <c r="F14" s="57">
         <v>4.12</v>
       </c>
-      <c r="G14" s="78">
-        <v>0</v>
-      </c>
-      <c r="H14" s="78">
-        <v>0</v>
-      </c>
-      <c r="I14" s="73">
+      <c r="G14" s="63">
+        <v>0</v>
+      </c>
+      <c r="H14" s="63">
+        <v>0</v>
+      </c>
+      <c r="I14" s="58">
         <v>1</v>
       </c>
       <c r="J14" s="55">
@@ -1546,7 +1546,7 @@
         <v>23</v>
       </c>
       <c r="B15" s="55">
-        <v>3.5779999999999998</v>
+        <v>1.5780000000000001</v>
       </c>
       <c r="C15" s="55">
         <v>1.006</v>
@@ -1557,16 +1557,16 @@
       <c r="E15" s="55">
         <v>1.3029999999999999</v>
       </c>
-      <c r="F15" s="72">
-        <v>2</v>
-      </c>
-      <c r="G15" s="78">
-        <v>1</v>
-      </c>
-      <c r="H15" s="78">
-        <v>0</v>
-      </c>
-      <c r="I15" s="73">
+      <c r="F15" s="57">
+        <v>2</v>
+      </c>
+      <c r="G15" s="63">
+        <v>1</v>
+      </c>
+      <c r="H15" s="63">
+        <v>0</v>
+      </c>
+      <c r="I15" s="58">
         <v>0</v>
       </c>
       <c r="J15" s="55">
@@ -1592,16 +1592,16 @@
       <c r="E16" s="55">
         <v>1.405</v>
       </c>
-      <c r="F16" s="72">
+      <c r="F16" s="57">
         <v>4.4000000000000004</v>
       </c>
-      <c r="G16" s="78">
-        <v>1</v>
-      </c>
-      <c r="H16" s="78">
-        <v>0</v>
-      </c>
-      <c r="I16" s="73">
+      <c r="G16" s="63">
+        <v>1</v>
+      </c>
+      <c r="H16" s="63">
+        <v>0</v>
+      </c>
+      <c r="I16" s="58">
         <v>0</v>
       </c>
       <c r="J16" s="55">
@@ -1627,16 +1627,16 @@
       <c r="E17" s="55">
         <v>3.6720000000000002</v>
       </c>
-      <c r="F17" s="72">
-        <v>2</v>
-      </c>
-      <c r="G17" s="78">
-        <v>0</v>
-      </c>
-      <c r="H17" s="78">
-        <v>0</v>
-      </c>
-      <c r="I17" s="73">
+      <c r="F17" s="57">
+        <v>2</v>
+      </c>
+      <c r="G17" s="63">
+        <v>0</v>
+      </c>
+      <c r="H17" s="63">
+        <v>0</v>
+      </c>
+      <c r="I17" s="58">
         <v>1</v>
       </c>
       <c r="J17" s="55">
@@ -1662,16 +1662,16 @@
       <c r="E18" s="55">
         <v>1.806</v>
       </c>
-      <c r="F18" s="72">
+      <c r="F18" s="57">
         <v>2.234</v>
       </c>
-      <c r="G18" s="78">
-        <v>1</v>
-      </c>
-      <c r="H18" s="78">
-        <v>0</v>
-      </c>
-      <c r="I18" s="73">
+      <c r="G18" s="63">
+        <v>1</v>
+      </c>
+      <c r="H18" s="63">
+        <v>0</v>
+      </c>
+      <c r="I18" s="58">
         <v>1</v>
       </c>
       <c r="J18" s="55">
@@ -1686,7 +1686,7 @@
         <v>27</v>
       </c>
       <c r="B19" s="55">
-        <v>4.8540000000000001</v>
+        <v>3.9540000000000002</v>
       </c>
       <c r="C19" s="55">
         <v>2.3E-2</v>
@@ -1697,16 +1697,16 @@
       <c r="E19" s="55">
         <v>3.8740000000000001</v>
       </c>
-      <c r="F19" s="72">
+      <c r="F19" s="57">
         <v>0.23400000000000001</v>
       </c>
-      <c r="G19" s="78">
-        <v>1</v>
-      </c>
-      <c r="H19" s="78">
-        <v>0</v>
-      </c>
-      <c r="I19" s="73">
+      <c r="G19" s="63">
+        <v>1</v>
+      </c>
+      <c r="H19" s="63">
+        <v>0</v>
+      </c>
+      <c r="I19" s="58">
         <v>0</v>
       </c>
       <c r="J19" s="55">
@@ -1726,8 +1726,8 @@
   <dimension ref="A1:H21"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="4" max="4" width="8.88671875" style="76"/>
-    <col min="5" max="6" width="8.88671875" style="71"/>
+    <col min="4" max="4" width="8.88671875" style="61"/>
+    <col min="5" max="6" width="8.88671875" style="56"/>
     <col min="8" max="8" width="39.6640625" customWidth="1"/>
   </cols>
   <sheetData>
@@ -1741,13 +1741,13 @@
       <c r="C1" s="15" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="74" t="s">
+      <c r="D1" s="59" t="s">
         <v>96</v>
       </c>
-      <c r="E1" s="79" t="s">
-        <v>4</v>
-      </c>
-      <c r="F1" s="79" t="s">
+      <c r="E1" s="64" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="64" t="s">
         <v>5</v>
       </c>
       <c r="G1" s="17" t="s">
@@ -1767,13 +1767,13 @@
       <c r="C2" s="53">
         <v>5.4450791916772837E-2</v>
       </c>
-      <c r="D2" s="75">
+      <c r="D2" s="60">
         <v>0.61191053879833257</v>
       </c>
-      <c r="E2" s="80">
+      <c r="E2" s="65">
         <v>0.106720019477238</v>
       </c>
-      <c r="F2" s="80">
+      <c r="F2" s="65">
         <v>0.152651963522863</v>
       </c>
       <c r="G2" s="54">
@@ -1793,13 +1793,13 @@
       <c r="C3" s="53">
         <v>9.1150810219638279E-2</v>
       </c>
-      <c r="D3" s="75">
+      <c r="D3" s="60">
         <v>0.61026173707464948</v>
       </c>
-      <c r="E3" s="80">
+      <c r="E3" s="65">
         <v>0.18945464506061421</v>
       </c>
-      <c r="F3" s="80">
+      <c r="F3" s="65">
         <v>0.10155365833498819</v>
       </c>
       <c r="G3" s="54">
@@ -1819,13 +1819,13 @@
       <c r="C4" s="53">
         <v>0.25457641457483893</v>
       </c>
-      <c r="D4" s="75">
+      <c r="D4" s="60">
         <v>0.60726173707464903</v>
       </c>
-      <c r="E4" s="80">
+      <c r="E4" s="65">
         <v>0.24824483374410089</v>
       </c>
-      <c r="F4" s="80">
+      <c r="F4" s="65">
         <v>0.2881274398577503</v>
       </c>
       <c r="G4" s="54">
@@ -1845,13 +1845,13 @@
       <c r="C5" s="53">
         <v>6.516607737331874E-2</v>
       </c>
-      <c r="D5" s="75">
+      <c r="D5" s="60">
         <v>0.58371425606695315</v>
       </c>
-      <c r="E5" s="80">
+      <c r="E5" s="65">
         <v>0.28577314002182541</v>
       </c>
-      <c r="F5" s="80">
+      <c r="F5" s="65">
         <v>0.16710661185701839</v>
       </c>
       <c r="G5" s="54">
@@ -1871,13 +1871,13 @@
       <c r="C6" s="53">
         <v>0.16109848730107321</v>
       </c>
-      <c r="D6" s="75">
+      <c r="D6" s="60">
         <v>0.54893726307541901</v>
       </c>
-      <c r="E6" s="80">
+      <c r="E6" s="65">
         <v>0.17008933186008149</v>
       </c>
-      <c r="F6" s="80">
+      <c r="F6" s="65">
         <v>0.27528967563063772</v>
       </c>
       <c r="G6" s="54">
@@ -1897,13 +1897,13 @@
       <c r="C7" s="53">
         <v>0.26040571421757103</v>
       </c>
-      <c r="D7" s="75">
+      <c r="D7" s="60">
         <v>0.53524476184674197</v>
       </c>
-      <c r="E7" s="80">
+      <c r="E7" s="65">
         <v>0.1067200194772385</v>
       </c>
-      <c r="F7" s="80">
+      <c r="F7" s="65">
         <v>0.10155365833498819</v>
       </c>
       <c r="G7" s="54">
@@ -1923,13 +1923,13 @@
       <c r="C8" s="53">
         <v>0.12208818407051721</v>
       </c>
-      <c r="D8" s="75">
+      <c r="D8" s="60">
         <v>0.50118862071605097</v>
       </c>
-      <c r="E8" s="80">
+      <c r="E8" s="65">
         <v>0.32446059664501697</v>
       </c>
-      <c r="F8" s="80">
+      <c r="F8" s="65">
         <v>0.10155365833498819</v>
       </c>
       <c r="G8" s="54">
@@ -1949,13 +1949,13 @@
       <c r="C9" s="53">
         <v>0.26693912830951111</v>
       </c>
-      <c r="D9" s="75">
+      <c r="D9" s="60">
         <v>0.47418990241855702</v>
       </c>
-      <c r="E9" s="80">
+      <c r="E9" s="65">
         <v>0.1067200194772385</v>
       </c>
-      <c r="F9" s="80">
+      <c r="F9" s="65">
         <v>0.10155365833498819</v>
       </c>
       <c r="G9" s="54">
@@ -1975,13 +1975,13 @@
       <c r="C10" s="53">
         <v>0.15483029452809721</v>
       </c>
-      <c r="D10" s="75">
+      <c r="D10" s="60">
         <v>0.43507948585385298</v>
       </c>
-      <c r="E10" s="80">
+      <c r="E10" s="65">
         <v>0.16962970966432209</v>
       </c>
-      <c r="F10" s="80">
+      <c r="F10" s="65">
         <v>0.10155365833498819</v>
       </c>
       <c r="G10" s="54">
@@ -2001,13 +2001,13 @@
       <c r="C11" s="53">
         <v>6.6813196513184861E-2</v>
       </c>
-      <c r="D11" s="75">
+      <c r="D11" s="60">
         <v>0.399950545031311</v>
       </c>
-      <c r="E11" s="80">
+      <c r="E11" s="65">
         <v>0.12896323351417149</v>
       </c>
-      <c r="F11" s="80">
+      <c r="F11" s="65">
         <v>0.12518162852531989</v>
       </c>
       <c r="G11" s="54">
@@ -2027,13 +2027,13 @@
       <c r="C12" s="53">
         <v>0.16985306196136299</v>
       </c>
-      <c r="D12" s="75">
+      <c r="D12" s="60">
         <v>0.388563554257354</v>
       </c>
-      <c r="E12" s="80">
+      <c r="E12" s="65">
         <v>0.24861374555913729</v>
       </c>
-      <c r="F12" s="80">
+      <c r="F12" s="65">
         <v>0.25064404411660468</v>
       </c>
       <c r="G12" s="54">
@@ -2053,13 +2053,13 @@
       <c r="C13" s="53">
         <v>0.19024045650357649</v>
       </c>
-      <c r="D13" s="75">
+      <c r="D13" s="60">
         <v>0.34034996285317798</v>
       </c>
-      <c r="E13" s="80">
+      <c r="E13" s="65">
         <v>0.27804323994842262</v>
       </c>
-      <c r="F13" s="80">
+      <c r="F13" s="65">
         <v>0.119152078029859</v>
       </c>
       <c r="G13" s="54">
@@ -2079,13 +2079,13 @@
       <c r="C14" s="53">
         <v>0.25457641457483893</v>
       </c>
-      <c r="D14" s="75">
+      <c r="D14" s="60">
         <v>0.28126564060459602</v>
       </c>
-      <c r="E14" s="80">
+      <c r="E14" s="65">
         <v>0.24206895072120549</v>
       </c>
-      <c r="F14" s="80">
+      <c r="F14" s="65">
         <v>0.10155365833498819</v>
       </c>
       <c r="G14" s="54">
@@ -2105,13 +2105,13 @@
       <c r="C15" s="53">
         <v>7.3418276193979989E-2</v>
       </c>
-      <c r="D15" s="75">
+      <c r="D15" s="60">
         <v>0.24790607253205099</v>
       </c>
-      <c r="E15" s="80">
+      <c r="E15" s="65">
         <v>0.29100442200694832</v>
       </c>
-      <c r="F15" s="80">
+      <c r="F15" s="65">
         <v>0.108246470664996</v>
       </c>
       <c r="G15" s="54">
@@ -2131,13 +2131,13 @@
       <c r="C16" s="53">
         <v>9.6546504644227593E-2</v>
       </c>
-      <c r="D16" s="75">
+      <c r="D16" s="60">
         <v>0.21705211340986499</v>
       </c>
-      <c r="E16" s="80">
+      <c r="E16" s="65">
         <v>0.1067200194772385</v>
       </c>
-      <c r="F16" s="80">
+      <c r="F16" s="65">
         <v>0.10155365833498819</v>
       </c>
       <c r="G16" s="54">
@@ -2157,13 +2157,13 @@
       <c r="C17" s="53">
         <v>0.243834865733492</v>
       </c>
-      <c r="D17" s="75">
+      <c r="D17" s="60">
         <v>0.19145012390986499</v>
       </c>
-      <c r="E17" s="80">
+      <c r="E17" s="65">
         <v>0.183331251224816</v>
       </c>
-      <c r="F17" s="80">
+      <c r="F17" s="65">
         <v>0.20155365833498801</v>
       </c>
       <c r="G17" s="54">
@@ -2183,13 +2183,13 @@
       <c r="C18" s="53">
         <v>0.10691631099167261</v>
       </c>
-      <c r="D18" s="75">
+      <c r="D18" s="60">
         <v>0.17137146890986499</v>
       </c>
-      <c r="E18" s="80">
+      <c r="E18" s="65">
         <v>0.29128321359242249</v>
       </c>
-      <c r="F18" s="80">
+      <c r="F18" s="65">
         <v>0.23155365833498801</v>
       </c>
       <c r="G18" s="54">
@@ -2209,13 +2209,13 @@
       <c r="C19" s="53">
         <v>7.3418276193979989E-2</v>
       </c>
-      <c r="D19" s="75">
+      <c r="D19" s="60">
         <v>0.13737146890986501</v>
       </c>
-      <c r="E19" s="80">
+      <c r="E19" s="65">
         <v>0.31938813314298031</v>
       </c>
-      <c r="F19" s="80">
+      <c r="F19" s="65">
         <v>0.10155365833498819</v>
       </c>
       <c r="G19" s="54">
@@ -2235,13 +2235,13 @@
       <c r="C20" s="53">
         <v>0.27341827619398001</v>
       </c>
-      <c r="D20" s="75">
+      <c r="D20" s="60">
         <v>0.117371468909865</v>
       </c>
-      <c r="E20" s="80">
+      <c r="E20" s="65">
         <v>0.102500150077396</v>
       </c>
-      <c r="F20" s="80">
+      <c r="F20" s="65">
         <v>0.1127673895923734</v>
       </c>
       <c r="G20" s="54">
@@ -2261,13 +2261,13 @@
       <c r="C21" s="53">
         <v>0.2048960971299689</v>
       </c>
-      <c r="D21" s="75">
+      <c r="D21" s="60">
         <v>9.7371468909865005E-2</v>
       </c>
-      <c r="E21" s="80">
+      <c r="E21" s="65">
         <v>0.15672001947723799</v>
       </c>
-      <c r="F21" s="80">
+      <c r="F21" s="65">
         <v>0.10155365833498819</v>
       </c>
       <c r="G21" s="54">
@@ -2834,22 +2834,22 @@
       </c>
     </row>
     <row r="12" spans="2:24" x14ac:dyDescent="0.3">
-      <c r="B12" s="56" t="s">
+      <c r="B12" s="66" t="s">
         <v>54</v>
       </c>
-      <c r="C12" s="60" t="s">
-        <v>1</v>
-      </c>
-      <c r="D12" s="58" t="s">
-        <v>2</v>
-      </c>
-      <c r="E12" s="58" t="s">
-        <v>3</v>
-      </c>
-      <c r="F12" s="58" t="s">
-        <v>4</v>
-      </c>
-      <c r="G12" s="62" t="s">
+      <c r="C12" s="70" t="s">
+        <v>1</v>
+      </c>
+      <c r="D12" s="68" t="s">
+        <v>2</v>
+      </c>
+      <c r="E12" s="68" t="s">
+        <v>3</v>
+      </c>
+      <c r="F12" s="68" t="s">
+        <v>4</v>
+      </c>
+      <c r="G12" s="72" t="s">
         <v>5</v>
       </c>
       <c r="J12" s="19" t="s">
@@ -2863,12 +2863,12 @@
       </c>
     </row>
     <row r="13" spans="2:24" ht="34.950000000000003" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B13" s="57"/>
-      <c r="C13" s="61"/>
-      <c r="D13" s="59"/>
-      <c r="E13" s="59"/>
-      <c r="F13" s="59"/>
-      <c r="G13" s="63"/>
+      <c r="B13" s="67"/>
+      <c r="C13" s="71"/>
+      <c r="D13" s="69"/>
+      <c r="E13" s="69"/>
+      <c r="F13" s="69"/>
+      <c r="G13" s="73"/>
       <c r="J13" s="19" t="s">
         <v>58</v>
       </c>
@@ -5136,22 +5136,22 @@
       </c>
     </row>
     <row r="12" spans="2:26" x14ac:dyDescent="0.3">
-      <c r="B12" s="56" t="s">
+      <c r="B12" s="66" t="s">
         <v>54</v>
       </c>
-      <c r="C12" s="60" t="s">
-        <v>1</v>
-      </c>
-      <c r="D12" s="58" t="s">
-        <v>2</v>
-      </c>
-      <c r="E12" s="58" t="s">
-        <v>3</v>
-      </c>
-      <c r="F12" s="58" t="s">
-        <v>4</v>
-      </c>
-      <c r="G12" s="62" t="s">
+      <c r="C12" s="70" t="s">
+        <v>1</v>
+      </c>
+      <c r="D12" s="68" t="s">
+        <v>2</v>
+      </c>
+      <c r="E12" s="68" t="s">
+        <v>3</v>
+      </c>
+      <c r="F12" s="68" t="s">
+        <v>4</v>
+      </c>
+      <c r="G12" s="72" t="s">
         <v>5</v>
       </c>
       <c r="J12" s="19" t="s">
@@ -5171,12 +5171,12 @@
       </c>
     </row>
     <row r="13" spans="2:26" ht="34.950000000000003" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B13" s="57"/>
-      <c r="C13" s="61"/>
-      <c r="D13" s="59"/>
-      <c r="E13" s="59"/>
-      <c r="F13" s="59"/>
-      <c r="G13" s="63"/>
+      <c r="B13" s="67"/>
+      <c r="C13" s="71"/>
+      <c r="D13" s="69"/>
+      <c r="E13" s="69"/>
+      <c r="F13" s="69"/>
+      <c r="G13" s="73"/>
       <c r="J13" s="19" t="s">
         <v>58</v>
       </c>
@@ -7285,22 +7285,22 @@
       </c>
     </row>
     <row r="12" spans="2:24" x14ac:dyDescent="0.3">
-      <c r="B12" s="56" t="s">
+      <c r="B12" s="66" t="s">
         <v>54</v>
       </c>
-      <c r="C12" s="60" t="s">
-        <v>1</v>
-      </c>
-      <c r="D12" s="58" t="s">
-        <v>2</v>
-      </c>
-      <c r="E12" s="58" t="s">
-        <v>3</v>
-      </c>
-      <c r="F12" s="58" t="s">
-        <v>4</v>
-      </c>
-      <c r="G12" s="62" t="s">
+      <c r="C12" s="70" t="s">
+        <v>1</v>
+      </c>
+      <c r="D12" s="68" t="s">
+        <v>2</v>
+      </c>
+      <c r="E12" s="68" t="s">
+        <v>3</v>
+      </c>
+      <c r="F12" s="68" t="s">
+        <v>4</v>
+      </c>
+      <c r="G12" s="72" t="s">
         <v>5</v>
       </c>
       <c r="J12" s="19" t="s">
@@ -7314,12 +7314,12 @@
       </c>
     </row>
     <row r="13" spans="2:24" ht="34.950000000000003" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B13" s="57"/>
-      <c r="C13" s="61"/>
-      <c r="D13" s="59"/>
-      <c r="E13" s="59"/>
-      <c r="F13" s="59"/>
-      <c r="G13" s="63"/>
+      <c r="B13" s="67"/>
+      <c r="C13" s="71"/>
+      <c r="D13" s="69"/>
+      <c r="E13" s="69"/>
+      <c r="F13" s="69"/>
+      <c r="G13" s="73"/>
       <c r="J13" s="19" t="s">
         <v>58</v>
       </c>
@@ -8872,22 +8872,22 @@
       </c>
     </row>
     <row r="12" spans="2:24" x14ac:dyDescent="0.3">
-      <c r="B12" s="56" t="s">
+      <c r="B12" s="66" t="s">
         <v>54</v>
       </c>
-      <c r="C12" s="60" t="s">
-        <v>1</v>
-      </c>
-      <c r="D12" s="58" t="s">
-        <v>2</v>
-      </c>
-      <c r="E12" s="58" t="s">
-        <v>3</v>
-      </c>
-      <c r="F12" s="58" t="s">
-        <v>4</v>
-      </c>
-      <c r="G12" s="62" t="s">
+      <c r="C12" s="70" t="s">
+        <v>1</v>
+      </c>
+      <c r="D12" s="68" t="s">
+        <v>2</v>
+      </c>
+      <c r="E12" s="68" t="s">
+        <v>3</v>
+      </c>
+      <c r="F12" s="68" t="s">
+        <v>4</v>
+      </c>
+      <c r="G12" s="72" t="s">
         <v>5</v>
       </c>
       <c r="J12" s="19" t="s">
@@ -8901,12 +8901,12 @@
       </c>
     </row>
     <row r="13" spans="2:24" ht="34.950000000000003" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B13" s="57"/>
-      <c r="C13" s="61"/>
-      <c r="D13" s="59"/>
-      <c r="E13" s="59"/>
-      <c r="F13" s="59"/>
-      <c r="G13" s="63"/>
+      <c r="B13" s="67"/>
+      <c r="C13" s="71"/>
+      <c r="D13" s="69"/>
+      <c r="E13" s="69"/>
+      <c r="F13" s="69"/>
+      <c r="G13" s="73"/>
       <c r="J13" s="19" t="s">
         <v>58</v>
       </c>
@@ -10287,22 +10287,22 @@
       </c>
     </row>
     <row r="12" spans="2:18" x14ac:dyDescent="0.3">
-      <c r="B12" s="56" t="s">
+      <c r="B12" s="66" t="s">
         <v>54</v>
       </c>
-      <c r="C12" s="60" t="s">
-        <v>1</v>
-      </c>
-      <c r="D12" s="58" t="s">
-        <v>2</v>
-      </c>
-      <c r="E12" s="58" t="s">
-        <v>3</v>
-      </c>
-      <c r="F12" s="58" t="s">
-        <v>4</v>
-      </c>
-      <c r="G12" s="62" t="s">
+      <c r="C12" s="70" t="s">
+        <v>1</v>
+      </c>
+      <c r="D12" s="68" t="s">
+        <v>2</v>
+      </c>
+      <c r="E12" s="68" t="s">
+        <v>3</v>
+      </c>
+      <c r="F12" s="68" t="s">
+        <v>4</v>
+      </c>
+      <c r="G12" s="72" t="s">
         <v>5</v>
       </c>
       <c r="J12" s="19" t="s">
@@ -10316,12 +10316,12 @@
       </c>
     </row>
     <row r="13" spans="2:18" ht="34.950000000000003" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B13" s="57"/>
-      <c r="C13" s="61"/>
-      <c r="D13" s="59"/>
-      <c r="E13" s="59"/>
-      <c r="F13" s="59"/>
-      <c r="G13" s="63"/>
+      <c r="B13" s="67"/>
+      <c r="C13" s="71"/>
+      <c r="D13" s="69"/>
+      <c r="E13" s="69"/>
+      <c r="F13" s="69"/>
+      <c r="G13" s="73"/>
       <c r="J13" s="19" t="s">
         <v>58</v>
       </c>
@@ -10574,97 +10574,91 @@
       </c>
     </row>
     <row r="31" spans="1:18" x14ac:dyDescent="0.3">
-      <c r="B31" s="70" t="s">
-        <v>0</v>
-      </c>
-      <c r="C31" s="67" t="s">
+      <c r="B31" s="77" t="s">
+        <v>0</v>
+      </c>
+      <c r="C31" s="78" t="s">
         <v>88</v>
       </c>
-      <c r="D31" s="68"/>
-      <c r="E31" s="68"/>
-      <c r="F31" s="68"/>
+      <c r="D31" s="79"/>
+      <c r="E31" s="79"/>
+      <c r="F31" s="79"/>
     </row>
     <row r="32" spans="1:18" x14ac:dyDescent="0.3">
-      <c r="B32" s="57"/>
-      <c r="C32" s="69"/>
-      <c r="D32" s="68"/>
-      <c r="E32" s="68"/>
-      <c r="F32" s="68"/>
+      <c r="B32" s="67"/>
+      <c r="C32" s="80"/>
+      <c r="D32" s="79"/>
+      <c r="E32" s="79"/>
+      <c r="F32" s="79"/>
     </row>
     <row r="33" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B33" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="C33" s="64" t="s">
+      <c r="C33" s="74" t="s">
         <v>89</v>
       </c>
-      <c r="D33" s="65"/>
-      <c r="E33" s="65"/>
-      <c r="F33" s="66"/>
+      <c r="D33" s="75"/>
+      <c r="E33" s="75"/>
+      <c r="F33" s="76"/>
     </row>
     <row r="34" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B34" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="C34" s="64" t="s">
+      <c r="C34" s="74" t="s">
         <v>90</v>
       </c>
-      <c r="D34" s="65"/>
-      <c r="E34" s="65"/>
-      <c r="F34" s="66"/>
+      <c r="D34" s="75"/>
+      <c r="E34" s="75"/>
+      <c r="F34" s="76"/>
     </row>
     <row r="35" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B35" s="12" t="s">
         <v>10</v>
       </c>
-      <c r="C35" s="64" t="s">
+      <c r="C35" s="74" t="s">
         <v>91</v>
       </c>
-      <c r="D35" s="65"/>
-      <c r="E35" s="65"/>
-      <c r="F35" s="66"/>
+      <c r="D35" s="75"/>
+      <c r="E35" s="75"/>
+      <c r="F35" s="76"/>
     </row>
     <row r="36" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B36" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="C36" s="64" t="s">
+      <c r="C36" s="74" t="s">
         <v>92</v>
       </c>
-      <c r="D36" s="65"/>
-      <c r="E36" s="65"/>
-      <c r="F36" s="66"/>
+      <c r="D36" s="75"/>
+      <c r="E36" s="75"/>
+      <c r="F36" s="76"/>
     </row>
     <row r="37" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B37" s="13" t="s">
         <v>93</v>
       </c>
-      <c r="C37" s="64" t="s">
+      <c r="C37" s="74" t="s">
         <v>94</v>
       </c>
-      <c r="D37" s="65"/>
-      <c r="E37" s="65"/>
-      <c r="F37" s="66"/>
+      <c r="D37" s="75"/>
+      <c r="E37" s="75"/>
+      <c r="F37" s="76"/>
     </row>
     <row r="38" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B38" s="12" t="s">
         <v>15</v>
       </c>
-      <c r="C38" s="64" t="s">
+      <c r="C38" s="74" t="s">
         <v>95</v>
       </c>
-      <c r="D38" s="65"/>
-      <c r="E38" s="65"/>
-      <c r="F38" s="66"/>
+      <c r="D38" s="75"/>
+      <c r="E38" s="75"/>
+      <c r="F38" s="76"/>
     </row>
   </sheetData>
   <mergeCells count="14">
-    <mergeCell ref="B12:B13"/>
-    <mergeCell ref="E12:E13"/>
-    <mergeCell ref="C34:F34"/>
-    <mergeCell ref="C12:C13"/>
-    <mergeCell ref="F12:F13"/>
-    <mergeCell ref="B31:B32"/>
     <mergeCell ref="G12:G13"/>
     <mergeCell ref="C38:F38"/>
     <mergeCell ref="C33:F33"/>
@@ -10673,6 +10667,12 @@
     <mergeCell ref="C37:F37"/>
     <mergeCell ref="C36:F36"/>
     <mergeCell ref="C35:F35"/>
+    <mergeCell ref="B12:B13"/>
+    <mergeCell ref="E12:E13"/>
+    <mergeCell ref="C34:F34"/>
+    <mergeCell ref="C12:C13"/>
+    <mergeCell ref="F12:F13"/>
+    <mergeCell ref="B31:B32"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Buyer utility added. comparative simulations added
</commit_message>
<xml_diff>
--- a/Arya_Phones_Supplier_Selection.xlsx
+++ b/Arya_Phones_Supplier_Selection.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\LENOVO\Desktop\Asistan\Arya Phone\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8020EA01-E9B5-4B13-A759-906C1D96E5F3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{257C911A-5CEF-4D91-B0C5-CA0BA03CBE22}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Supplier" sheetId="1" r:id="rId1"/>
@@ -841,14 +841,14 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1765,7 +1765,7 @@
         <v>0.18141826864259999</v>
       </c>
       <c r="C2" s="53">
-        <v>5.4450791916772837E-2</v>
+        <v>0.254450791916772</v>
       </c>
       <c r="D2" s="60">
         <v>0.61191053879833257</v>
@@ -1791,7 +1791,7 @@
         <v>0.29731528292090348</v>
       </c>
       <c r="C3" s="53">
-        <v>9.1150810219638279E-2</v>
+        <v>0.29115081021963801</v>
       </c>
       <c r="D3" s="60">
         <v>0.61026173707464948</v>
@@ -10574,22 +10574,22 @@
       </c>
     </row>
     <row r="31" spans="1:18" x14ac:dyDescent="0.3">
-      <c r="B31" s="77" t="s">
-        <v>0</v>
-      </c>
-      <c r="C31" s="78" t="s">
+      <c r="B31" s="80" t="s">
+        <v>0</v>
+      </c>
+      <c r="C31" s="77" t="s">
         <v>88</v>
       </c>
-      <c r="D31" s="79"/>
-      <c r="E31" s="79"/>
-      <c r="F31" s="79"/>
+      <c r="D31" s="78"/>
+      <c r="E31" s="78"/>
+      <c r="F31" s="78"/>
     </row>
     <row r="32" spans="1:18" x14ac:dyDescent="0.3">
       <c r="B32" s="67"/>
-      <c r="C32" s="80"/>
-      <c r="D32" s="79"/>
-      <c r="E32" s="79"/>
-      <c r="F32" s="79"/>
+      <c r="C32" s="79"/>
+      <c r="D32" s="78"/>
+      <c r="E32" s="78"/>
+      <c r="F32" s="78"/>
     </row>
     <row r="33" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B33" s="7" t="s">
@@ -10659,6 +10659,12 @@
     </row>
   </sheetData>
   <mergeCells count="14">
+    <mergeCell ref="B12:B13"/>
+    <mergeCell ref="E12:E13"/>
+    <mergeCell ref="C34:F34"/>
+    <mergeCell ref="C12:C13"/>
+    <mergeCell ref="F12:F13"/>
+    <mergeCell ref="B31:B32"/>
     <mergeCell ref="G12:G13"/>
     <mergeCell ref="C38:F38"/>
     <mergeCell ref="C33:F33"/>
@@ -10667,12 +10673,6 @@
     <mergeCell ref="C37:F37"/>
     <mergeCell ref="C36:F36"/>
     <mergeCell ref="C35:F35"/>
-    <mergeCell ref="B12:B13"/>
-    <mergeCell ref="E12:E13"/>
-    <mergeCell ref="C34:F34"/>
-    <mergeCell ref="C12:C13"/>
-    <mergeCell ref="F12:F13"/>
-    <mergeCell ref="B31:B32"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Cost sorting of the data matched with the distribution model. Sorted low to high. Namings and tables edited
</commit_message>
<xml_diff>
--- a/Arya_Phones_Supplier_Selection.xlsx
+++ b/Arya_Phones_Supplier_Selection.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\LENOVO\Desktop\Asistan\Arya Phone\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{257C911A-5CEF-4D91-B0C5-CA0BA03CBE22}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{126C6FDA-92FA-469E-B520-CDD86EA51C2C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -22,6 +22,7 @@
     <sheet name="Arya Case" sheetId="7" r:id="rId7"/>
   </sheets>
   <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">User!$A$1:$H$21</definedName>
     <definedName name="solver_eng" localSheetId="2" hidden="1">1</definedName>
     <definedName name="solver_neg" localSheetId="2" hidden="1">1</definedName>
     <definedName name="solver_num" localSheetId="2" hidden="1">0</definedName>
@@ -841,14 +842,14 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1759,146 +1760,146 @@
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A2" s="43">
-        <v>1</v>
+        <v>20</v>
       </c>
       <c r="B2" s="53">
-        <v>0.18141826864259999</v>
+        <v>0.19849199345865401</v>
       </c>
       <c r="C2" s="53">
-        <v>0.254450791916772</v>
+        <v>0.2048960971299689</v>
       </c>
       <c r="D2" s="60">
-        <v>0.61191053879833257</v>
+        <v>9.7371468909865005E-2</v>
       </c>
       <c r="E2" s="65">
-        <v>0.106720019477238</v>
+        <v>0.15672001947723799</v>
       </c>
       <c r="F2" s="65">
-        <v>0.152651963522863</v>
+        <v>0.10155365833498819</v>
       </c>
       <c r="G2" s="54">
-        <v>0.1037612453176729</v>
+        <v>0.27114700608346642</v>
       </c>
       <c r="H2" s="1" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A3" s="43">
-        <v>2</v>
+        <v>19</v>
       </c>
       <c r="B3" s="53">
-        <v>0.29731528292090348</v>
+        <v>0.28227114589511132</v>
       </c>
       <c r="C3" s="53">
-        <v>0.29115081021963801</v>
+        <v>0.27341827619398001</v>
       </c>
       <c r="D3" s="60">
-        <v>0.61026173707464948</v>
+        <v>0.117371468909865</v>
       </c>
       <c r="E3" s="65">
-        <v>0.18945464506061421</v>
+        <v>0.102500150077396</v>
       </c>
       <c r="F3" s="65">
-        <v>0.10155365833498819</v>
+        <v>0.1127673895923734</v>
       </c>
       <c r="G3" s="54">
-        <v>0.29588315318380942</v>
+        <v>0.1020081514064624</v>
       </c>
       <c r="H3" s="1" t="s">
-        <v>34</v>
+        <v>43</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A4" s="43">
-        <v>3</v>
+        <v>18</v>
       </c>
       <c r="B4" s="53">
-        <v>5.133819847534786E-2</v>
+        <v>0.19511378053770029</v>
       </c>
       <c r="C4" s="53">
-        <v>0.25457641457483893</v>
+        <v>7.3418276193979989E-2</v>
       </c>
       <c r="D4" s="60">
-        <v>0.60726173707464903</v>
+        <v>0.13737146890986501</v>
       </c>
       <c r="E4" s="65">
-        <v>0.24824483374410089</v>
+        <v>0.31938813314298031</v>
       </c>
       <c r="F4" s="65">
-        <v>0.2881274398577503</v>
+        <v>0.10155365833498819</v>
       </c>
       <c r="G4" s="54">
-        <v>0.26426915998857842</v>
+        <v>0.100629661763317</v>
       </c>
       <c r="H4" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A5" s="43">
-        <v>4</v>
+        <v>17</v>
       </c>
       <c r="B5" s="53">
-        <v>0.28227114589511132</v>
+        <v>6.067934013561796E-2</v>
       </c>
       <c r="C5" s="53">
-        <v>6.516607737331874E-2</v>
+        <v>0.10691631099167261</v>
       </c>
       <c r="D5" s="60">
-        <v>0.58371425606695315</v>
+        <v>0.17137146890986499</v>
       </c>
       <c r="E5" s="65">
-        <v>0.28577314002182541</v>
+        <v>0.29128321359242249</v>
       </c>
       <c r="F5" s="65">
-        <v>0.16710661185701839</v>
+        <v>0.23155365833498801</v>
       </c>
       <c r="G5" s="54">
-        <v>0.15996685766432919</v>
+        <v>0.1096077760804178</v>
       </c>
       <c r="H5" s="1" t="s">
-        <v>49</v>
+        <v>40</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A6" s="43">
-        <v>5</v>
+        <v>16</v>
       </c>
       <c r="B6" s="53">
-        <v>0.1202053717041603</v>
+        <v>0.156765667715111</v>
       </c>
       <c r="C6" s="53">
-        <v>0.16109848730107321</v>
+        <v>0.243834865733492</v>
       </c>
       <c r="D6" s="60">
-        <v>0.54893726307541901</v>
+        <v>0.19145012390986499</v>
       </c>
       <c r="E6" s="65">
-        <v>0.17008933186008149</v>
+        <v>0.183331251224816</v>
       </c>
       <c r="F6" s="65">
-        <v>0.27528967563063772</v>
+        <v>0.20155365833498801</v>
       </c>
       <c r="G6" s="54">
-        <v>0.16758907375405899</v>
+        <v>0.10840881707564209</v>
       </c>
       <c r="H6" s="1" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A7" s="43">
-        <v>6</v>
+        <v>15</v>
       </c>
       <c r="B7" s="53">
-        <v>6.2008630366313218E-2</v>
+        <v>0.19188915259436859</v>
       </c>
       <c r="C7" s="53">
-        <v>0.26040571421757103</v>
+        <v>9.6546504644227593E-2</v>
       </c>
       <c r="D7" s="60">
-        <v>0.53524476184674197</v>
+        <v>0.21705211340986499</v>
       </c>
       <c r="E7" s="65">
         <v>0.1067200194772385</v>
@@ -1907,53 +1908,53 @@
         <v>0.10155365833498819</v>
       </c>
       <c r="G7" s="54">
-        <v>0.2560017363633072</v>
+        <v>0.27864380253183429</v>
       </c>
       <c r="H7" s="1" t="s">
-        <v>30</v>
+        <v>33</v>
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A8" s="43">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="B8" s="53">
-        <v>8.4653338407399248E-2</v>
+        <v>0.1262867946106227</v>
       </c>
       <c r="C8" s="53">
-        <v>0.12208818407051721</v>
+        <v>7.3418276193979989E-2</v>
       </c>
       <c r="D8" s="60">
-        <v>0.50118862071605097</v>
+        <v>0.24790607253205099</v>
       </c>
       <c r="E8" s="65">
-        <v>0.32446059664501697</v>
+        <v>0.29100442200694832</v>
       </c>
       <c r="F8" s="65">
-        <v>0.10155365833498819</v>
+        <v>0.108246470664996</v>
       </c>
       <c r="G8" s="54">
-        <v>0.13823591172591559</v>
+        <v>0.1139929232648282</v>
       </c>
       <c r="H8" s="1" t="s">
-        <v>46</v>
+        <v>31</v>
       </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A9" s="43">
-        <v>8</v>
+        <v>13</v>
       </c>
       <c r="B9" s="53">
-        <v>0.10536952724685961</v>
+        <v>0.25691282528883602</v>
       </c>
       <c r="C9" s="53">
-        <v>0.26693912830951111</v>
+        <v>0.25457641457483893</v>
       </c>
       <c r="D9" s="60">
-        <v>0.47418990241855702</v>
+        <v>0.28126564060459602</v>
       </c>
       <c r="E9" s="65">
-        <v>0.1067200194772385</v>
+        <v>0.24206895072120549</v>
       </c>
       <c r="F9" s="65">
         <v>0.10155365833498819</v>
@@ -1962,128 +1963,128 @@
         <v>0.1037612453176729</v>
       </c>
       <c r="H9" s="1" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A10" s="43">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="B10" s="53">
-        <v>6.4227033173094625E-2</v>
+        <v>0.1039433720356735</v>
       </c>
       <c r="C10" s="53">
-        <v>0.15483029452809721</v>
+        <v>0.19024045650357649</v>
       </c>
       <c r="D10" s="60">
-        <v>0.43507948585385298</v>
+        <v>0.34034996285317798</v>
       </c>
       <c r="E10" s="65">
-        <v>0.16962970966432209</v>
+        <v>0.27804323994842262</v>
       </c>
       <c r="F10" s="65">
-        <v>0.10155365833498819</v>
+        <v>0.119152078029859</v>
       </c>
       <c r="G10" s="54">
-        <v>0.29345450745565288</v>
+        <v>0.1037612453176729</v>
       </c>
       <c r="H10" s="1" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A11" s="43">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B11" s="53">
-        <v>6.067934013561796E-2</v>
+        <v>0.1216495133482835</v>
       </c>
       <c r="C11" s="53">
-        <v>6.6813196513184861E-2</v>
+        <v>0.16985306196136299</v>
       </c>
       <c r="D11" s="60">
-        <v>0.399950545031311</v>
+        <v>0.388563554257354</v>
       </c>
       <c r="E11" s="65">
-        <v>0.12896323351417149</v>
+        <v>0.24861374555913729</v>
       </c>
       <c r="F11" s="65">
-        <v>0.12518162852531989</v>
+        <v>0.25064404411660468</v>
       </c>
       <c r="G11" s="54">
-        <v>0.21570645620864939</v>
+        <v>0.16999576138077049</v>
       </c>
       <c r="H11" s="1" t="s">
-        <v>32</v>
+        <v>38</v>
       </c>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A12" s="43">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B12" s="53">
-        <v>0.1216495133482835</v>
+        <v>6.067934013561796E-2</v>
       </c>
       <c r="C12" s="53">
-        <v>0.16985306196136299</v>
+        <v>6.6813196513184861E-2</v>
       </c>
       <c r="D12" s="60">
-        <v>0.388563554257354</v>
+        <v>0.399950545031311</v>
       </c>
       <c r="E12" s="65">
-        <v>0.24861374555913729</v>
+        <v>0.12896323351417149</v>
       </c>
       <c r="F12" s="65">
-        <v>0.25064404411660468</v>
+        <v>0.12518162852531989</v>
       </c>
       <c r="G12" s="54">
-        <v>0.16999576138077049</v>
+        <v>0.21570645620864939</v>
       </c>
       <c r="H12" s="1" t="s">
-        <v>38</v>
+        <v>32</v>
       </c>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A13" s="43">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="B13" s="53">
-        <v>0.1039433720356735</v>
+        <v>6.4227033173094625E-2</v>
       </c>
       <c r="C13" s="53">
-        <v>0.19024045650357649</v>
+        <v>0.15483029452809721</v>
       </c>
       <c r="D13" s="60">
-        <v>0.34034996285317798</v>
+        <v>0.43507948585385298</v>
       </c>
       <c r="E13" s="65">
-        <v>0.27804323994842262</v>
+        <v>0.16962970966432209</v>
       </c>
       <c r="F13" s="65">
-        <v>0.119152078029859</v>
+        <v>0.10155365833498819</v>
       </c>
       <c r="G13" s="54">
-        <v>0.1037612453176729</v>
+        <v>0.29345450745565288</v>
       </c>
       <c r="H13" s="1" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A14" s="43">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="B14" s="53">
-        <v>0.25691282528883602</v>
+        <v>0.10536952724685961</v>
       </c>
       <c r="C14" s="53">
-        <v>0.25457641457483893</v>
+        <v>0.26693912830951111</v>
       </c>
       <c r="D14" s="60">
-        <v>0.28126564060459602</v>
+        <v>0.47418990241855702</v>
       </c>
       <c r="E14" s="65">
-        <v>0.24206895072120549</v>
+        <v>0.1067200194772385</v>
       </c>
       <c r="F14" s="65">
         <v>0.10155365833498819</v>
@@ -2092,47 +2093,47 @@
         <v>0.1037612453176729</v>
       </c>
       <c r="H14" s="1" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A15" s="43">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="B15" s="53">
-        <v>0.1262867946106227</v>
+        <v>8.4653338407399248E-2</v>
       </c>
       <c r="C15" s="53">
-        <v>7.3418276193979989E-2</v>
+        <v>0.12208818407051721</v>
       </c>
       <c r="D15" s="60">
-        <v>0.24790607253205099</v>
+        <v>0.50118862071605097</v>
       </c>
       <c r="E15" s="65">
-        <v>0.29100442200694832</v>
+        <v>0.32446059664501697</v>
       </c>
       <c r="F15" s="65">
-        <v>0.108246470664996</v>
+        <v>0.10155365833498819</v>
       </c>
       <c r="G15" s="54">
-        <v>0.1139929232648282</v>
+        <v>0.13823591172591559</v>
       </c>
       <c r="H15" s="1" t="s">
-        <v>31</v>
+        <v>46</v>
       </c>
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A16" s="43">
-        <v>15</v>
+        <v>6</v>
       </c>
       <c r="B16" s="53">
-        <v>0.19188915259436859</v>
+        <v>6.2008630366313218E-2</v>
       </c>
       <c r="C16" s="53">
-        <v>9.6546504644227593E-2</v>
+        <v>0.26040571421757103</v>
       </c>
       <c r="D16" s="60">
-        <v>0.21705211340986499</v>
+        <v>0.53524476184674197</v>
       </c>
       <c r="E16" s="65">
         <v>0.1067200194772385</v>
@@ -2141,143 +2142,148 @@
         <v>0.10155365833498819</v>
       </c>
       <c r="G16" s="54">
-        <v>0.27864380253183429</v>
+        <v>0.2560017363633072</v>
       </c>
       <c r="H16" s="1" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
     </row>
     <row r="17" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A17" s="43">
-        <v>16</v>
+        <v>5</v>
       </c>
       <c r="B17" s="53">
-        <v>0.156765667715111</v>
+        <v>0.1202053717041603</v>
       </c>
       <c r="C17" s="53">
-        <v>0.243834865733492</v>
+        <v>0.16109848730107321</v>
       </c>
       <c r="D17" s="60">
-        <v>0.19145012390986499</v>
+        <v>0.54893726307541901</v>
       </c>
       <c r="E17" s="65">
-        <v>0.183331251224816</v>
+        <v>0.17008933186008149</v>
       </c>
       <c r="F17" s="65">
-        <v>0.20155365833498801</v>
+        <v>0.27528967563063772</v>
       </c>
       <c r="G17" s="54">
-        <v>0.10840881707564209</v>
+        <v>0.16758907375405899</v>
       </c>
       <c r="H17" s="1" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
     </row>
     <row r="18" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A18" s="43">
-        <v>17</v>
+        <v>4</v>
       </c>
       <c r="B18" s="53">
-        <v>6.067934013561796E-2</v>
+        <v>0.28227114589511132</v>
       </c>
       <c r="C18" s="53">
-        <v>0.10691631099167261</v>
+        <v>6.516607737331874E-2</v>
       </c>
       <c r="D18" s="60">
-        <v>0.17137146890986499</v>
+        <v>0.58371425606695315</v>
       </c>
       <c r="E18" s="65">
-        <v>0.29128321359242249</v>
+        <v>0.28577314002182541</v>
       </c>
       <c r="F18" s="65">
-        <v>0.23155365833498801</v>
+        <v>0.16710661185701839</v>
       </c>
       <c r="G18" s="54">
-        <v>0.1096077760804178</v>
+        <v>0.15996685766432919</v>
       </c>
       <c r="H18" s="1" t="s">
-        <v>40</v>
+        <v>49</v>
       </c>
     </row>
     <row r="19" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A19" s="43">
-        <v>18</v>
+        <v>3</v>
       </c>
       <c r="B19" s="53">
-        <v>0.19511378053770029</v>
+        <v>5.133819847534786E-2</v>
       </c>
       <c r="C19" s="53">
-        <v>7.3418276193979989E-2</v>
+        <v>0.25457641457483893</v>
       </c>
       <c r="D19" s="60">
-        <v>0.13737146890986501</v>
+        <v>0.60726173707464903</v>
       </c>
       <c r="E19" s="65">
-        <v>0.31938813314298031</v>
+        <v>0.24824483374410089</v>
       </c>
       <c r="F19" s="65">
-        <v>0.10155365833498819</v>
+        <v>0.2881274398577503</v>
       </c>
       <c r="G19" s="54">
-        <v>0.100629661763317</v>
+        <v>0.26426915998857842</v>
       </c>
       <c r="H19" s="1" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
     </row>
     <row r="20" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A20" s="43">
-        <v>19</v>
+        <v>2</v>
       </c>
       <c r="B20" s="53">
-        <v>0.28227114589511132</v>
+        <v>0.29731528292090348</v>
       </c>
       <c r="C20" s="53">
-        <v>0.27341827619398001</v>
+        <v>0.29115081021963801</v>
       </c>
       <c r="D20" s="60">
-        <v>0.117371468909865</v>
+        <v>0.61026173707464948</v>
       </c>
       <c r="E20" s="65">
-        <v>0.102500150077396</v>
+        <v>0.18945464506061421</v>
       </c>
       <c r="F20" s="65">
-        <v>0.1127673895923734</v>
+        <v>0.10155365833498819</v>
       </c>
       <c r="G20" s="54">
-        <v>0.1020081514064624</v>
+        <v>0.29588315318380942</v>
       </c>
       <c r="H20" s="1" t="s">
-        <v>43</v>
+        <v>34</v>
       </c>
     </row>
     <row r="21" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A21" s="43">
-        <v>20</v>
+        <v>1</v>
       </c>
       <c r="B21" s="53">
-        <v>0.19849199345865401</v>
+        <v>0.18141826864259999</v>
       </c>
       <c r="C21" s="53">
-        <v>0.2048960971299689</v>
+        <v>0.254450791916772</v>
       </c>
       <c r="D21" s="60">
-        <v>9.7371468909865005E-2</v>
+        <v>0.61191053879833257</v>
       </c>
       <c r="E21" s="65">
-        <v>0.15672001947723799</v>
+        <v>0.106720019477238</v>
       </c>
       <c r="F21" s="65">
-        <v>0.10155365833498819</v>
+        <v>0.152651963522863</v>
       </c>
       <c r="G21" s="54">
-        <v>0.27114700608346642</v>
+        <v>0.1037612453176729</v>
       </c>
       <c r="H21" s="1" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:H21" xr:uid="{00000000-0001-0000-0100-000000000000}">
+    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:H21">
+      <sortCondition ref="D1:D21"/>
+    </sortState>
+  </autoFilter>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -10574,22 +10580,22 @@
       </c>
     </row>
     <row r="31" spans="1:18" x14ac:dyDescent="0.3">
-      <c r="B31" s="80" t="s">
-        <v>0</v>
-      </c>
-      <c r="C31" s="77" t="s">
+      <c r="B31" s="77" t="s">
+        <v>0</v>
+      </c>
+      <c r="C31" s="78" t="s">
         <v>88</v>
       </c>
-      <c r="D31" s="78"/>
-      <c r="E31" s="78"/>
-      <c r="F31" s="78"/>
+      <c r="D31" s="79"/>
+      <c r="E31" s="79"/>
+      <c r="F31" s="79"/>
     </row>
     <row r="32" spans="1:18" x14ac:dyDescent="0.3">
       <c r="B32" s="67"/>
-      <c r="C32" s="79"/>
-      <c r="D32" s="78"/>
-      <c r="E32" s="78"/>
-      <c r="F32" s="78"/>
+      <c r="C32" s="80"/>
+      <c r="D32" s="79"/>
+      <c r="E32" s="79"/>
+      <c r="F32" s="79"/>
     </row>
     <row r="33" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B33" s="7" t="s">
@@ -10659,12 +10665,6 @@
     </row>
   </sheetData>
   <mergeCells count="14">
-    <mergeCell ref="B12:B13"/>
-    <mergeCell ref="E12:E13"/>
-    <mergeCell ref="C34:F34"/>
-    <mergeCell ref="C12:C13"/>
-    <mergeCell ref="F12:F13"/>
-    <mergeCell ref="B31:B32"/>
     <mergeCell ref="G12:G13"/>
     <mergeCell ref="C38:F38"/>
     <mergeCell ref="C33:F33"/>
@@ -10673,6 +10673,12 @@
     <mergeCell ref="C37:F37"/>
     <mergeCell ref="C36:F36"/>
     <mergeCell ref="C35:F35"/>
+    <mergeCell ref="B12:B13"/>
+    <mergeCell ref="E12:E13"/>
+    <mergeCell ref="C34:F34"/>
+    <mergeCell ref="C12:C13"/>
+    <mergeCell ref="F12:F13"/>
+    <mergeCell ref="B31:B32"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>